<commit_message>
Tighten Phase 1 league match + add SofaScore H2H labels in Phase 3
- Phase 1: replace substring league hints with exact-name set per country
  so LaLiga2 / MLS Next Pro / Premier League 2 etc. no longer leak into
  ready_for_phase_2. Strip "COUNTRY: " prefix Flashscore prepends to some
  league names before comparison.

- Phase 3: pull head-to-head trend labels from SofaScore's
  /api/v1/event/{id}/team-streaks endpoint (the only public h2h-shaped
  endpoint that responds 200 for an upcoming match). Resolve the
  upcoming SofaScore event ID via /team/{id}/events/next/0 first, then
  fetch labels and derive a meeting-count from the X/N label values.
  Adds h2h_labels column carrying the raw SofaScore H2H signals.

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/agent-system/outputs/Phase1_Fixture_Slate.xlsx
+++ b/docs/agent-system/outputs/Phase1_Fixture_Slate.xlsx
@@ -126,7 +126,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-05-04 06:56:40 ACST</t>
+          <t>2026-05-04 07:11:06 ACST</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -233,7 +233,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-05-04 06:56:40 ACST</t>
+          <t>2026-05-04 07:11:06 ACST</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -340,7 +340,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-05-04 06:56:40 ACST</t>
+          <t>2026-05-04 07:11:06 ACST</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -370,7 +370,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>flashscore:GOQASy66</t>
+          <t>flashscore:zs3PZaZa</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -380,7 +380,7 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>04:00</t>
+          <t>04:30</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
@@ -390,7 +390,7 @@
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>1777919400</t>
+          <t>1777921200</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
@@ -400,22 +400,22 @@
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>Almeria</t>
+          <t>Sevilla</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>flashscore:almeria</t>
+          <t>flashscore:sevilla</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>Mirandes</t>
+          <t>Real Sociedad</t>
         </is>
       </c>
       <c r="P4" t="inlineStr">
         <is>
-          <t>flashscore:mirandes</t>
+          <t>flashscore:realsociedad</t>
         </is>
       </c>
       <c r="Q4" t="inlineStr">
@@ -447,7 +447,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-05-04 06:56:40 ACST</t>
+          <t>2026-05-04 07:11:06 ACST</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -462,7 +462,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>17</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -472,12 +472,12 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>LaLiga</t>
+          <t>Premier League</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>flashscore:zs3PZaZa</t>
+          <t>flashscore:rTwrFuZR</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -507,22 +507,22 @@
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>Sevilla</t>
+          <t>Everton</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>flashscore:sevilla</t>
+          <t>flashscore:everton</t>
         </is>
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>Real Sociedad</t>
+          <t>Manchester City</t>
         </is>
       </c>
       <c r="P5" t="inlineStr">
         <is>
-          <t>flashscore:realsociedad</t>
+          <t>flashscore:manchestercity</t>
         </is>
       </c>
       <c r="Q5" t="inlineStr">
@@ -546,113 +546,6 @@
         </is>
       </c>
       <c r="U5" t="inlineStr">
-        <is>
-          <t>Keyless Flashscore fixture feed.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>2026-05-04 06:56:40 ACST</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Flashscore</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>healthy</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>17</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>Premier League</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>flashscore:rTwrFuZR</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>2026-05-05</t>
-        </is>
-      </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>04:30</t>
-        </is>
-      </c>
-      <c r="J6" t="inlineStr">
-        <is>
-          <t>Australia/Adelaide</t>
-        </is>
-      </c>
-      <c r="K6" t="inlineStr">
-        <is>
-          <t>1777921200</t>
-        </is>
-      </c>
-      <c r="L6" t="inlineStr">
-        <is>
-          <t>live</t>
-        </is>
-      </c>
-      <c r="M6" t="inlineStr">
-        <is>
-          <t>Everton</t>
-        </is>
-      </c>
-      <c r="N6" t="inlineStr">
-        <is>
-          <t>flashscore:everton</t>
-        </is>
-      </c>
-      <c r="O6" t="inlineStr">
-        <is>
-          <t>Manchester City</t>
-        </is>
-      </c>
-      <c r="P6" t="inlineStr">
-        <is>
-          <t>flashscore:manchestercity</t>
-        </is>
-      </c>
-      <c r="Q6" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="R6" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="S6" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="T6" t="inlineStr">
-        <is>
-          <t>ready_for_phase_2</t>
-        </is>
-      </c>
-      <c r="U6" t="inlineStr">
         <is>
           <t>Keyless Flashscore fixture feed.</t>
         </is>
@@ -775,7 +668,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-05-04 06:56:40 ACST</t>
+          <t>2026-05-04 07:11:06 ACST</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -882,7 +775,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-05-04 06:56:40 ACST</t>
+          <t>2026-05-04 07:11:06 ACST</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -989,7 +882,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-05-04 06:56:40 ACST</t>
+          <t>2026-05-04 07:11:06 ACST</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -1019,7 +912,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>flashscore:GOQASy66</t>
+          <t>flashscore:zs3PZaZa</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -1029,7 +922,7 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>04:00</t>
+          <t>04:30</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
@@ -1039,7 +932,7 @@
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>1777919400</t>
+          <t>1777921200</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
@@ -1049,22 +942,22 @@
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>Almeria</t>
+          <t>Sevilla</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>flashscore:almeria</t>
+          <t>flashscore:sevilla</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>Mirandes</t>
+          <t>Real Sociedad</t>
         </is>
       </c>
       <c r="P4" t="inlineStr">
         <is>
-          <t>flashscore:mirandes</t>
+          <t>flashscore:realsociedad</t>
         </is>
       </c>
       <c r="Q4" t="inlineStr">
@@ -1096,7 +989,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-05-04 06:56:40 ACST</t>
+          <t>2026-05-04 07:11:06 ACST</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -1111,7 +1004,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>17</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -1121,12 +1014,12 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>LaLiga</t>
+          <t>Premier League</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>flashscore:zs3PZaZa</t>
+          <t>flashscore:rTwrFuZR</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -1156,22 +1049,22 @@
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>Sevilla</t>
+          <t>Everton</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>flashscore:sevilla</t>
+          <t>flashscore:everton</t>
         </is>
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>Real Sociedad</t>
+          <t>Manchester City</t>
         </is>
       </c>
       <c r="P5" t="inlineStr">
         <is>
-          <t>flashscore:realsociedad</t>
+          <t>flashscore:manchestercity</t>
         </is>
       </c>
       <c r="Q5" t="inlineStr">
@@ -1195,113 +1088,6 @@
         </is>
       </c>
       <c r="U5" t="inlineStr">
-        <is>
-          <t>Keyless Flashscore fixture feed.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>2026-05-04 06:56:40 ACST</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Flashscore</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>healthy</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>17</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>Premier League</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>flashscore:rTwrFuZR</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>2026-05-05</t>
-        </is>
-      </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>04:30</t>
-        </is>
-      </c>
-      <c r="J6" t="inlineStr">
-        <is>
-          <t>Australia/Adelaide</t>
-        </is>
-      </c>
-      <c r="K6" t="inlineStr">
-        <is>
-          <t>1777921200</t>
-        </is>
-      </c>
-      <c r="L6" t="inlineStr">
-        <is>
-          <t>live</t>
-        </is>
-      </c>
-      <c r="M6" t="inlineStr">
-        <is>
-          <t>Everton</t>
-        </is>
-      </c>
-      <c r="N6" t="inlineStr">
-        <is>
-          <t>flashscore:everton</t>
-        </is>
-      </c>
-      <c r="O6" t="inlineStr">
-        <is>
-          <t>Manchester City</t>
-        </is>
-      </c>
-      <c r="P6" t="inlineStr">
-        <is>
-          <t>flashscore:manchestercity</t>
-        </is>
-      </c>
-      <c r="Q6" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="R6" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="S6" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="T6" t="inlineStr">
-        <is>
-          <t>ready_for_phase_2</t>
-        </is>
-      </c>
-      <c r="U6" t="inlineStr">
         <is>
           <t>Keyless Flashscore fixture feed.</t>
         </is>
@@ -1622,12 +1408,12 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -1677,7 +1463,7 @@
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
@@ -1882,7 +1668,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-05-04 06:56:40 ACST</t>
+          <t>2026-05-04 07:11:06 ACST</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -1912,12 +1698,12 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>events=317 league_hit=5 skipped_women=0 out_of_window=0 matched=5 by_league={'Premier League': 2, 'LaLiga': 2, 'MLS': 1} sample_leagues=['Albania|ALBANIA: Kategoria e Parë', 'Algeria|ALGERIA: Ligue 1', 'Antigua &amp; Barbuda|ANTIGUA &amp; BARBUDA: ABFA Premier League', 'Argentina|ARGENTINA: Liga Profesional - Apertura', 'Argentina|ARGENTINA: Primera Nacional', 'Argentina|ARGENTINA: Torneo Federal', 'Argentina|ARGENTINA: Primera C', 'Argentina|ARGENTINA: Primera A Women - Apertura']</t>
+          <t>events=309 league_hit=4 skipped_women=0 out_of_window=0 matched=4 by_league={'Premier League': 2, 'LaLiga': 1, 'MLS': 1} sample_leagues=['Albania|ALBANIA: Kategoria e Parë', 'Algeria|ALGERIA: Ligue 1', 'Antigua &amp; Barbuda|ANTIGUA &amp; BARBUDA: ABFA Premier League', 'Argentina|ARGENTINA: Liga Profesional - Apertura', 'Argentina|ARGENTINA: Primera Nacional', 'Argentina|ARGENTINA: Torneo Federal', 'Argentina|ARGENTINA: Primera C', 'Argentina|ARGENTINA: Primera A Women - Apertura']</t>
         </is>
       </c>
     </row>
@@ -1984,7 +1770,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
     </row>
@@ -1996,7 +1782,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Wire Phase 1-7 orchestrator into run_daily.bat (non-fatal stage)
run_daily.bat now runs soccer_routine.py first (live dashboard, hard
exit on failure), then soccer_phases_routine.py (agent system, errors
logged but non-fatal so the daily can't be broken by Phase 2 IP blocks
or upstream API hiccups).

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/agent-system/outputs/Phase1_Fixture_Slate.xlsx
+++ b/docs/agent-system/outputs/Phase1_Fixture_Slate.xlsx
@@ -126,7 +126,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-05-04 07:11:06 ACST</t>
+          <t>2026-05-04 07:24:29 ACST</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -233,7 +233,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-05-04 07:11:06 ACST</t>
+          <t>2026-05-04 07:24:29 ACST</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -340,7 +340,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-05-04 07:11:06 ACST</t>
+          <t>2026-05-04 07:24:29 ACST</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -447,7 +447,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-05-04 07:11:06 ACST</t>
+          <t>2026-05-04 07:24:29 ACST</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -668,7 +668,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-05-04 07:11:06 ACST</t>
+          <t>2026-05-04 07:24:29 ACST</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -775,7 +775,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-05-04 07:11:06 ACST</t>
+          <t>2026-05-04 07:24:29 ACST</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -882,7 +882,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-05-04 07:11:06 ACST</t>
+          <t>2026-05-04 07:24:29 ACST</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -989,7 +989,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-05-04 07:11:06 ACST</t>
+          <t>2026-05-04 07:24:29 ACST</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -1668,7 +1668,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-05-04 07:11:06 ACST</t>
+          <t>2026-05-04 07:24:29 ACST</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -1703,7 +1703,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>events=309 league_hit=4 skipped_women=0 out_of_window=0 matched=4 by_league={'Premier League': 2, 'LaLiga': 1, 'MLS': 1} sample_leagues=['Albania|ALBANIA: Kategoria e Parë', 'Algeria|ALGERIA: Ligue 1', 'Antigua &amp; Barbuda|ANTIGUA &amp; BARBUDA: ABFA Premier League', 'Argentina|ARGENTINA: Liga Profesional - Apertura', 'Argentina|ARGENTINA: Primera Nacional', 'Argentina|ARGENTINA: Torneo Federal', 'Argentina|ARGENTINA: Primera C', 'Argentina|ARGENTINA: Primera A Women - Apertura']</t>
+          <t>events=308 league_hit=4 skipped_women=0 out_of_window=0 matched=4 by_league={'Premier League': 2, 'LaLiga': 1, 'MLS': 1} sample_leagues=['Albania|ALBANIA: Kategoria e Parë', 'Algeria|ALGERIA: Ligue 1', 'Antigua &amp; Barbuda|ANTIGUA &amp; BARBUDA: ABFA Premier League', 'Argentina|ARGENTINA: Liga Profesional - Apertura', 'Argentina|ARGENTINA: Primera Nacional', 'Argentina|ARGENTINA: Torneo Federal', 'Argentina|ARGENTINA: Primera C', 'Argentina|ARGENTINA: Primera A Women - Apertura']</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix run_daily.bat call to auto_push.bat using script-dir resolution
When run_daily.bat is invoked via cmd /c with a relative path,
`call auto_push.bat` fails because cmd does not search PWD for
batch files in that context. Use %~dp0 (script directory) so
the call works regardless of how run_daily.bat is invoked.

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/agent-system/outputs/Phase1_Fixture_Slate.xlsx
+++ b/docs/agent-system/outputs/Phase1_Fixture_Slate.xlsx
@@ -126,7 +126,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-05-04 07:24:29 ACST</t>
+          <t>2026-05-04 07:33:44 ACST</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -233,7 +233,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-05-04 07:24:29 ACST</t>
+          <t>2026-05-04 07:33:44 ACST</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -340,7 +340,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-05-04 07:24:29 ACST</t>
+          <t>2026-05-04 07:33:44 ACST</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -447,7 +447,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-05-04 07:24:29 ACST</t>
+          <t>2026-05-04 07:33:44 ACST</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -668,7 +668,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-05-04 07:24:29 ACST</t>
+          <t>2026-05-04 07:33:44 ACST</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -775,7 +775,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-05-04 07:24:29 ACST</t>
+          <t>2026-05-04 07:33:44 ACST</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -882,7 +882,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-05-04 07:24:29 ACST</t>
+          <t>2026-05-04 07:33:44 ACST</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -989,7 +989,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-05-04 07:24:29 ACST</t>
+          <t>2026-05-04 07:33:44 ACST</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -1668,7 +1668,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-05-04 07:24:29 ACST</t>
+          <t>2026-05-04 07:33:44 ACST</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -1703,7 +1703,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>events=308 league_hit=4 skipped_women=0 out_of_window=0 matched=4 by_league={'Premier League': 2, 'LaLiga': 1, 'MLS': 1} sample_leagues=['Albania|ALBANIA: Kategoria e Parë', 'Algeria|ALGERIA: Ligue 1', 'Antigua &amp; Barbuda|ANTIGUA &amp; BARBUDA: ABFA Premier League', 'Argentina|ARGENTINA: Liga Profesional - Apertura', 'Argentina|ARGENTINA: Primera Nacional', 'Argentina|ARGENTINA: Torneo Federal', 'Argentina|ARGENTINA: Primera C', 'Argentina|ARGENTINA: Primera A Women - Apertura']</t>
+          <t>events=307 league_hit=4 skipped_women=0 out_of_window=0 matched=4 by_league={'Premier League': 2, 'LaLiga': 1, 'MLS': 1} sample_leagues=['Albania|ALBANIA: Kategoria e Parë', 'Algeria|ALGERIA: Ligue 1', 'Antigua &amp; Barbuda|ANTIGUA &amp; BARBUDA: ABFA Premier League', 'Argentina|ARGENTINA: Liga Profesional - Apertura', 'Argentina|ARGENTINA: Primera Nacional', 'Argentina|ARGENTINA: Torneo Federal', 'Argentina|ARGENTINA: Primera C', 'Argentina|ARGENTINA: Primera A Women - Apertura']</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto-push 2026-05-04T11:09: settle results + forecasts
</commit_message>
<xml_diff>
--- a/docs/agent-system/outputs/Phase1_Fixture_Slate.xlsx
+++ b/docs/agent-system/outputs/Phase1_Fixture_Slate.xlsx
@@ -126,7 +126,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-05-04 07:33:44 ACST</t>
+          <t>2026-05-04 11:08:52 ACST</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -141,7 +141,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>242</t>
+          <t>17</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -151,12 +151,12 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>MLS</t>
+          <t>Premier League</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>flashscore:2qevfSqS</t>
+          <t>flashscore:n1pZG14F</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -166,7 +166,7 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>07:00</t>
+          <t>23:30</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
@@ -176,7 +176,7 @@
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>1777843800</t>
+          <t>1777903200</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
@@ -186,22 +186,22 @@
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>Austin FC</t>
+          <t>Chelsea</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>flashscore:austinfc</t>
+          <t>flashscore:chelsea</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>St. Louis City</t>
+          <t>Nottingham</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>flashscore:stlouiscity</t>
+          <t>flashscore:nottingham</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
@@ -233,7 +233,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-05-04 07:33:44 ACST</t>
+          <t>2026-05-04 11:08:52 ACST</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -248,7 +248,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>242</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -258,12 +258,12 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Premier League</t>
+          <t>MLS</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>flashscore:n1pZG14F</t>
+          <t>flashscore:2qevfSqS</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -273,7 +273,7 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>23:30</t>
+          <t>FT</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
@@ -283,32 +283,32 @@
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>1777903200</t>
+          <t>1777843800</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>live</t>
+          <t>FT</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>Chelsea</t>
+          <t>Austin FC</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>flashscore:chelsea</t>
+          <t>flashscore:austinfc</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>Nottingham</t>
+          <t>St. Louis City</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>flashscore:nottingham</t>
+          <t>flashscore:stlouiscity</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
@@ -340,7 +340,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-05-04 07:33:44 ACST</t>
+          <t>2026-05-04 11:08:52 ACST</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -447,7 +447,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-05-04 07:33:44 ACST</t>
+          <t>2026-05-04 11:08:52 ACST</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -668,7 +668,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-05-04 07:33:44 ACST</t>
+          <t>2026-05-04 11:08:52 ACST</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -683,7 +683,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>242</t>
+          <t>17</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -693,12 +693,12 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>MLS</t>
+          <t>Premier League</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>flashscore:2qevfSqS</t>
+          <t>flashscore:n1pZG14F</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -708,7 +708,7 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>07:00</t>
+          <t>23:30</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
@@ -718,7 +718,7 @@
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>1777843800</t>
+          <t>1777903200</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
@@ -728,22 +728,22 @@
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>Austin FC</t>
+          <t>Chelsea</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>flashscore:austinfc</t>
+          <t>flashscore:chelsea</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>St. Louis City</t>
+          <t>Nottingham</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>flashscore:stlouiscity</t>
+          <t>flashscore:nottingham</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
@@ -775,7 +775,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-05-04 07:33:44 ACST</t>
+          <t>2026-05-04 11:08:52 ACST</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -790,7 +790,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>242</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -800,12 +800,12 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Premier League</t>
+          <t>MLS</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>flashscore:n1pZG14F</t>
+          <t>flashscore:2qevfSqS</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -815,7 +815,7 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>23:30</t>
+          <t>FT</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
@@ -825,32 +825,32 @@
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>1777903200</t>
+          <t>1777843800</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>live</t>
+          <t>FT</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>Chelsea</t>
+          <t>Austin FC</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>flashscore:chelsea</t>
+          <t>flashscore:austinfc</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>Nottingham</t>
+          <t>St. Louis City</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>flashscore:nottingham</t>
+          <t>flashscore:stlouiscity</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
@@ -882,7 +882,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-05-04 07:33:44 ACST</t>
+          <t>2026-05-04 11:08:52 ACST</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -989,7 +989,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-05-04 07:33:44 ACST</t>
+          <t>2026-05-04 11:08:52 ACST</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -1535,12 +1535,12 @@
       </c>
       <c r="M3" t="inlineStr">
         <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
           <t>1</t>
-        </is>
-      </c>
-      <c r="N3" t="inlineStr">
-        <is>
-          <t>0</t>
         </is>
       </c>
     </row>
@@ -1668,7 +1668,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-05-04 07:33:44 ACST</t>
+          <t>2026-05-04 11:08:52 ACST</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -1703,7 +1703,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>events=307 league_hit=4 skipped_women=0 out_of_window=0 matched=4 by_league={'Premier League': 2, 'LaLiga': 1, 'MLS': 1} sample_leagues=['Albania|ALBANIA: Kategoria e Parë', 'Algeria|ALGERIA: Ligue 1', 'Antigua &amp; Barbuda|ANTIGUA &amp; BARBUDA: ABFA Premier League', 'Argentina|ARGENTINA: Liga Profesional - Apertura', 'Argentina|ARGENTINA: Primera Nacional', 'Argentina|ARGENTINA: Torneo Federal', 'Argentina|ARGENTINA: Primera C', 'Argentina|ARGENTINA: Primera A Women - Apertura']</t>
+          <t>events=296 league_hit=4 skipped_women=0 out_of_window=0 matched=4 by_league={'Premier League': 2, 'LaLiga': 1, 'MLS': 1} sample_leagues=['Albania|ALBANIA: Kategoria e Parë', 'Algeria|ALGERIA: Ligue 1', 'Antigua &amp; Barbuda|ANTIGUA &amp; BARBUDA: ABFA Premier League', 'Argentina|ARGENTINA: Liga Profesional - Apertura', 'Argentina|ARGENTINA: Primera Nacional', 'Argentina|ARGENTINA: Torneo Federal', 'Argentina|ARGENTINA: Primera C', 'Argentina|ARGENTINA: Primera A Women - Apertura']</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto-push 2026-05-05T01:24: settle results + forecasts
</commit_message>
<xml_diff>
--- a/docs/agent-system/outputs/Phase1_Fixture_Slate.xlsx
+++ b/docs/agent-system/outputs/Phase1_Fixture_Slate.xlsx
@@ -126,7 +126,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-05-04 11:08:52 ACST</t>
+          <t>2026-05-05 01:24:14 ACST</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -141,7 +141,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>8</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -151,22 +151,22 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Premier League</t>
+          <t>LaLiga</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>flashscore:n1pZG14F</t>
+          <t>flashscore:zs3PZaZa</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>23:30</t>
+          <t>04:30</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
@@ -176,7 +176,7 @@
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>1777903200</t>
+          <t>1777921200</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
@@ -186,22 +186,22 @@
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>Chelsea</t>
+          <t>Sevilla</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>flashscore:chelsea</t>
+          <t>flashscore:sevilla</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>Nottingham</t>
+          <t>Real Sociedad</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>flashscore:nottingham</t>
+          <t>flashscore:realsociedad</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
@@ -233,7 +233,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-05-04 11:08:52 ACST</t>
+          <t>2026-05-05 01:24:14 ACST</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -248,7 +248,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>242</t>
+          <t>17</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -258,22 +258,22 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>MLS</t>
+          <t>Premier League</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>flashscore:2qevfSqS</t>
+          <t>flashscore:rTwrFuZR</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>FT</t>
+          <t>04:30</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
@@ -283,32 +283,32 @@
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>1777843800</t>
+          <t>1777921200</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>FT</t>
+          <t>live</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>Austin FC</t>
+          <t>Everton</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>flashscore:austinfc</t>
+          <t>flashscore:everton</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>St. Louis City</t>
+          <t>Manchester City</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>flashscore:stlouiscity</t>
+          <t>flashscore:manchestercity</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
@@ -332,220 +332,6 @@
         </is>
       </c>
       <c r="U3" t="inlineStr">
-        <is>
-          <t>Keyless Flashscore fixture feed.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>2026-05-04 11:08:52 ACST</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Flashscore</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>healthy</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>8</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>LaLiga</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>flashscore:zs3PZaZa</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>2026-05-05</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>04:30</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>Australia/Adelaide</t>
-        </is>
-      </c>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>1777921200</t>
-        </is>
-      </c>
-      <c r="L4" t="inlineStr">
-        <is>
-          <t>live</t>
-        </is>
-      </c>
-      <c r="M4" t="inlineStr">
-        <is>
-          <t>Sevilla</t>
-        </is>
-      </c>
-      <c r="N4" t="inlineStr">
-        <is>
-          <t>flashscore:sevilla</t>
-        </is>
-      </c>
-      <c r="O4" t="inlineStr">
-        <is>
-          <t>Real Sociedad</t>
-        </is>
-      </c>
-      <c r="P4" t="inlineStr">
-        <is>
-          <t>flashscore:realsociedad</t>
-        </is>
-      </c>
-      <c r="Q4" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="R4" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="S4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="T4" t="inlineStr">
-        <is>
-          <t>ready_for_phase_2</t>
-        </is>
-      </c>
-      <c r="U4" t="inlineStr">
-        <is>
-          <t>Keyless Flashscore fixture feed.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>2026-05-04 11:08:52 ACST</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Flashscore</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>healthy</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>17</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>Premier League</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>flashscore:rTwrFuZR</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>2026-05-05</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>04:30</t>
-        </is>
-      </c>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t>Australia/Adelaide</t>
-        </is>
-      </c>
-      <c r="K5" t="inlineStr">
-        <is>
-          <t>1777921200</t>
-        </is>
-      </c>
-      <c r="L5" t="inlineStr">
-        <is>
-          <t>live</t>
-        </is>
-      </c>
-      <c r="M5" t="inlineStr">
-        <is>
-          <t>Everton</t>
-        </is>
-      </c>
-      <c r="N5" t="inlineStr">
-        <is>
-          <t>flashscore:everton</t>
-        </is>
-      </c>
-      <c r="O5" t="inlineStr">
-        <is>
-          <t>Manchester City</t>
-        </is>
-      </c>
-      <c r="P5" t="inlineStr">
-        <is>
-          <t>flashscore:manchestercity</t>
-        </is>
-      </c>
-      <c r="Q5" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="R5" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="S5" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="T5" t="inlineStr">
-        <is>
-          <t>ready_for_phase_2</t>
-        </is>
-      </c>
-      <c r="U5" t="inlineStr">
         <is>
           <t>Keyless Flashscore fixture feed.</t>
         </is>
@@ -668,7 +454,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-05-04 11:08:52 ACST</t>
+          <t>2026-05-05 01:24:14 ACST</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -683,7 +469,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>8</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -693,22 +479,22 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Premier League</t>
+          <t>LaLiga</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>flashscore:n1pZG14F</t>
+          <t>flashscore:zs3PZaZa</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>23:30</t>
+          <t>04:30</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
@@ -718,7 +504,7 @@
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>1777903200</t>
+          <t>1777921200</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
@@ -728,22 +514,22 @@
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>Chelsea</t>
+          <t>Sevilla</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>flashscore:chelsea</t>
+          <t>flashscore:sevilla</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>Nottingham</t>
+          <t>Real Sociedad</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>flashscore:nottingham</t>
+          <t>flashscore:realsociedad</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
@@ -775,7 +561,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-05-04 11:08:52 ACST</t>
+          <t>2026-05-05 01:24:14 ACST</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -790,7 +576,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>242</t>
+          <t>17</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -800,22 +586,22 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>MLS</t>
+          <t>Premier League</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>flashscore:2qevfSqS</t>
+          <t>flashscore:rTwrFuZR</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-05-05</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>FT</t>
+          <t>04:30</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
@@ -825,32 +611,32 @@
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>1777843800</t>
+          <t>1777921200</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>FT</t>
+          <t>live</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>Austin FC</t>
+          <t>Everton</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>flashscore:austinfc</t>
+          <t>flashscore:everton</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>St. Louis City</t>
+          <t>Manchester City</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>flashscore:stlouiscity</t>
+          <t>flashscore:manchestercity</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
@@ -874,220 +660,6 @@
         </is>
       </c>
       <c r="U3" t="inlineStr">
-        <is>
-          <t>Keyless Flashscore fixture feed.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>2026-05-04 11:08:52 ACST</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Flashscore</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>healthy</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>8</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>LaLiga</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>flashscore:zs3PZaZa</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>2026-05-05</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>04:30</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>Australia/Adelaide</t>
-        </is>
-      </c>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>1777921200</t>
-        </is>
-      </c>
-      <c r="L4" t="inlineStr">
-        <is>
-          <t>live</t>
-        </is>
-      </c>
-      <c r="M4" t="inlineStr">
-        <is>
-          <t>Sevilla</t>
-        </is>
-      </c>
-      <c r="N4" t="inlineStr">
-        <is>
-          <t>flashscore:sevilla</t>
-        </is>
-      </c>
-      <c r="O4" t="inlineStr">
-        <is>
-          <t>Real Sociedad</t>
-        </is>
-      </c>
-      <c r="P4" t="inlineStr">
-        <is>
-          <t>flashscore:realsociedad</t>
-        </is>
-      </c>
-      <c r="Q4" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="R4" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="S4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="T4" t="inlineStr">
-        <is>
-          <t>ready_for_phase_2</t>
-        </is>
-      </c>
-      <c r="U4" t="inlineStr">
-        <is>
-          <t>Keyless Flashscore fixture feed.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>2026-05-04 11:08:52 ACST</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Flashscore</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>healthy</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>17</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>Premier League</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>flashscore:rTwrFuZR</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>2026-05-05</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>04:30</t>
-        </is>
-      </c>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t>Australia/Adelaide</t>
-        </is>
-      </c>
-      <c r="K5" t="inlineStr">
-        <is>
-          <t>1777921200</t>
-        </is>
-      </c>
-      <c r="L5" t="inlineStr">
-        <is>
-          <t>live</t>
-        </is>
-      </c>
-      <c r="M5" t="inlineStr">
-        <is>
-          <t>Everton</t>
-        </is>
-      </c>
-      <c r="N5" t="inlineStr">
-        <is>
-          <t>flashscore:everton</t>
-        </is>
-      </c>
-      <c r="O5" t="inlineStr">
-        <is>
-          <t>Manchester City</t>
-        </is>
-      </c>
-      <c r="P5" t="inlineStr">
-        <is>
-          <t>flashscore:manchestercity</t>
-        </is>
-      </c>
-      <c r="Q5" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="R5" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="S5" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="T5" t="inlineStr">
-        <is>
-          <t>ready_for_phase_2</t>
-        </is>
-      </c>
-      <c r="U5" t="inlineStr">
         <is>
           <t>Keyless Flashscore fixture feed.</t>
         </is>
@@ -1475,7 +1047,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>MLS</t>
+          <t>Premier League</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -1535,82 +1107,10 @@
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Premier League</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="L4" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="M4" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="N4" t="inlineStr">
         <is>
           <t>0</t>
         </is>
@@ -1668,7 +1168,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-05-04 11:08:52 ACST</t>
+          <t>2026-05-05 01:24:14 ACST</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -1683,7 +1183,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-05-04 to 2026-05-05</t>
+          <t>2026-05-05 to 2026-05-06</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -1698,12 +1198,12 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>2</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>events=296 league_hit=4 skipped_women=0 out_of_window=0 matched=4 by_league={'Premier League': 2, 'LaLiga': 1, 'MLS': 1} sample_leagues=['Albania|ALBANIA: Kategoria e Parë', 'Algeria|ALGERIA: Ligue 1', 'Antigua &amp; Barbuda|ANTIGUA &amp; BARBUDA: ABFA Premier League', 'Argentina|ARGENTINA: Liga Profesional - Apertura', 'Argentina|ARGENTINA: Primera Nacional', 'Argentina|ARGENTINA: Torneo Federal', 'Argentina|ARGENTINA: Primera C', 'Argentina|ARGENTINA: Primera A Women - Apertura']</t>
+          <t>events=295 league_hit=4 skipped_women=0 out_of_window=2 matched=2 by_league={'Premier League': 1, 'LaLiga': 1} sample_leagues=['Albania|ALBANIA: Kategoria e Parë', 'Algeria|ALGERIA: Ligue 1', 'Antigua &amp; Barbuda|ANTIGUA &amp; BARBUDA: ABFA Premier League', 'Argentina|ARGENTINA: Liga Profesional - Apertura', 'Argentina|ARGENTINA: Primera Nacional', 'Argentina|ARGENTINA: Torneo Federal', 'Argentina|ARGENTINA: Primera C', 'Argentina|ARGENTINA: Primera A Women - Apertura']</t>
         </is>
       </c>
     </row>
@@ -1734,7 +1234,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-05-04 to 2026-05-05</t>
+          <t>2026-05-05 to 2026-05-06</t>
         </is>
       </c>
     </row>
@@ -1770,7 +1270,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>2</t>
         </is>
       </c>
     </row>
@@ -1782,7 +1282,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>2</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto-push 2026-05-05T01:28: settle results + forecasts
</commit_message>
<xml_diff>
--- a/docs/agent-system/outputs/Phase1_Fixture_Slate.xlsx
+++ b/docs/agent-system/outputs/Phase1_Fixture_Slate.xlsx
@@ -126,7 +126,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-05-05 01:24:14 ACST</t>
+          <t>2026-05-05 01:28:20 ACST</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -233,7 +233,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-05-05 01:24:14 ACST</t>
+          <t>2026-05-05 01:28:20 ACST</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -454,7 +454,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-05-05 01:24:14 ACST</t>
+          <t>2026-05-05 01:28:20 ACST</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -561,7 +561,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-05-05 01:24:14 ACST</t>
+          <t>2026-05-05 01:28:20 ACST</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -1168,7 +1168,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-05-05 01:24:14 ACST</t>
+          <t>2026-05-05 01:28:20 ACST</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">

</xml_diff>

<commit_message>
Auto-push 2026-05-06T01:40: settle results + forecasts
</commit_message>
<xml_diff>
--- a/docs/agent-system/outputs/Phase1_Fixture_Slate.xlsx
+++ b/docs/agent-system/outputs/Phase1_Fixture_Slate.xlsx
@@ -126,47 +126,47 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-05-05 01:28:20 ACST</t>
+          <t>2026-05-06 01:40:37 ACST</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Flashscore</t>
+          <t>local match_data.json</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>healthy</t>
+          <t>source_unverified</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>37</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t/>
+          <t>88</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>LaLiga</t>
+          <t>Eredivisie</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>flashscore:zs3PZaZa</t>
+          <t>16072838</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-02</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>04:30</t>
+          <t>12:00</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
@@ -176,32 +176,32 @@
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>1777921200</t>
+          <t/>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>live</t>
+          <t>upcoming</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>Sevilla</t>
+          <t>Roda JC Kerkrade</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>flashscore:sevilla</t>
+          <t>2954</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>Real Sociedad</t>
+          <t>RKC Waalwijk</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>flashscore:realsociedad</t>
+          <t>2956</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
@@ -211,7 +211,7 @@
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
@@ -221,119 +221,440 @@
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>ready_for_phase_2</t>
+          <t>needs_settlement</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
         <is>
-          <t>Keyless Flashscore fixture feed.</t>
+          <t>Fallback row from current match_data.json; API-Football key not available. Past fixture is still not confirmed FT.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-05-05 01:28:20 ACST</t>
+          <t>2026-05-06 01:40:37 ACST</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Flashscore</t>
+          <t>local match_data.json</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>healthy</t>
+          <t>source_unverified</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>37</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t/>
+          <t>88</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Premier League</t>
+          <t>Eredivisie</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>flashscore:rTwrFuZR</t>
+          <t>16115678</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>2026-05-05</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
+          <t>02:15</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>Australia/Adelaide</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>upcoming</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>RKC Waalwijk</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>2956</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>Willem II Tilburg</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>2961</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="S3" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="T3" t="inlineStr">
+        <is>
+          <t>source_unverified</t>
+        </is>
+      </c>
+      <c r="U3" t="inlineStr">
+        <is>
+          <t>Fallback row from current match_data.json; API-Football key not available. Primary source did not validate this fixture.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-05-06 01:40:37 ACST</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>local match_data.json</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>source_unverified</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>UEFA Champions League</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>15632635</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>2026-05-06</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
           <t>04:30</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr">
+      <c r="J4" t="inlineStr">
         <is>
           <t>Australia/Adelaide</t>
         </is>
       </c>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>1777921200</t>
-        </is>
-      </c>
-      <c r="L3" t="inlineStr">
-        <is>
-          <t>live</t>
-        </is>
-      </c>
-      <c r="M3" t="inlineStr">
-        <is>
-          <t>Everton</t>
-        </is>
-      </c>
-      <c r="N3" t="inlineStr">
-        <is>
-          <t>flashscore:everton</t>
-        </is>
-      </c>
-      <c r="O3" t="inlineStr">
-        <is>
-          <t>Manchester City</t>
-        </is>
-      </c>
-      <c r="P3" t="inlineStr">
-        <is>
-          <t>flashscore:manchestercity</t>
-        </is>
-      </c>
-      <c r="Q3" t="inlineStr">
+      <c r="K4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>upcoming</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>Arsenal</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>42</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>Atlético Madrid</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>2836</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="R3" t="inlineStr">
+      <c r="R4" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="S3" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="T3" t="inlineStr">
-        <is>
-          <t>ready_for_phase_2</t>
-        </is>
-      </c>
-      <c r="U3" t="inlineStr">
-        <is>
-          <t>Keyless Flashscore fixture feed.</t>
+      <c r="S4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="T4" t="inlineStr">
+        <is>
+          <t>source_unverified</t>
+        </is>
+      </c>
+      <c r="U4" t="inlineStr">
+        <is>
+          <t>Fallback row from current match_data.json; API-Football key not available. Primary source did not validate this fixture.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-05-06 01:40:37 ACST</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>local match_data.json</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>source_unverified</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>37</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>88</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Eredivisie</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>16115794</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>02:15</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>Australia/Adelaide</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>upcoming</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>Almere City FC</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>2990</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>De Graafschap</t>
+        </is>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>2949</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="S5" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="T5" t="inlineStr">
+        <is>
+          <t>source_unverified</t>
+        </is>
+      </c>
+      <c r="U5" t="inlineStr">
+        <is>
+          <t>Fallback row from current match_data.json; API-Football key not available. Primary source did not validate this fixture.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-05-06 01:40:37 ACST</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>local match_data.json</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>source_unverified</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>UEFA Champions League</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>15632634</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>04:30</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>Australia/Adelaide</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>upcoming</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>FC Bayern München</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>2672</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>Paris Saint-Germain</t>
+        </is>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>1644</t>
+        </is>
+      </c>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R6" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="S6" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="T6" t="inlineStr">
+        <is>
+          <t>source_unverified</t>
+        </is>
+      </c>
+      <c r="U6" t="inlineStr">
+        <is>
+          <t>Fallback row from current match_data.json; API-Football key not available. Primary source did not validate this fixture.</t>
         </is>
       </c>
     </row>
@@ -451,220 +772,6 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>2026-05-05 01:28:20 ACST</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Flashscore</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>healthy</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>8</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>LaLiga</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>flashscore:zs3PZaZa</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>2026-05-05</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>04:30</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>Australia/Adelaide</t>
-        </is>
-      </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>1777921200</t>
-        </is>
-      </c>
-      <c r="L2" t="inlineStr">
-        <is>
-          <t>live</t>
-        </is>
-      </c>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>Sevilla</t>
-        </is>
-      </c>
-      <c r="N2" t="inlineStr">
-        <is>
-          <t>flashscore:sevilla</t>
-        </is>
-      </c>
-      <c r="O2" t="inlineStr">
-        <is>
-          <t>Real Sociedad</t>
-        </is>
-      </c>
-      <c r="P2" t="inlineStr">
-        <is>
-          <t>flashscore:realsociedad</t>
-        </is>
-      </c>
-      <c r="Q2" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="R2" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="S2" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="T2" t="inlineStr">
-        <is>
-          <t>ready_for_phase_2</t>
-        </is>
-      </c>
-      <c r="U2" t="inlineStr">
-        <is>
-          <t>Keyless Flashscore fixture feed.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>2026-05-05 01:28:20 ACST</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Flashscore</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>healthy</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>17</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>Premier League</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>flashscore:rTwrFuZR</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>2026-05-05</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>04:30</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>Australia/Adelaide</t>
-        </is>
-      </c>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>1777921200</t>
-        </is>
-      </c>
-      <c r="L3" t="inlineStr">
-        <is>
-          <t>live</t>
-        </is>
-      </c>
-      <c r="M3" t="inlineStr">
-        <is>
-          <t>Everton</t>
-        </is>
-      </c>
-      <c r="N3" t="inlineStr">
-        <is>
-          <t>flashscore:everton</t>
-        </is>
-      </c>
-      <c r="O3" t="inlineStr">
-        <is>
-          <t>Manchester City</t>
-        </is>
-      </c>
-      <c r="P3" t="inlineStr">
-        <is>
-          <t>flashscore:manchestercity</t>
-        </is>
-      </c>
-      <c r="Q3" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="R3" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="S3" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="T3" t="inlineStr">
-        <is>
-          <t>ready_for_phase_2</t>
-        </is>
-      </c>
-      <c r="U3" t="inlineStr">
-        <is>
-          <t>Keyless Flashscore fixture feed.</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
 </worksheet>
 </file>
@@ -779,6 +886,113 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2026-05-06 01:40:37 ACST</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>local match_data.json</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>source_unverified</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>37</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>88</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Eredivisie</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>16072838</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>2026-05-02</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>12:00</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>Australia/Adelaide</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>upcoming</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>Roda JC Kerkrade</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>2954</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>RKC Waalwijk</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>2956</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="S2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="T2" t="inlineStr">
+        <is>
+          <t>needs_settlement</t>
+        </is>
+      </c>
+      <c r="U2" t="inlineStr">
+        <is>
+          <t>Fallback row from current match_data.json; API-Football key not available. Past fixture is still not confirmed FT.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
@@ -893,6 +1107,434 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2026-05-06 01:40:37 ACST</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>local match_data.json</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>source_unverified</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>37</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>88</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Eredivisie</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>16115678</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>2026-05-06</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>02:15</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>Australia/Adelaide</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>upcoming</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>RKC Waalwijk</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>2956</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>Willem II Tilburg</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>2961</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="S2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="T2" t="inlineStr">
+        <is>
+          <t>source_unverified</t>
+        </is>
+      </c>
+      <c r="U2" t="inlineStr">
+        <is>
+          <t>Fallback row from current match_data.json; API-Football key not available. Primary source did not validate this fixture.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-05-06 01:40:37 ACST</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>local match_data.json</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>source_unverified</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>UEFA Champions League</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>15632635</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>2026-05-06</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>04:30</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>Australia/Adelaide</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>upcoming</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>Arsenal</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>42</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>Atlético Madrid</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>2836</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="S3" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="T3" t="inlineStr">
+        <is>
+          <t>source_unverified</t>
+        </is>
+      </c>
+      <c r="U3" t="inlineStr">
+        <is>
+          <t>Fallback row from current match_data.json; API-Football key not available. Primary source did not validate this fixture.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-05-06 01:40:37 ACST</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>local match_data.json</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>source_unverified</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>37</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>88</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Eredivisie</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>16115794</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>02:15</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>Australia/Adelaide</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>upcoming</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>Almere City FC</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>2990</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>De Graafschap</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>2949</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="S4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="T4" t="inlineStr">
+        <is>
+          <t>source_unverified</t>
+        </is>
+      </c>
+      <c r="U4" t="inlineStr">
+        <is>
+          <t>Fallback row from current match_data.json; API-Football key not available. Primary source did not validate this fixture.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-05-06 01:40:37 ACST</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>local match_data.json</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>source_unverified</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>UEFA Champions League</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>15632634</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>04:30</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>Australia/Adelaide</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>upcoming</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>FC Bayern München</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>2672</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>Paris Saint-Germain</t>
+        </is>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>1644</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="S5" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="T5" t="inlineStr">
+        <is>
+          <t>source_unverified</t>
+        </is>
+      </c>
+      <c r="U5" t="inlineStr">
+        <is>
+          <t>Fallback row from current match_data.json; API-Football key not available. Primary source did not validate this fixture.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
@@ -975,27 +1617,27 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>LaLiga</t>
+          <t>Eredivisie</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
           <t>1</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>2</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -1030,12 +1672,12 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>3</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
@@ -1047,17 +1689,17 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Premier League</t>
+          <t>UEFA Champions League</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -1067,7 +1709,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>2</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -1102,12 +1744,12 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>2</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
@@ -1168,7 +1810,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-05-05 01:28:20 ACST</t>
+          <t>2026-05-06 01:40:37 ACST</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -1183,7 +1825,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-05-05 to 2026-05-06</t>
+          <t>2026-05-06 to 2026-05-07</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -1198,12 +1840,54 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>events=295 league_hit=4 skipped_women=0 out_of_window=2 matched=2 by_league={'Premier League': 1, 'LaLiga': 1} sample_leagues=['Albania|ALBANIA: Kategoria e Parë', 'Algeria|ALGERIA: Ligue 1', 'Antigua &amp; Barbuda|ANTIGUA &amp; BARBUDA: ABFA Premier League', 'Argentina|ARGENTINA: Liga Profesional - Apertura', 'Argentina|ARGENTINA: Primera Nacional', 'Argentina|ARGENTINA: Torneo Federal', 'Argentina|ARGENTINA: Primera C', 'Argentina|ARGENTINA: Primera A Women - Apertura']</t>
+          <t>events=231 league_hit=0 skipped_women=0 out_of_window=0 matched=0 by_league={} sample_leagues=['Argentina|ARGENTINA: Liga Profesional - Apertura', 'Argentina|ARGENTINA: Primera Nacional', 'Argentina|ARGENTINA: Primera B', 'Argentina|ARGENTINA: Reserve League - Apertura', 'Armenia|ARMENIA: First League', 'Aruba|ARUBA: Division di Honor - Relegation', 'Asia|ASIA: AFC Asian Cup U17', 'Asia|ASIA: AFC Asian Cup Women U17']</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-05-06 01:40:37 ACST</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>API-Football</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>/fixtures</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>blocked</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Missing API_FOOTBALL_KEY/APISPORTS_KEY; used local match_data.json fallback.</t>
         </is>
       </c>
     </row>
@@ -1234,7 +1918,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-05-05 to 2026-05-06</t>
+          <t>2026-05-06 to 2026-05-07</t>
         </is>
       </c>
     </row>
@@ -1258,7 +1942,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Flashscore</t>
+          <t>local fallback</t>
         </is>
       </c>
     </row>
@@ -1270,7 +1954,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>5</t>
         </is>
       </c>
     </row>
@@ -1282,7 +1966,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0</t>
         </is>
       </c>
     </row>
@@ -1294,7 +1978,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
     </row>
@@ -1306,7 +1990,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>4</t>
         </is>
       </c>
     </row>
@@ -1318,7 +2002,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto-push 2026-05-07T01:37: settle results + forecasts
</commit_message>
<xml_diff>
--- a/docs/agent-system/outputs/Phase1_Fixture_Slate.xlsx
+++ b/docs/agent-system/outputs/Phase1_Fixture_Slate.xlsx
@@ -126,7 +126,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-05-06 01:40:37 ACST</t>
+          <t>2026-05-07 01:36:40 ACST</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -233,7 +233,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-05-06 01:40:37 ACST</t>
+          <t>2026-05-07 01:36:40 ACST</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -263,12 +263,12 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>16115678</t>
+          <t>16115794</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -293,22 +293,22 @@
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>RKC Waalwijk</t>
+          <t>Almere City FC</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>2956</t>
+          <t>2990</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>Willem II Tilburg</t>
+          <t>De Graafschap</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>2961</t>
+          <t>2949</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
@@ -340,7 +340,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-05-06 01:40:37 ACST</t>
+          <t>2026-05-07 01:36:40 ACST</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -370,12 +370,12 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>15632635</t>
+          <t>15632634</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -400,22 +400,22 @@
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>Arsenal</t>
+          <t>FC Bayern München</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>42</t>
+          <t>2672</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>Atlético Madrid</t>
+          <t>Paris Saint-Germain</t>
         </is>
       </c>
       <c r="P4" t="inlineStr">
         <is>
-          <t>2836</t>
+          <t>1644</t>
         </is>
       </c>
       <c r="Q4" t="inlineStr">
@@ -447,7 +447,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-05-06 01:40:37 ACST</t>
+          <t>2026-05-07 01:36:40 ACST</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -462,32 +462,32 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>37</t>
+          <t>35</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>88</t>
+          <t>78</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Eredivisie</t>
+          <t>Bundesliga</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>16115794</t>
+          <t>14065245</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>02:15</t>
+          <t>04:00</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
@@ -507,22 +507,22 @@
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>Almere City FC</t>
+          <t>Borussia Dortmund</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>2990</t>
+          <t>2673</t>
         </is>
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>De Graafschap</t>
+          <t>Eintracht Frankfurt</t>
         </is>
       </c>
       <c r="P5" t="inlineStr">
         <is>
-          <t>2949</t>
+          <t>2674</t>
         </is>
       </c>
       <c r="Q5" t="inlineStr">
@@ -554,7 +554,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-05-06 01:40:37 ACST</t>
+          <t>2026-05-07 01:36:40 ACST</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -569,90 +569,518 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>34</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>61</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>UEFA Champions League</t>
+          <t>Ligue 1</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>15632634</t>
+          <t>14064514</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
+          <t>04:15</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>Australia/Adelaide</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>upcoming</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>RC Lens</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>1648</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>Nantes</t>
+        </is>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>1647</t>
+        </is>
+      </c>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R6" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="S6" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="T6" t="inlineStr">
+        <is>
+          <t>source_unverified</t>
+        </is>
+      </c>
+      <c r="U6" t="inlineStr">
+        <is>
+          <t>Fallback row from current match_data.json; API-Football key not available. Primary source did not validate this fixture.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-05-07 01:36:40 ACST</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>local match_data.json</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>source_unverified</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Championship</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>16116799</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>2026-05-09</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
           <t>04:30</t>
         </is>
       </c>
-      <c r="J6" t="inlineStr">
+      <c r="J7" t="inlineStr">
         <is>
           <t>Australia/Adelaide</t>
         </is>
       </c>
-      <c r="K6" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="L6" t="inlineStr">
+      <c r="K7" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
         <is>
           <t>upcoming</t>
         </is>
       </c>
-      <c r="M6" t="inlineStr">
-        <is>
-          <t>FC Bayern München</t>
-        </is>
-      </c>
-      <c r="N6" t="inlineStr">
-        <is>
-          <t>2672</t>
-        </is>
-      </c>
-      <c r="O6" t="inlineStr">
-        <is>
-          <t>Paris Saint-Germain</t>
-        </is>
-      </c>
-      <c r="P6" t="inlineStr">
-        <is>
-          <t>1644</t>
-        </is>
-      </c>
-      <c r="Q6" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="R6" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="S6" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="T6" t="inlineStr">
-        <is>
-          <t>source_unverified</t>
-        </is>
-      </c>
-      <c r="U6" t="inlineStr">
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>Hull City</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>96</t>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>Millwall</t>
+        </is>
+      </c>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R7" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="S7" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="T7" t="inlineStr">
+        <is>
+          <t>source_unverified</t>
+        </is>
+      </c>
+      <c r="U7" t="inlineStr">
+        <is>
+          <t>Fallback row from current match_data.json; API-Football key not available. Primary source did not validate this fixture.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-05-07 01:36:40 ACST</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>local match_data.json</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>source_unverified</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>140</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>LaLiga</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>14083568</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>2026-05-09</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>04:30</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>Australia/Adelaide</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>upcoming</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>Levante UD</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>2849</t>
+        </is>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>Osasuna</t>
+        </is>
+      </c>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>2820</t>
+        </is>
+      </c>
+      <c r="Q8" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R8" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="S8" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="T8" t="inlineStr">
+        <is>
+          <t>source_unverified</t>
+        </is>
+      </c>
+      <c r="U8" t="inlineStr">
+        <is>
+          <t>Fallback row from current match_data.json; API-Football key not available. Primary source did not validate this fixture.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-05-07 01:36:40 ACST</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>local match_data.json</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>source_unverified</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Championship</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>16116800</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>2026-05-09</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>21:00</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>Australia/Adelaide</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>upcoming</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>Middlesbrough</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>36</t>
+        </is>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>Southampton</t>
+        </is>
+      </c>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t>45</t>
+        </is>
+      </c>
+      <c r="Q9" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R9" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="S9" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="T9" t="inlineStr">
+        <is>
+          <t>source_unverified</t>
+        </is>
+      </c>
+      <c r="U9" t="inlineStr">
+        <is>
+          <t>Fallback row from current match_data.json; API-Football key not available. Primary source did not validate this fixture.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-05-07 01:36:40 ACST</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>local match_data.json</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>source_unverified</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>17</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>39</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Premier League</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>14024024</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>2026-05-09</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>21:00</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>Australia/Adelaide</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>upcoming</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>Liverpool FC</t>
+        </is>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>44</t>
+        </is>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>Chelsea</t>
+        </is>
+      </c>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t>38</t>
+        </is>
+      </c>
+      <c r="Q10" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R10" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="S10" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="T10" t="inlineStr">
+        <is>
+          <t>source_unverified</t>
+        </is>
+      </c>
+      <c r="U10" t="inlineStr">
         <is>
           <t>Fallback row from current match_data.json; API-Football key not available. Primary source did not validate this fixture.</t>
         </is>
@@ -889,7 +1317,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-05-06 01:40:37 ACST</t>
+          <t>2026-05-07 01:36:40 ACST</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -1110,7 +1538,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-05-06 01:40:37 ACST</t>
+          <t>2026-05-07 01:36:40 ACST</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -1140,12 +1568,12 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>16115678</t>
+          <t>16115794</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -1170,22 +1598,22 @@
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>RKC Waalwijk</t>
+          <t>Almere City FC</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>2956</t>
+          <t>2990</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>Willem II Tilburg</t>
+          <t>De Graafschap</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>2961</t>
+          <t>2949</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
@@ -1217,7 +1645,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-05-06 01:40:37 ACST</t>
+          <t>2026-05-07 01:36:40 ACST</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -1247,12 +1675,12 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>15632635</t>
+          <t>15632634</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -1277,22 +1705,22 @@
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>Arsenal</t>
+          <t>FC Bayern München</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>42</t>
+          <t>2672</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>Atlético Madrid</t>
+          <t>Paris Saint-Germain</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>2836</t>
+          <t>1644</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
@@ -1324,7 +1752,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-05-06 01:40:37 ACST</t>
+          <t>2026-05-07 01:36:40 ACST</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -1339,32 +1767,32 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>37</t>
+          <t>35</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>88</t>
+          <t>78</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Eredivisie</t>
+          <t>Bundesliga</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>16115794</t>
+          <t>14065245</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>02:15</t>
+          <t>04:00</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
@@ -1384,22 +1812,22 @@
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>Almere City FC</t>
+          <t>Borussia Dortmund</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>2990</t>
+          <t>2673</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>De Graafschap</t>
+          <t>Eintracht Frankfurt</t>
         </is>
       </c>
       <c r="P4" t="inlineStr">
         <is>
-          <t>2949</t>
+          <t>2674</t>
         </is>
       </c>
       <c r="Q4" t="inlineStr">
@@ -1431,7 +1859,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-05-06 01:40:37 ACST</t>
+          <t>2026-05-07 01:36:40 ACST</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -1446,90 +1874,518 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>34</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>61</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>UEFA Champions League</t>
+          <t>Ligue 1</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>15632634</t>
+          <t>14064514</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
+          <t>04:15</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>Australia/Adelaide</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>upcoming</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>RC Lens</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>1648</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>Nantes</t>
+        </is>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>1647</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="S5" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="T5" t="inlineStr">
+        <is>
+          <t>source_unverified</t>
+        </is>
+      </c>
+      <c r="U5" t="inlineStr">
+        <is>
+          <t>Fallback row from current match_data.json; API-Football key not available. Primary source did not validate this fixture.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-05-07 01:36:40 ACST</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>local match_data.json</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>source_unverified</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Championship</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>16116799</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>2026-05-09</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
           <t>04:30</t>
         </is>
       </c>
-      <c r="J5" t="inlineStr">
+      <c r="J6" t="inlineStr">
         <is>
           <t>Australia/Adelaide</t>
         </is>
       </c>
-      <c r="K5" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="L5" t="inlineStr">
+      <c r="K6" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
         <is>
           <t>upcoming</t>
         </is>
       </c>
-      <c r="M5" t="inlineStr">
-        <is>
-          <t>FC Bayern München</t>
-        </is>
-      </c>
-      <c r="N5" t="inlineStr">
-        <is>
-          <t>2672</t>
-        </is>
-      </c>
-      <c r="O5" t="inlineStr">
-        <is>
-          <t>Paris Saint-Germain</t>
-        </is>
-      </c>
-      <c r="P5" t="inlineStr">
-        <is>
-          <t>1644</t>
-        </is>
-      </c>
-      <c r="Q5" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="R5" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="S5" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="T5" t="inlineStr">
-        <is>
-          <t>source_unverified</t>
-        </is>
-      </c>
-      <c r="U5" t="inlineStr">
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>Hull City</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>96</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>Millwall</t>
+        </is>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R6" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="S6" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="T6" t="inlineStr">
+        <is>
+          <t>source_unverified</t>
+        </is>
+      </c>
+      <c r="U6" t="inlineStr">
+        <is>
+          <t>Fallback row from current match_data.json; API-Football key not available. Primary source did not validate this fixture.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-05-07 01:36:40 ACST</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>local match_data.json</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>source_unverified</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>140</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>LaLiga</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>14083568</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>2026-05-09</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>04:30</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>Australia/Adelaide</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>upcoming</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>Levante UD</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>2849</t>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>Osasuna</t>
+        </is>
+      </c>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>2820</t>
+        </is>
+      </c>
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R7" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="S7" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="T7" t="inlineStr">
+        <is>
+          <t>source_unverified</t>
+        </is>
+      </c>
+      <c r="U7" t="inlineStr">
+        <is>
+          <t>Fallback row from current match_data.json; API-Football key not available. Primary source did not validate this fixture.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-05-07 01:36:40 ACST</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>local match_data.json</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>source_unverified</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Championship</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>16116800</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>2026-05-09</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>21:00</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>Australia/Adelaide</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>upcoming</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>Middlesbrough</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>36</t>
+        </is>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>Southampton</t>
+        </is>
+      </c>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>45</t>
+        </is>
+      </c>
+      <c r="Q8" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R8" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="S8" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="T8" t="inlineStr">
+        <is>
+          <t>source_unverified</t>
+        </is>
+      </c>
+      <c r="U8" t="inlineStr">
+        <is>
+          <t>Fallback row from current match_data.json; API-Football key not available. Primary source did not validate this fixture.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-05-07 01:36:40 ACST</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>local match_data.json</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>source_unverified</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>17</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>39</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Premier League</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>14024024</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>2026-05-09</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>21:00</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>Australia/Adelaide</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>upcoming</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>Liverpool FC</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>44</t>
+        </is>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>Chelsea</t>
+        </is>
+      </c>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t>38</t>
+        </is>
+      </c>
+      <c r="Q9" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="R9" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="S9" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="T9" t="inlineStr">
+        <is>
+          <t>source_unverified</t>
+        </is>
+      </c>
+      <c r="U9" t="inlineStr">
         <is>
           <t>Fallback row from current match_data.json; API-Football key not available. Primary source did not validate this fixture.</t>
         </is>
@@ -1617,12 +2473,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Eredivisie</t>
+          <t>Bundesliga</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -1632,14 +2488,14 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
           <t>1</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
       <c r="F2" t="inlineStr">
         <is>
           <t>0</t>
@@ -1672,7 +2528,7 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
@@ -1689,70 +2545,430 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
+          <t>Championship</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Eredivisie</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>LaLiga</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Ligue 1</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Premier League</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
           <t>UEFA Champions League</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="L3" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="M3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="N3" t="inlineStr">
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr">
         <is>
           <t>0</t>
         </is>
@@ -1810,7 +3026,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-05-06 01:40:37 ACST</t>
+          <t>2026-05-07 01:36:40 ACST</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -1825,7 +3041,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-05-06 to 2026-05-07</t>
+          <t>2026-05-07 to 2026-05-08</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -1845,14 +3061,14 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>events=231 league_hit=0 skipped_women=0 out_of_window=0 matched=0 by_league={} sample_leagues=['Argentina|ARGENTINA: Liga Profesional - Apertura', 'Argentina|ARGENTINA: Primera Nacional', 'Argentina|ARGENTINA: Primera B', 'Argentina|ARGENTINA: Reserve League - Apertura', 'Armenia|ARMENIA: First League', 'Aruba|ARUBA: Division di Honor - Relegation', 'Asia|ASIA: AFC Asian Cup U17', 'Asia|ASIA: AFC Asian Cup Women U17']</t>
+          <t>events=356 league_hit=0 skipped_women=0 out_of_window=0 matched=0 by_league={} sample_leagues=['Albania|ALBANIA: Abissnet Superiore', 'Angola|ANGOLA: Girabola', 'Argentina|ARGENTINA: Reserve League - Apertura', 'Armenia|ARMENIA: Premier League', 'Armenia|ARMENIA: First League', 'Aruba|ARUBA: Division di Honor - Relegation', 'Asia|ASIA: ASEAN Club Championship - Play Offs', 'Asia|ASIA: AFC Asian Cup U17']</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-05-06 01:40:37 ACST</t>
+          <t>2026-05-07 01:36:40 ACST</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -1918,7 +3134,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-05-06 to 2026-05-07</t>
+          <t>2026-05-07 to 2026-05-08</t>
         </is>
       </c>
     </row>
@@ -1954,7 +3170,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>9</t>
         </is>
       </c>
     </row>
@@ -1990,7 +3206,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>8</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto-run 2026-05-16T17:44: settle results + new forecasts + odds refresh
</commit_message>
<xml_diff>
--- a/docs/agent-system/outputs/Phase1_Fixture_Slate.xlsx
+++ b/docs/agent-system/outputs/Phase1_Fixture_Slate.xlsx
@@ -126,7 +126,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-05-16 14:45:11 ACST</t>
+          <t>2026-05-16 17:39:51 ACST</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -233,7 +233,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-05-16 14:45:11 ACST</t>
+          <t>2026-05-16 17:39:51 ACST</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -340,7 +340,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-05-16 14:45:11 ACST</t>
+          <t>2026-05-16 17:39:51 ACST</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -447,7 +447,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-05-16 14:45:11 ACST</t>
+          <t>2026-05-16 17:39:51 ACST</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -554,7 +554,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-05-16 14:45:11 ACST</t>
+          <t>2026-05-16 17:39:51 ACST</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -661,7 +661,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-05-16 14:45:11 ACST</t>
+          <t>2026-05-16 17:39:51 ACST</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -768,7 +768,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-05-16 14:45:11 ACST</t>
+          <t>2026-05-16 17:39:51 ACST</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -875,7 +875,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-05-16 14:45:11 ACST</t>
+          <t>2026-05-16 17:39:51 ACST</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -1096,7 +1096,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-05-16 14:45:11 ACST</t>
+          <t>2026-05-16 17:39:51 ACST</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -1203,7 +1203,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-05-16 14:45:11 ACST</t>
+          <t>2026-05-16 17:39:51 ACST</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -1310,7 +1310,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-05-16 14:45:11 ACST</t>
+          <t>2026-05-16 17:39:51 ACST</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -1417,7 +1417,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-05-16 14:45:11 ACST</t>
+          <t>2026-05-16 17:39:51 ACST</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -1524,7 +1524,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-05-16 14:45:11 ACST</t>
+          <t>2026-05-16 17:39:51 ACST</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -1631,7 +1631,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-05-16 14:45:11 ACST</t>
+          <t>2026-05-16 17:39:51 ACST</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -1738,7 +1738,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-05-16 14:45:11 ACST</t>
+          <t>2026-05-16 17:39:51 ACST</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -1845,7 +1845,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-05-16 14:45:11 ACST</t>
+          <t>2026-05-16 17:39:51 ACST</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -2452,7 +2452,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-05-16 14:45:11 ACST</t>
+          <t>2026-05-16 17:39:51 ACST</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -2487,7 +2487,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>events=1429 league_hit=10 skipped_women=2 out_of_window=0 matched=8 by_league={'Bundesliga': 7, 'MLS': 1} sample_leagues=['Africa|AFRICA: CAF Confederation Cup - Play Offs', 'Africa|AFRICA: Africa Cup of Nations U17', 'Albania|ALBANIA: Abissnet Superiore - Final Group', 'Albania|ALBANIA: Abissnet Superiore - Relegation', 'Algeria|ALGERIA: Ligue 1', 'Algeria|ALGERIA: Ligue 2 - Promotion - Play Offs', 'Andorra|ANDORRA: Primera Divisió', 'Angola|ANGOLA: Girabola']</t>
+          <t>events=1428 league_hit=10 skipped_women=2 out_of_window=0 matched=8 by_league={'Bundesliga': 7, 'MLS': 1} sample_leagues=['Africa|AFRICA: CAF Confederation Cup - Play Offs', 'Africa|AFRICA: Africa Cup of Nations U17', 'Albania|ALBANIA: Abissnet Superiore - Final Group', 'Albania|ALBANIA: Abissnet Superiore - Relegation', 'Algeria|ALGERIA: Ligue 1', 'Algeria|ALGERIA: Ligue 2 - Promotion - Play Offs', 'Andorra|ANDORRA: Primera Divisió', 'Angola|ANGOLA: Girabola']</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto-run 2026-05-16T19:54: settle results + new forecasts + odds refresh
</commit_message>
<xml_diff>
--- a/docs/agent-system/outputs/Phase1_Fixture_Slate.xlsx
+++ b/docs/agent-system/outputs/Phase1_Fixture_Slate.xlsx
@@ -126,7 +126,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-05-16 17:39:51 ACST</t>
+          <t>2026-05-16 19:49:28 ACST</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -233,7 +233,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-05-16 17:39:51 ACST</t>
+          <t>2026-05-16 19:49:28 ACST</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -340,7 +340,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-05-16 17:39:51 ACST</t>
+          <t>2026-05-16 19:49:28 ACST</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -447,7 +447,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-05-16 17:39:51 ACST</t>
+          <t>2026-05-16 19:49:28 ACST</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -554,7 +554,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-05-16 17:39:51 ACST</t>
+          <t>2026-05-16 19:49:28 ACST</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -661,7 +661,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-05-16 17:39:51 ACST</t>
+          <t>2026-05-16 19:49:28 ACST</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -768,7 +768,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-05-16 17:39:51 ACST</t>
+          <t>2026-05-16 19:49:28 ACST</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -875,7 +875,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-05-16 17:39:51 ACST</t>
+          <t>2026-05-16 19:49:28 ACST</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -1096,7 +1096,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-05-16 17:39:51 ACST</t>
+          <t>2026-05-16 19:49:28 ACST</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -1203,7 +1203,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-05-16 17:39:51 ACST</t>
+          <t>2026-05-16 19:49:28 ACST</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -1310,7 +1310,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-05-16 17:39:51 ACST</t>
+          <t>2026-05-16 19:49:28 ACST</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -1417,7 +1417,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-05-16 17:39:51 ACST</t>
+          <t>2026-05-16 19:49:28 ACST</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -1524,7 +1524,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-05-16 17:39:51 ACST</t>
+          <t>2026-05-16 19:49:28 ACST</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -1631,7 +1631,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-05-16 17:39:51 ACST</t>
+          <t>2026-05-16 19:49:28 ACST</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -1738,7 +1738,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-05-16 17:39:51 ACST</t>
+          <t>2026-05-16 19:49:28 ACST</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -1845,7 +1845,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-05-16 17:39:51 ACST</t>
+          <t>2026-05-16 19:49:28 ACST</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -2452,7 +2452,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-05-16 17:39:51 ACST</t>
+          <t>2026-05-16 19:49:28 ACST</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -2487,7 +2487,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>events=1428 league_hit=10 skipped_women=2 out_of_window=0 matched=8 by_league={'Bundesliga': 7, 'MLS': 1} sample_leagues=['Africa|AFRICA: CAF Confederation Cup - Play Offs', 'Africa|AFRICA: Africa Cup of Nations U17', 'Albania|ALBANIA: Abissnet Superiore - Final Group', 'Albania|ALBANIA: Abissnet Superiore - Relegation', 'Algeria|ALGERIA: Ligue 1', 'Algeria|ALGERIA: Ligue 2 - Promotion - Play Offs', 'Andorra|ANDORRA: Primera Divisió', 'Angola|ANGOLA: Girabola']</t>
+          <t>events=1431 league_hit=10 skipped_women=2 out_of_window=0 matched=8 by_league={'Bundesliga': 7, 'MLS': 1} sample_leagues=['Africa|AFRICA: CAF Confederation Cup - Play Offs', 'Africa|AFRICA: Africa Cup of Nations U17', 'Albania|ALBANIA: Abissnet Superiore - Final Group', 'Albania|ALBANIA: Abissnet Superiore - Relegation', 'Algeria|ALGERIA: Ligue 1', 'Algeria|ALGERIA: Ligue 2 - Promotion - Play Offs', 'Andorra|ANDORRA: Primera Divisió', 'Angola|ANGOLA: Girabola']</t>
         </is>
       </c>
     </row>
@@ -2614,7 +2614,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Set API_FOOTBALL_KEY or APISPORTS_KEY before run_daily for live Phase 1 collection.</t>
+          <t>Set API_FOOTBALL_KEY/APISPORTS_KEY for richer Phase 1 collection; TheSportsDB free API is available as fallback.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update dashboard favorites and Firestore data flow
</commit_message>
<xml_diff>
--- a/docs/agent-system/outputs/Phase1_Fixture_Slate.xlsx
+++ b/docs/agent-system/outputs/Phase1_Fixture_Slate.xlsx
@@ -141,7 +141,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-05-17 13:35:09 ACST</t>
+          <t>2026-05-17 16:11:50 ACST</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -156,7 +156,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>242</t>
+          <t>196</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -166,7 +166,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>MLS</t>
+          <t>J1 League</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -176,7 +176,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>flashscore:juAhRoT7</t>
+          <t>flashscore:ClNUHToB</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -186,7 +186,7 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>12:00</t>
+          <t>14:30</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
@@ -196,7 +196,7 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>1778985000</t>
+          <t>1778994000</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
@@ -206,12 +206,12 @@
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>San Jose Earthquakes</t>
+          <t>Chiba</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>flashscore:sanjoseearthquakes</t>
+          <t>flashscore:chiba</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
@@ -221,12 +221,12 @@
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>FC Dallas</t>
+          <t>Kashima Antlers</t>
         </is>
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>flashscore:fcdallas</t>
+          <t>flashscore:kashimaantlers</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
@@ -263,7 +263,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-05-17 13:35:09 ACST</t>
+          <t>2026-05-17 16:11:50 ACST</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -298,7 +298,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>flashscore:GMTLJkHb</t>
+          <t>flashscore:p2LxG7GN</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -308,7 +308,7 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>13:30</t>
+          <t>14:30</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
@@ -318,7 +318,7 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>1778990400</t>
+          <t>1778994000</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
@@ -328,12 +328,12 @@
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>V-Varen Nagasaki</t>
+          <t>Okayama</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>flashscore:vvarennagasaki</t>
+          <t>flashscore:okayama</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
@@ -343,12 +343,12 @@
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>Vissel Kobe</t>
+          <t>Shimizu S-Pulse</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>flashscore:visselkobe</t>
+          <t>flashscore:shimizuspulse</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
@@ -385,7 +385,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-05-17 13:35:09 ACST</t>
+          <t>2026-05-17 16:11:50 ACST</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -420,7 +420,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>flashscore:ClNUHToB</t>
+          <t>flashscore:UPgeYlWi</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -430,7 +430,7 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>14:30</t>
+          <t>15:30</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
@@ -440,7 +440,7 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>1778994000</t>
+          <t>1778997600</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
@@ -450,12 +450,12 @@
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>Chiba</t>
+          <t>Cerezo Osaka</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>flashscore:chiba</t>
+          <t>flashscore:cerezoosaka</t>
         </is>
       </c>
       <c r="P4" t="inlineStr">
@@ -465,12 +465,12 @@
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>Kashima Antlers</t>
+          <t>Nagoya Grampus</t>
         </is>
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>flashscore:kashimaantlers</t>
+          <t>flashscore:nagoyagrampus</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
@@ -507,7 +507,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-05-17 13:35:09 ACST</t>
+          <t>2026-05-17 16:11:50 ACST</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -542,7 +542,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>flashscore:p2LxG7GN</t>
+          <t>flashscore:4n29Aovo</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
@@ -552,7 +552,7 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>14:30</t>
+          <t>15:30</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
@@ -562,7 +562,7 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>1778994000</t>
+          <t>1778997600</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
@@ -572,12 +572,12 @@
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>Okayama</t>
+          <t>Kyoto</t>
         </is>
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>flashscore:okayama</t>
+          <t>flashscore:kyoto</t>
         </is>
       </c>
       <c r="P5" t="inlineStr">
@@ -587,12 +587,12 @@
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>Shimizu S-Pulse</t>
+          <t>Sanfrecce Hiroshima</t>
         </is>
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>flashscore:shimizuspulse</t>
+          <t>flashscore:sanfreccehiroshima</t>
         </is>
       </c>
       <c r="S5" t="inlineStr">
@@ -629,7 +629,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-05-17 13:35:09 ACST</t>
+          <t>2026-05-17 16:11:50 ACST</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -664,7 +664,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>flashscore:UPgeYlWi</t>
+          <t>flashscore:b5oCU6VG</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
@@ -674,7 +674,7 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>15:30</t>
+          <t>19:30</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
@@ -684,7 +684,7 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>1778997600</t>
+          <t>1779012000</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
@@ -694,12 +694,12 @@
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>Cerezo Osaka</t>
+          <t>Kawasaki Frontale</t>
         </is>
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>flashscore:cerezoosaka</t>
+          <t>flashscore:kawasakifrontale</t>
         </is>
       </c>
       <c r="P6" t="inlineStr">
@@ -709,12 +709,12 @@
       </c>
       <c r="Q6" t="inlineStr">
         <is>
-          <t>Nagoya Grampus</t>
+          <t>Machida</t>
         </is>
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>flashscore:nagoyagrampus</t>
+          <t>flashscore:machida</t>
         </is>
       </c>
       <c r="S6" t="inlineStr">
@@ -751,7 +751,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-05-17 13:35:09 ACST</t>
+          <t>2026-05-17 16:11:50 ACST</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -766,7 +766,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>196</t>
+          <t>23</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -776,7 +776,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>J1 League</t>
+          <t>Serie A</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -786,7 +786,7 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>flashscore:4n29Aovo</t>
+          <t>flashscore:jH1dEhfL</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
@@ -796,7 +796,7 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>15:30</t>
+          <t>19:30</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
@@ -806,7 +806,7 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>1778997600</t>
+          <t>1779012000</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
@@ -816,12 +816,12 @@
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>Kyoto</t>
+          <t>AS Roma</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>flashscore:kyoto</t>
+          <t>flashscore:asroma</t>
         </is>
       </c>
       <c r="P7" t="inlineStr">
@@ -831,12 +831,12 @@
       </c>
       <c r="Q7" t="inlineStr">
         <is>
-          <t>Sanfrecce Hiroshima</t>
+          <t>Lazio</t>
         </is>
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>flashscore:sanfreccehiroshima</t>
+          <t>flashscore:lazio</t>
         </is>
       </c>
       <c r="S7" t="inlineStr">
@@ -873,7 +873,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-05-17 13:35:09 ACST</t>
+          <t>2026-05-17 16:11:50 ACST</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -888,7 +888,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>196</t>
+          <t>23</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -898,7 +898,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>J1 League</t>
+          <t>Serie A</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -908,7 +908,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>flashscore:b5oCU6VG</t>
+          <t>flashscore:6V6CE1l4</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
@@ -938,12 +938,12 @@
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>Kawasaki Frontale</t>
+          <t>Como</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>flashscore:kawasakifrontale</t>
+          <t>flashscore:como</t>
         </is>
       </c>
       <c r="P8" t="inlineStr">
@@ -953,12 +953,12 @@
       </c>
       <c r="Q8" t="inlineStr">
         <is>
-          <t>Machida</t>
+          <t>Parma</t>
         </is>
       </c>
       <c r="R8" t="inlineStr">
         <is>
-          <t>flashscore:machida</t>
+          <t>flashscore:parma</t>
         </is>
       </c>
       <c r="S8" t="inlineStr">
@@ -995,7 +995,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-05-17 13:35:09 ACST</t>
+          <t>2026-05-17 16:11:50 ACST</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -1030,7 +1030,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>flashscore:jH1dEhfL</t>
+          <t>flashscore:2c0LCuJG</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
@@ -1060,12 +1060,12 @@
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>AS Roma</t>
+          <t>Genoa</t>
         </is>
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>flashscore:asroma</t>
+          <t>flashscore:genoa</t>
         </is>
       </c>
       <c r="P9" t="inlineStr">
@@ -1075,12 +1075,12 @@
       </c>
       <c r="Q9" t="inlineStr">
         <is>
-          <t>Lazio</t>
+          <t>AC Milan</t>
         </is>
       </c>
       <c r="R9" t="inlineStr">
         <is>
-          <t>flashscore:lazio</t>
+          <t>flashscore:acmilan</t>
         </is>
       </c>
       <c r="S9" t="inlineStr">
@@ -1117,7 +1117,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-05-17 13:35:09 ACST</t>
+          <t>2026-05-17 16:11:50 ACST</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -1152,7 +1152,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>flashscore:6V6CE1l4</t>
+          <t>flashscore:SrG1hBX1</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
@@ -1182,12 +1182,12 @@
       </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>Como</t>
+          <t>Juventus</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>flashscore:como</t>
+          <t>flashscore:juventus</t>
         </is>
       </c>
       <c r="P10" t="inlineStr">
@@ -1197,12 +1197,12 @@
       </c>
       <c r="Q10" t="inlineStr">
         <is>
-          <t>Parma</t>
+          <t>Fiorentina</t>
         </is>
       </c>
       <c r="R10" t="inlineStr">
         <is>
-          <t>flashscore:parma</t>
+          <t>flashscore:fiorentina</t>
         </is>
       </c>
       <c r="S10" t="inlineStr">
@@ -1239,7 +1239,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-05-17 13:35:09 ACST</t>
+          <t>2026-05-17 16:11:50 ACST</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -1274,7 +1274,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>flashscore:2c0LCuJG</t>
+          <t>flashscore:fk8mGEP8</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
@@ -1304,12 +1304,12 @@
       </c>
       <c r="N11" t="inlineStr">
         <is>
-          <t>Genoa</t>
+          <t>Pisa</t>
         </is>
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>flashscore:genoa</t>
+          <t>flashscore:pisa</t>
         </is>
       </c>
       <c r="P11" t="inlineStr">
@@ -1319,12 +1319,12 @@
       </c>
       <c r="Q11" t="inlineStr">
         <is>
-          <t>AC Milan</t>
+          <t>Napoli</t>
         </is>
       </c>
       <c r="R11" t="inlineStr">
         <is>
-          <t>flashscore:acmilan</t>
+          <t>flashscore:napoli</t>
         </is>
       </c>
       <c r="S11" t="inlineStr">
@@ -1361,7 +1361,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-05-17 13:35:09 ACST</t>
+          <t>2026-05-17 16:11:50 ACST</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -1376,7 +1376,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>17</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -1386,7 +1386,7 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Serie A</t>
+          <t>Premier League</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -1396,7 +1396,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>flashscore:SrG1hBX1</t>
+          <t>flashscore:r7lSurwo</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
@@ -1406,7 +1406,7 @@
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>19:30</t>
+          <t>21:00</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
@@ -1416,7 +1416,7 @@
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>1779012000</t>
+          <t>1779017400</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
@@ -1426,12 +1426,12 @@
       </c>
       <c r="N12" t="inlineStr">
         <is>
-          <t>Juventus</t>
+          <t>Manchester Utd</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>flashscore:juventus</t>
+          <t>flashscore:manchesterutd</t>
         </is>
       </c>
       <c r="P12" t="inlineStr">
@@ -1441,12 +1441,12 @@
       </c>
       <c r="Q12" t="inlineStr">
         <is>
-          <t>Fiorentina</t>
+          <t>Nottingham</t>
         </is>
       </c>
       <c r="R12" t="inlineStr">
         <is>
-          <t>flashscore:fiorentina</t>
+          <t>flashscore:nottingham</t>
         </is>
       </c>
       <c r="S12" t="inlineStr">
@@ -1483,7 +1483,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-05-17 13:35:09 ACST</t>
+          <t>2026-05-17 16:11:50 ACST</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1498,7 +1498,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>37</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -1508,7 +1508,7 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Serie A</t>
+          <t>Eredivisie</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -1518,7 +1518,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>flashscore:fk8mGEP8</t>
+          <t>flashscore:h8KKYP3b</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
@@ -1528,7 +1528,7 @@
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>19:30</t>
+          <t>22:00</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
@@ -1538,7 +1538,7 @@
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>1779012000</t>
+          <t>1779021000</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
@@ -1548,12 +1548,12 @@
       </c>
       <c r="N13" t="inlineStr">
         <is>
-          <t>Pisa</t>
+          <t>AZ Alkmaar</t>
         </is>
       </c>
       <c r="O13" t="inlineStr">
         <is>
-          <t>flashscore:pisa</t>
+          <t>flashscore:azalkmaar</t>
         </is>
       </c>
       <c r="P13" t="inlineStr">
@@ -1563,12 +1563,12 @@
       </c>
       <c r="Q13" t="inlineStr">
         <is>
-          <t>Napoli</t>
+          <t>NAC Breda</t>
         </is>
       </c>
       <c r="R13" t="inlineStr">
         <is>
-          <t>flashscore:napoli</t>
+          <t>flashscore:nacbreda</t>
         </is>
       </c>
       <c r="S13" t="inlineStr">
@@ -1605,7 +1605,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-05-17 13:35:09 ACST</t>
+          <t>2026-05-17 16:11:50 ACST</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -1620,7 +1620,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>37</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -1630,7 +1630,7 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Premier League</t>
+          <t>Eredivisie</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -1640,7 +1640,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>flashscore:r7lSurwo</t>
+          <t>flashscore:6Ho2GrlU</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
@@ -1650,7 +1650,7 @@
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>21:00</t>
+          <t>22:00</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
@@ -1660,7 +1660,7 @@
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>1779017400</t>
+          <t>1779021000</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
@@ -1670,12 +1670,12 @@
       </c>
       <c r="N14" t="inlineStr">
         <is>
-          <t>Manchester Utd</t>
+          <t>FC Volendam</t>
         </is>
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>flashscore:manchesterutd</t>
+          <t>flashscore:fcvolendam</t>
         </is>
       </c>
       <c r="P14" t="inlineStr">
@@ -1685,12 +1685,12 @@
       </c>
       <c r="Q14" t="inlineStr">
         <is>
-          <t>Nottingham</t>
+          <t>Telstar</t>
         </is>
       </c>
       <c r="R14" t="inlineStr">
         <is>
-          <t>flashscore:nottingham</t>
+          <t>flashscore:telstar</t>
         </is>
       </c>
       <c r="S14" t="inlineStr">
@@ -1727,7 +1727,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-05-17 13:35:09 ACST</t>
+          <t>2026-05-17 16:11:50 ACST</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1762,7 +1762,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>flashscore:h8KKYP3b</t>
+          <t>flashscore:lIKARQtP</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
@@ -1792,12 +1792,12 @@
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>AZ Alkmaar</t>
+          <t>Heerenveen</t>
         </is>
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>flashscore:azalkmaar</t>
+          <t>flashscore:heerenveen</t>
         </is>
       </c>
       <c r="P15" t="inlineStr">
@@ -1807,12 +1807,12 @@
       </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t>NAC Breda</t>
+          <t>Ajax</t>
         </is>
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>flashscore:nacbreda</t>
+          <t>flashscore:ajax</t>
         </is>
       </c>
       <c r="S15" t="inlineStr">
@@ -1849,7 +1849,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-05-17 13:35:09 ACST</t>
+          <t>2026-05-17 16:11:50 ACST</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -1884,7 +1884,7 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>flashscore:6Ho2GrlU</t>
+          <t>flashscore:p2cgI4JH</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
@@ -1914,12 +1914,12 @@
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>FC Volendam</t>
+          <t>Heracles</t>
         </is>
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>flashscore:fcvolendam</t>
+          <t>flashscore:heracles</t>
         </is>
       </c>
       <c r="P16" t="inlineStr">
@@ -1929,12 +1929,12 @@
       </c>
       <c r="Q16" t="inlineStr">
         <is>
-          <t>Telstar</t>
+          <t>Groningen</t>
         </is>
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>flashscore:telstar</t>
+          <t>flashscore:groningen</t>
         </is>
       </c>
       <c r="S16" t="inlineStr">
@@ -1971,7 +1971,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-05-17 13:35:09 ACST</t>
+          <t>2026-05-17 16:11:50 ACST</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -2006,7 +2006,7 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>flashscore:lIKARQtP</t>
+          <t>flashscore:hfunKQl5</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
@@ -2036,12 +2036,12 @@
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>Heerenveen</t>
+          <t>Nijmegen</t>
         </is>
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>flashscore:heerenveen</t>
+          <t>flashscore:nijmegen</t>
         </is>
       </c>
       <c r="P17" t="inlineStr">
@@ -2051,12 +2051,12 @@
       </c>
       <c r="Q17" t="inlineStr">
         <is>
-          <t>Ajax</t>
+          <t>G.A. Eagles</t>
         </is>
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>flashscore:ajax</t>
+          <t>flashscore:gaeagles</t>
         </is>
       </c>
       <c r="S17" t="inlineStr">
@@ -2093,7 +2093,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-05-17 13:35:09 ACST</t>
+          <t>2026-05-17 16:11:50 ACST</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -2128,7 +2128,7 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>flashscore:p2cgI4JH</t>
+          <t>flashscore:OEmVN8kt</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
@@ -2158,12 +2158,12 @@
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>Heracles</t>
+          <t>PSV</t>
         </is>
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>flashscore:heracles</t>
+          <t>flashscore:psv</t>
         </is>
       </c>
       <c r="P18" t="inlineStr">
@@ -2173,12 +2173,12 @@
       </c>
       <c r="Q18" t="inlineStr">
         <is>
-          <t>Groningen</t>
+          <t>Twente</t>
         </is>
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>flashscore:groningen</t>
+          <t>flashscore:twente</t>
         </is>
       </c>
       <c r="S18" t="inlineStr">
@@ -2215,7 +2215,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-05-17 13:35:09 ACST</t>
+          <t>2026-05-17 16:11:50 ACST</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -2250,7 +2250,7 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>flashscore:hfunKQl5</t>
+          <t>flashscore:21M2TnCC</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
@@ -2280,12 +2280,12 @@
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>Nijmegen</t>
+          <t>Sparta Rotterdam</t>
         </is>
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>flashscore:nijmegen</t>
+          <t>flashscore:spartarotterdam</t>
         </is>
       </c>
       <c r="P19" t="inlineStr">
@@ -2295,12 +2295,12 @@
       </c>
       <c r="Q19" t="inlineStr">
         <is>
-          <t>G.A. Eagles</t>
+          <t>Excelsior</t>
         </is>
       </c>
       <c r="R19" t="inlineStr">
         <is>
-          <t>flashscore:gaeagles</t>
+          <t>flashscore:excelsior</t>
         </is>
       </c>
       <c r="S19" t="inlineStr">
@@ -2337,7 +2337,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-05-17 13:35:09 ACST</t>
+          <t>2026-05-17 16:11:50 ACST</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -2372,7 +2372,7 @@
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>flashscore:OEmVN8kt</t>
+          <t>flashscore:dtRBznZo</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
@@ -2402,12 +2402,12 @@
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>PSV</t>
+          <t>Utrecht</t>
         </is>
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>flashscore:psv</t>
+          <t>flashscore:utrecht</t>
         </is>
       </c>
       <c r="P20" t="inlineStr">
@@ -2417,12 +2417,12 @@
       </c>
       <c r="Q20" t="inlineStr">
         <is>
-          <t>Twente</t>
+          <t>Sittard</t>
         </is>
       </c>
       <c r="R20" t="inlineStr">
         <is>
-          <t>flashscore:twente</t>
+          <t>flashscore:sittard</t>
         </is>
       </c>
       <c r="S20" t="inlineStr">
@@ -2459,7 +2459,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-05-17 13:35:09 ACST</t>
+          <t>2026-05-17 16:11:50 ACST</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -2494,7 +2494,7 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>flashscore:21M2TnCC</t>
+          <t>flashscore:dSowMnKh</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
@@ -2524,12 +2524,12 @@
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>Sparta Rotterdam</t>
+          <t>Zwolle</t>
         </is>
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>flashscore:spartarotterdam</t>
+          <t>flashscore:zwolle</t>
         </is>
       </c>
       <c r="P21" t="inlineStr">
@@ -2539,12 +2539,12 @@
       </c>
       <c r="Q21" t="inlineStr">
         <is>
-          <t>Excelsior</t>
+          <t>Feyenoord</t>
         </is>
       </c>
       <c r="R21" t="inlineStr">
         <is>
-          <t>flashscore:excelsior</t>
+          <t>flashscore:feyenoord</t>
         </is>
       </c>
       <c r="S21" t="inlineStr">
@@ -2581,7 +2581,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-05-17 13:35:09 ACST</t>
+          <t>2026-05-17 16:11:50 ACST</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -2596,7 +2596,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>37</t>
+          <t>23</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -2606,7 +2606,7 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Eredivisie</t>
+          <t>Serie A</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -2616,7 +2616,7 @@
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>flashscore:dtRBznZo</t>
+          <t>flashscore:6TRhfX2k</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
@@ -2626,7 +2626,7 @@
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>22:00</t>
+          <t>22:30</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
@@ -2636,7 +2636,7 @@
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>1779021000</t>
+          <t>1779022800</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
@@ -2646,12 +2646,12 @@
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>Utrecht</t>
+          <t>Inter</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>flashscore:utrecht</t>
+          <t>flashscore:inter</t>
         </is>
       </c>
       <c r="P22" t="inlineStr">
@@ -2661,12 +2661,12 @@
       </c>
       <c r="Q22" t="inlineStr">
         <is>
-          <t>Sittard</t>
+          <t>Verona</t>
         </is>
       </c>
       <c r="R22" t="inlineStr">
         <is>
-          <t>flashscore:sittard</t>
+          <t>flashscore:verona</t>
         </is>
       </c>
       <c r="S22" t="inlineStr">
@@ -2703,7 +2703,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-05-17 13:35:09 ACST</t>
+          <t>2026-05-17 16:11:50 ACST</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -2718,7 +2718,7 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>37</t>
+          <t>17</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -2728,7 +2728,7 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Eredivisie</t>
+          <t>Premier League</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -2738,7 +2738,7 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>flashscore:dSowMnKh</t>
+          <t>flashscore:MF2Xj8on</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
@@ -2748,7 +2748,7 @@
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>22:00</t>
+          <t>23:30</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
@@ -2758,7 +2758,7 @@
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>1779021000</t>
+          <t>1779026400</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
@@ -2768,12 +2768,12 @@
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>Zwolle</t>
+          <t>Brentford</t>
         </is>
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>flashscore:zwolle</t>
+          <t>flashscore:brentford</t>
         </is>
       </c>
       <c r="P23" t="inlineStr">
@@ -2783,12 +2783,12 @@
       </c>
       <c r="Q23" t="inlineStr">
         <is>
-          <t>Feyenoord</t>
+          <t>Crystal Palace</t>
         </is>
       </c>
       <c r="R23" t="inlineStr">
         <is>
-          <t>flashscore:feyenoord</t>
+          <t>flashscore:crystalpalace</t>
         </is>
       </c>
       <c r="S23" t="inlineStr">
@@ -2825,7 +2825,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2026-05-17 13:35:09 ACST</t>
+          <t>2026-05-17 16:11:50 ACST</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -2840,7 +2840,7 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>17</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -2850,7 +2850,7 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Serie A</t>
+          <t>Premier League</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -2860,7 +2860,7 @@
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>flashscore:6TRhfX2k</t>
+          <t>flashscore:jeflmQpB</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
@@ -2870,7 +2870,7 @@
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>22:30</t>
+          <t>23:30</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
@@ -2880,7 +2880,7 @@
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>1779022800</t>
+          <t>1779026400</t>
         </is>
       </c>
       <c r="M24" t="inlineStr">
@@ -2890,12 +2890,12 @@
       </c>
       <c r="N24" t="inlineStr">
         <is>
-          <t>Inter</t>
+          <t>Everton</t>
         </is>
       </c>
       <c r="O24" t="inlineStr">
         <is>
-          <t>flashscore:inter</t>
+          <t>flashscore:everton</t>
         </is>
       </c>
       <c r="P24" t="inlineStr">
@@ -2905,12 +2905,12 @@
       </c>
       <c r="Q24" t="inlineStr">
         <is>
-          <t>Verona</t>
+          <t>Sunderland</t>
         </is>
       </c>
       <c r="R24" t="inlineStr">
         <is>
-          <t>flashscore:verona</t>
+          <t>flashscore:sunderland</t>
         </is>
       </c>
       <c r="S24" t="inlineStr">
@@ -2947,7 +2947,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-05-17 13:35:09 ACST</t>
+          <t>2026-05-17 16:11:50 ACST</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -2982,7 +2982,7 @@
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>flashscore:MF2Xj8on</t>
+          <t>flashscore:OM7eo4FN</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
@@ -3012,12 +3012,12 @@
       </c>
       <c r="N25" t="inlineStr">
         <is>
-          <t>Brentford</t>
+          <t>Leeds</t>
         </is>
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>flashscore:brentford</t>
+          <t>flashscore:leeds</t>
         </is>
       </c>
       <c r="P25" t="inlineStr">
@@ -3027,12 +3027,12 @@
       </c>
       <c r="Q25" t="inlineStr">
         <is>
-          <t>Crystal Palace</t>
+          <t>Brighton</t>
         </is>
       </c>
       <c r="R25" t="inlineStr">
         <is>
-          <t>flashscore:crystalpalace</t>
+          <t>flashscore:brighton</t>
         </is>
       </c>
       <c r="S25" t="inlineStr">
@@ -3069,7 +3069,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2026-05-17 13:35:09 ACST</t>
+          <t>2026-05-17 16:11:50 ACST</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -3084,7 +3084,7 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>196</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -3094,7 +3094,7 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>Premier League</t>
+          <t>J1 League</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -3104,7 +3104,7 @@
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>flashscore:jeflmQpB</t>
+          <t>flashscore:GMTLJkHb</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
@@ -3114,7 +3114,7 @@
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>23:30</t>
+          <t>FT</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
@@ -3124,22 +3124,22 @@
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>1779026400</t>
+          <t>1778990400</t>
         </is>
       </c>
       <c r="M26" t="inlineStr">
         <is>
-          <t>live</t>
+          <t>FT</t>
         </is>
       </c>
       <c r="N26" t="inlineStr">
         <is>
-          <t>Everton</t>
+          <t>V-Varen Nagasaki</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>flashscore:everton</t>
+          <t>flashscore:vvarennagasaki</t>
         </is>
       </c>
       <c r="P26" t="inlineStr">
@@ -3149,12 +3149,12 @@
       </c>
       <c r="Q26" t="inlineStr">
         <is>
-          <t>Sunderland</t>
+          <t>Vissel Kobe</t>
         </is>
       </c>
       <c r="R26" t="inlineStr">
         <is>
-          <t>flashscore:sunderland</t>
+          <t>flashscore:visselkobe</t>
         </is>
       </c>
       <c r="S26" t="inlineStr">
@@ -3191,7 +3191,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-05-17 13:35:09 ACST</t>
+          <t>2026-05-17 16:11:50 ACST</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -3206,7 +3206,7 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>242</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -3216,7 +3216,7 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>Premier League</t>
+          <t>MLS</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -3226,7 +3226,7 @@
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>flashscore:OM7eo4FN</t>
+          <t>flashscore:dIYdxCy9</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
@@ -3236,7 +3236,7 @@
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>23:30</t>
+          <t>FT</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
@@ -3246,22 +3246,22 @@
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>1779026400</t>
+          <t>1778977800</t>
         </is>
       </c>
       <c r="M27" t="inlineStr">
         <is>
-          <t>live</t>
+          <t>FT</t>
         </is>
       </c>
       <c r="N27" t="inlineStr">
         <is>
-          <t>Leeds</t>
+          <t>Austin FC</t>
         </is>
       </c>
       <c r="O27" t="inlineStr">
         <is>
-          <t>flashscore:leeds</t>
+          <t>flashscore:austinfc</t>
         </is>
       </c>
       <c r="P27" t="inlineStr">
@@ -3271,12 +3271,12 @@
       </c>
       <c r="Q27" t="inlineStr">
         <is>
-          <t>Brighton</t>
+          <t>Sporting Kansas City</t>
         </is>
       </c>
       <c r="R27" t="inlineStr">
         <is>
-          <t>flashscore:brighton</t>
+          <t>flashscore:sportingkansascity</t>
         </is>
       </c>
       <c r="S27" t="inlineStr">
@@ -3313,7 +3313,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2026-05-17 13:35:09 ACST</t>
+          <t>2026-05-17 16:11:50 ACST</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -3348,7 +3348,7 @@
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>flashscore:dIYdxCy9</t>
+          <t>flashscore:bX3pLsxi</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
@@ -3368,7 +3368,7 @@
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>1778977800</t>
+          <t>1778963400</t>
         </is>
       </c>
       <c r="M28" t="inlineStr">
@@ -3378,12 +3378,12 @@
       </c>
       <c r="N28" t="inlineStr">
         <is>
-          <t>Austin FC</t>
+          <t>CF Montreal</t>
         </is>
       </c>
       <c r="O28" t="inlineStr">
         <is>
-          <t>flashscore:austinfc</t>
+          <t>flashscore:cfmontreal</t>
         </is>
       </c>
       <c r="P28" t="inlineStr">
@@ -3393,12 +3393,12 @@
       </c>
       <c r="Q28" t="inlineStr">
         <is>
-          <t>Sporting Kansas City</t>
+          <t>Chicago Fire</t>
         </is>
       </c>
       <c r="R28" t="inlineStr">
         <is>
-          <t>flashscore:sportingkansascity</t>
+          <t>flashscore:chicagofire</t>
         </is>
       </c>
       <c r="S28" t="inlineStr">
@@ -3435,7 +3435,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-05-17 13:35:09 ACST</t>
+          <t>2026-05-17 16:11:50 ACST</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -3470,7 +3470,7 @@
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>flashscore:bX3pLsxi</t>
+          <t>flashscore:21IEQ3ET</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
@@ -3490,7 +3490,7 @@
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>1778963400</t>
+          <t>1778974200</t>
         </is>
       </c>
       <c r="M29" t="inlineStr">
@@ -3500,12 +3500,12 @@
       </c>
       <c r="N29" t="inlineStr">
         <is>
-          <t>CF Montreal</t>
+          <t>Charlotte</t>
         </is>
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>flashscore:cfmontreal</t>
+          <t>flashscore:charlotte</t>
         </is>
       </c>
       <c r="P29" t="inlineStr">
@@ -3515,12 +3515,12 @@
       </c>
       <c r="Q29" t="inlineStr">
         <is>
-          <t>Chicago Fire</t>
+          <t>Toronto FC</t>
         </is>
       </c>
       <c r="R29" t="inlineStr">
         <is>
-          <t>flashscore:chicagofire</t>
+          <t>flashscore:torontofc</t>
         </is>
       </c>
       <c r="S29" t="inlineStr">
@@ -3557,7 +3557,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2026-05-17 13:35:09 ACST</t>
+          <t>2026-05-17 16:11:50 ACST</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -3592,7 +3592,7 @@
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>flashscore:21IEQ3ET</t>
+          <t>flashscore:6PmDxLVi</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
@@ -3622,12 +3622,12 @@
       </c>
       <c r="N30" t="inlineStr">
         <is>
-          <t>Charlotte</t>
+          <t>DC United</t>
         </is>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>flashscore:charlotte</t>
+          <t>flashscore:dcunited</t>
         </is>
       </c>
       <c r="P30" t="inlineStr">
@@ -3637,12 +3637,12 @@
       </c>
       <c r="Q30" t="inlineStr">
         <is>
-          <t>Toronto FC</t>
+          <t>St. Louis City</t>
         </is>
       </c>
       <c r="R30" t="inlineStr">
         <is>
-          <t>flashscore:torontofc</t>
+          <t>flashscore:stlouiscity</t>
         </is>
       </c>
       <c r="S30" t="inlineStr">
@@ -3679,7 +3679,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-05-17 13:35:09 ACST</t>
+          <t>2026-05-17 16:11:50 ACST</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -3714,7 +3714,7 @@
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>flashscore:6PmDxLVi</t>
+          <t>flashscore:SvxMza04</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
@@ -3744,12 +3744,12 @@
       </c>
       <c r="N31" t="inlineStr">
         <is>
-          <t>DC United</t>
+          <t>New England Revolution</t>
         </is>
       </c>
       <c r="O31" t="inlineStr">
         <is>
-          <t>flashscore:dcunited</t>
+          <t>flashscore:newenglandrevolution</t>
         </is>
       </c>
       <c r="P31" t="inlineStr">
@@ -3759,12 +3759,12 @@
       </c>
       <c r="Q31" t="inlineStr">
         <is>
-          <t>St. Louis City</t>
+          <t>Minnesota United</t>
         </is>
       </c>
       <c r="R31" t="inlineStr">
         <is>
-          <t>flashscore:stlouiscity</t>
+          <t>flashscore:minnesotaunited</t>
         </is>
       </c>
       <c r="S31" t="inlineStr">
@@ -3801,7 +3801,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2026-05-17 13:35:09 ACST</t>
+          <t>2026-05-17 16:11:50 ACST</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -3836,7 +3836,7 @@
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>flashscore:SvxMza04</t>
+          <t>flashscore:EezUYxVG</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
@@ -3866,12 +3866,12 @@
       </c>
       <c r="N32" t="inlineStr">
         <is>
-          <t>New England Revolution</t>
+          <t>New York Red Bulls</t>
         </is>
       </c>
       <c r="O32" t="inlineStr">
         <is>
-          <t>flashscore:newenglandrevolution</t>
+          <t>flashscore:newyorkredbulls</t>
         </is>
       </c>
       <c r="P32" t="inlineStr">
@@ -3881,12 +3881,12 @@
       </c>
       <c r="Q32" t="inlineStr">
         <is>
-          <t>Minnesota United</t>
+          <t>New York City</t>
         </is>
       </c>
       <c r="R32" t="inlineStr">
         <is>
-          <t>flashscore:minnesotaunited</t>
+          <t>flashscore:newyorkcity</t>
         </is>
       </c>
       <c r="S32" t="inlineStr">
@@ -3923,7 +3923,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-05-17 13:35:09 ACST</t>
+          <t>2026-05-17 16:11:50 ACST</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -3958,7 +3958,7 @@
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>flashscore:EezUYxVG</t>
+          <t>flashscore:8dh2GUEk</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
@@ -3988,12 +3988,12 @@
       </c>
       <c r="N33" t="inlineStr">
         <is>
-          <t>New York Red Bulls</t>
+          <t>Orlando City</t>
         </is>
       </c>
       <c r="O33" t="inlineStr">
         <is>
-          <t>flashscore:newyorkredbulls</t>
+          <t>flashscore:orlandocity</t>
         </is>
       </c>
       <c r="P33" t="inlineStr">
@@ -4003,12 +4003,12 @@
       </c>
       <c r="Q33" t="inlineStr">
         <is>
-          <t>New York City</t>
+          <t>Atlanta Utd</t>
         </is>
       </c>
       <c r="R33" t="inlineStr">
         <is>
-          <t>flashscore:newyorkcity</t>
+          <t>flashscore:atlantautd</t>
         </is>
       </c>
       <c r="S33" t="inlineStr">
@@ -4045,7 +4045,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>2026-05-17 13:35:09 ACST</t>
+          <t>2026-05-17 16:11:50 ACST</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -4080,7 +4080,7 @@
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>flashscore:8dh2GUEk</t>
+          <t>flashscore:tAjAE8q2</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
@@ -4110,12 +4110,12 @@
       </c>
       <c r="N34" t="inlineStr">
         <is>
-          <t>Orlando City</t>
+          <t>Philadelphia Union</t>
         </is>
       </c>
       <c r="O34" t="inlineStr">
         <is>
-          <t>flashscore:orlandocity</t>
+          <t>flashscore:philadelphiaunion</t>
         </is>
       </c>
       <c r="P34" t="inlineStr">
@@ -4125,12 +4125,12 @@
       </c>
       <c r="Q34" t="inlineStr">
         <is>
-          <t>Atlanta Utd</t>
+          <t>Columbus Crew</t>
         </is>
       </c>
       <c r="R34" t="inlineStr">
         <is>
-          <t>flashscore:atlantautd</t>
+          <t>flashscore:columbuscrew</t>
         </is>
       </c>
       <c r="S34" t="inlineStr">
@@ -4167,7 +4167,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-05-17 13:35:09 ACST</t>
+          <t>2026-05-17 16:11:50 ACST</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -4202,7 +4202,7 @@
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>flashscore:tAjAE8q2</t>
+          <t>flashscore:nmDyVTTr</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
@@ -4222,7 +4222,7 @@
       </c>
       <c r="L35" t="inlineStr">
         <is>
-          <t>1778974200</t>
+          <t>1778981400</t>
         </is>
       </c>
       <c r="M35" t="inlineStr">
@@ -4232,12 +4232,12 @@
       </c>
       <c r="N35" t="inlineStr">
         <is>
-          <t>Philadelphia Union</t>
+          <t>Real Salt Lake</t>
         </is>
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>flashscore:philadelphiaunion</t>
+          <t>flashscore:realsaltlake</t>
         </is>
       </c>
       <c r="P35" t="inlineStr">
@@ -4247,12 +4247,12 @@
       </c>
       <c r="Q35" t="inlineStr">
         <is>
-          <t>Columbus Crew</t>
+          <t>Colorado Rapids</t>
         </is>
       </c>
       <c r="R35" t="inlineStr">
         <is>
-          <t>flashscore:columbuscrew</t>
+          <t>flashscore:coloradorapids</t>
         </is>
       </c>
       <c r="S35" t="inlineStr">
@@ -4289,7 +4289,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>2026-05-17 13:35:09 ACST</t>
+          <t>2026-05-17 16:11:50 ACST</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -4324,7 +4324,7 @@
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>flashscore:nmDyVTTr</t>
+          <t>flashscore:fDGqT7be</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
@@ -4354,12 +4354,12 @@
       </c>
       <c r="N36" t="inlineStr">
         <is>
-          <t>Real Salt Lake</t>
+          <t>San Diego FC</t>
         </is>
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>flashscore:realsaltlake</t>
+          <t>flashscore:sandiegofc</t>
         </is>
       </c>
       <c r="P36" t="inlineStr">
@@ -4369,12 +4369,12 @@
       </c>
       <c r="Q36" t="inlineStr">
         <is>
-          <t>Colorado Rapids</t>
+          <t>FC Cincinnati</t>
         </is>
       </c>
       <c r="R36" t="inlineStr">
         <is>
-          <t>flashscore:coloradorapids</t>
+          <t>flashscore:fccincinnati</t>
         </is>
       </c>
       <c r="S36" t="inlineStr">
@@ -4411,7 +4411,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-05-17 13:35:09 ACST</t>
+          <t>2026-05-17 16:11:50 ACST</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -4446,7 +4446,7 @@
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>flashscore:fDGqT7be</t>
+          <t>flashscore:juAhRoT7</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
@@ -4466,7 +4466,7 @@
       </c>
       <c r="L37" t="inlineStr">
         <is>
-          <t>1778981400</t>
+          <t>1778985000</t>
         </is>
       </c>
       <c r="M37" t="inlineStr">
@@ -4476,12 +4476,12 @@
       </c>
       <c r="N37" t="inlineStr">
         <is>
-          <t>San Diego FC</t>
+          <t>San Jose Earthquakes</t>
         </is>
       </c>
       <c r="O37" t="inlineStr">
         <is>
-          <t>flashscore:sandiegofc</t>
+          <t>flashscore:sanjoseearthquakes</t>
         </is>
       </c>
       <c r="P37" t="inlineStr">
@@ -4491,12 +4491,12 @@
       </c>
       <c r="Q37" t="inlineStr">
         <is>
-          <t>FC Cincinnati</t>
+          <t>FC Dallas</t>
         </is>
       </c>
       <c r="R37" t="inlineStr">
         <is>
-          <t>flashscore:fccincinnati</t>
+          <t>flashscore:fcdallas</t>
         </is>
       </c>
       <c r="S37" t="inlineStr">
@@ -4533,7 +4533,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>2026-05-17 13:35:09 ACST</t>
+          <t>2026-05-17 16:11:50 ACST</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -4655,7 +4655,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-05-17 13:35:09 ACST</t>
+          <t>2026-05-17 16:11:50 ACST</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -4777,7 +4777,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>2026-05-17 13:35:09 ACST</t>
+          <t>2026-05-17 16:11:50 ACST</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -4899,7 +4899,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-05-17 13:35:09 ACST</t>
+          <t>2026-05-17 16:11:50 ACST</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -5021,7 +5021,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>2026-05-17 13:35:09 ACST</t>
+          <t>2026-05-17 16:11:50 ACST</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -5143,7 +5143,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-05-17 13:35:09 ACST</t>
+          <t>2026-05-17 16:11:50 ACST</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -5265,7 +5265,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>2026-05-17 13:35:09 ACST</t>
+          <t>2026-05-17 16:11:50 ACST</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -5387,7 +5387,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-05-17 13:35:09 ACST</t>
+          <t>2026-05-17 16:11:50 ACST</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -5509,7 +5509,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>2026-05-17 13:35:09 ACST</t>
+          <t>2026-05-17 16:11:50 ACST</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -5631,7 +5631,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-05-17 13:35:09 ACST</t>
+          <t>2026-05-17 16:11:50 ACST</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -5753,7 +5753,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>2026-05-17 13:35:09 ACST</t>
+          <t>2026-05-17 16:11:50 ACST</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -5875,7 +5875,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-05-17 13:35:09 ACST</t>
+          <t>2026-05-17 16:11:50 ACST</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -5997,7 +5997,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>2026-05-17 13:35:09 ACST</t>
+          <t>2026-05-17 16:11:50 ACST</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -6119,7 +6119,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-05-17 13:35:09 ACST</t>
+          <t>2026-05-17 16:11:50 ACST</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -6241,7 +6241,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>2026-05-17 13:35:09 ACST</t>
+          <t>2026-05-17 16:11:50 ACST</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -6363,7 +6363,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2026-05-17 13:35:09 ACST</t>
+          <t>2026-05-17 16:11:50 ACST</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -6485,7 +6485,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>2026-05-17 13:35:09 ACST</t>
+          <t>2026-05-17 16:11:50 ACST</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -6607,7 +6607,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2026-05-17 13:35:09 ACST</t>
+          <t>2026-05-17 16:11:50 ACST</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -6729,7 +6729,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>2026-05-17 13:35:09 ACST</t>
+          <t>2026-05-17 16:11:50 ACST</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -6851,7 +6851,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>2026-05-17 13:35:09 ACST</t>
+          <t>2026-05-17 16:11:50 ACST</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -6973,7 +6973,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>2026-05-17 13:35:09 ACST</t>
+          <t>2026-05-17 16:11:50 ACST</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -7095,7 +7095,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>2026-05-17 13:35:09 ACST</t>
+          <t>2026-05-17 16:11:50 ACST</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -7217,7 +7217,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>2026-05-17 13:35:09 ACST</t>
+          <t>2026-05-17 16:11:50 ACST</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -7339,7 +7339,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>2026-05-17 13:35:09 ACST</t>
+          <t>2026-05-17 16:11:50 ACST</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -7590,7 +7590,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-05-17 13:35:09 ACST</t>
+          <t>2026-05-17 16:11:50 ACST</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -7605,7 +7605,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>242</t>
+          <t>196</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -7615,7 +7615,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>MLS</t>
+          <t>J1 League</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -7625,7 +7625,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>flashscore:juAhRoT7</t>
+          <t>flashscore:ClNUHToB</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -7635,7 +7635,7 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>12:00</t>
+          <t>14:30</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
@@ -7645,7 +7645,7 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>1778985000</t>
+          <t>1778994000</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
@@ -7655,12 +7655,12 @@
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>San Jose Earthquakes</t>
+          <t>Chiba</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>flashscore:sanjoseearthquakes</t>
+          <t>flashscore:chiba</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
@@ -7670,12 +7670,12 @@
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>FC Dallas</t>
+          <t>Kashima Antlers</t>
         </is>
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>flashscore:fcdallas</t>
+          <t>flashscore:kashimaantlers</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
@@ -7712,7 +7712,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-05-17 13:35:09 ACST</t>
+          <t>2026-05-17 16:11:50 ACST</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -7747,7 +7747,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>flashscore:GMTLJkHb</t>
+          <t>flashscore:p2LxG7GN</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -7757,7 +7757,7 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>13:30</t>
+          <t>14:30</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
@@ -7767,7 +7767,7 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>1778990400</t>
+          <t>1778994000</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
@@ -7777,12 +7777,12 @@
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>V-Varen Nagasaki</t>
+          <t>Okayama</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>flashscore:vvarennagasaki</t>
+          <t>flashscore:okayama</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
@@ -7792,12 +7792,12 @@
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>Vissel Kobe</t>
+          <t>Shimizu S-Pulse</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>flashscore:visselkobe</t>
+          <t>flashscore:shimizuspulse</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
@@ -7834,7 +7834,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-05-17 13:35:09 ACST</t>
+          <t>2026-05-17 16:11:50 ACST</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -7869,7 +7869,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>flashscore:ClNUHToB</t>
+          <t>flashscore:UPgeYlWi</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -7879,7 +7879,7 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>14:30</t>
+          <t>15:30</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
@@ -7889,7 +7889,7 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>1778994000</t>
+          <t>1778997600</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
@@ -7899,12 +7899,12 @@
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>Chiba</t>
+          <t>Cerezo Osaka</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>flashscore:chiba</t>
+          <t>flashscore:cerezoosaka</t>
         </is>
       </c>
       <c r="P4" t="inlineStr">
@@ -7914,12 +7914,12 @@
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>Kashima Antlers</t>
+          <t>Nagoya Grampus</t>
         </is>
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>flashscore:kashimaantlers</t>
+          <t>flashscore:nagoyagrampus</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
@@ -7956,7 +7956,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-05-17 13:35:09 ACST</t>
+          <t>2026-05-17 16:11:50 ACST</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -7991,7 +7991,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>flashscore:p2LxG7GN</t>
+          <t>flashscore:4n29Aovo</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
@@ -8001,7 +8001,7 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>14:30</t>
+          <t>15:30</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
@@ -8011,7 +8011,7 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>1778994000</t>
+          <t>1778997600</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
@@ -8021,12 +8021,12 @@
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>Okayama</t>
+          <t>Kyoto</t>
         </is>
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>flashscore:okayama</t>
+          <t>flashscore:kyoto</t>
         </is>
       </c>
       <c r="P5" t="inlineStr">
@@ -8036,12 +8036,12 @@
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>Shimizu S-Pulse</t>
+          <t>Sanfrecce Hiroshima</t>
         </is>
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>flashscore:shimizuspulse</t>
+          <t>flashscore:sanfreccehiroshima</t>
         </is>
       </c>
       <c r="S5" t="inlineStr">
@@ -8078,7 +8078,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-05-17 13:35:09 ACST</t>
+          <t>2026-05-17 16:11:50 ACST</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -8113,7 +8113,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>flashscore:UPgeYlWi</t>
+          <t>flashscore:b5oCU6VG</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
@@ -8123,7 +8123,7 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>15:30</t>
+          <t>19:30</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
@@ -8133,7 +8133,7 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>1778997600</t>
+          <t>1779012000</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
@@ -8143,12 +8143,12 @@
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>Cerezo Osaka</t>
+          <t>Kawasaki Frontale</t>
         </is>
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>flashscore:cerezoosaka</t>
+          <t>flashscore:kawasakifrontale</t>
         </is>
       </c>
       <c r="P6" t="inlineStr">
@@ -8158,12 +8158,12 @@
       </c>
       <c r="Q6" t="inlineStr">
         <is>
-          <t>Nagoya Grampus</t>
+          <t>Machida</t>
         </is>
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>flashscore:nagoyagrampus</t>
+          <t>flashscore:machida</t>
         </is>
       </c>
       <c r="S6" t="inlineStr">
@@ -8200,7 +8200,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-05-17 13:35:09 ACST</t>
+          <t>2026-05-17 16:11:50 ACST</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -8215,7 +8215,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>196</t>
+          <t>23</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -8225,7 +8225,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>J1 League</t>
+          <t>Serie A</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -8235,7 +8235,7 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>flashscore:4n29Aovo</t>
+          <t>flashscore:jH1dEhfL</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
@@ -8245,7 +8245,7 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>15:30</t>
+          <t>19:30</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
@@ -8255,7 +8255,7 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>1778997600</t>
+          <t>1779012000</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
@@ -8265,12 +8265,12 @@
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>Kyoto</t>
+          <t>AS Roma</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>flashscore:kyoto</t>
+          <t>flashscore:asroma</t>
         </is>
       </c>
       <c r="P7" t="inlineStr">
@@ -8280,12 +8280,12 @@
       </c>
       <c r="Q7" t="inlineStr">
         <is>
-          <t>Sanfrecce Hiroshima</t>
+          <t>Lazio</t>
         </is>
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>flashscore:sanfreccehiroshima</t>
+          <t>flashscore:lazio</t>
         </is>
       </c>
       <c r="S7" t="inlineStr">
@@ -8322,7 +8322,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-05-17 13:35:09 ACST</t>
+          <t>2026-05-17 16:11:50 ACST</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -8337,7 +8337,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>196</t>
+          <t>23</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -8347,7 +8347,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>J1 League</t>
+          <t>Serie A</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -8357,7 +8357,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>flashscore:b5oCU6VG</t>
+          <t>flashscore:6V6CE1l4</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
@@ -8387,12 +8387,12 @@
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>Kawasaki Frontale</t>
+          <t>Como</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>flashscore:kawasakifrontale</t>
+          <t>flashscore:como</t>
         </is>
       </c>
       <c r="P8" t="inlineStr">
@@ -8402,12 +8402,12 @@
       </c>
       <c r="Q8" t="inlineStr">
         <is>
-          <t>Machida</t>
+          <t>Parma</t>
         </is>
       </c>
       <c r="R8" t="inlineStr">
         <is>
-          <t>flashscore:machida</t>
+          <t>flashscore:parma</t>
         </is>
       </c>
       <c r="S8" t="inlineStr">
@@ -8444,7 +8444,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-05-17 13:35:09 ACST</t>
+          <t>2026-05-17 16:11:50 ACST</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -8479,7 +8479,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>flashscore:jH1dEhfL</t>
+          <t>flashscore:2c0LCuJG</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
@@ -8509,12 +8509,12 @@
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>AS Roma</t>
+          <t>Genoa</t>
         </is>
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>flashscore:asroma</t>
+          <t>flashscore:genoa</t>
         </is>
       </c>
       <c r="P9" t="inlineStr">
@@ -8524,12 +8524,12 @@
       </c>
       <c r="Q9" t="inlineStr">
         <is>
-          <t>Lazio</t>
+          <t>AC Milan</t>
         </is>
       </c>
       <c r="R9" t="inlineStr">
         <is>
-          <t>flashscore:lazio</t>
+          <t>flashscore:acmilan</t>
         </is>
       </c>
       <c r="S9" t="inlineStr">
@@ -8566,7 +8566,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-05-17 13:35:09 ACST</t>
+          <t>2026-05-17 16:11:50 ACST</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -8601,7 +8601,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>flashscore:6V6CE1l4</t>
+          <t>flashscore:SrG1hBX1</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
@@ -8631,12 +8631,12 @@
       </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>Como</t>
+          <t>Juventus</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>flashscore:como</t>
+          <t>flashscore:juventus</t>
         </is>
       </c>
       <c r="P10" t="inlineStr">
@@ -8646,12 +8646,12 @@
       </c>
       <c r="Q10" t="inlineStr">
         <is>
-          <t>Parma</t>
+          <t>Fiorentina</t>
         </is>
       </c>
       <c r="R10" t="inlineStr">
         <is>
-          <t>flashscore:parma</t>
+          <t>flashscore:fiorentina</t>
         </is>
       </c>
       <c r="S10" t="inlineStr">
@@ -8688,7 +8688,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-05-17 13:35:09 ACST</t>
+          <t>2026-05-17 16:11:50 ACST</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -8723,7 +8723,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>flashscore:2c0LCuJG</t>
+          <t>flashscore:fk8mGEP8</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
@@ -8753,12 +8753,12 @@
       </c>
       <c r="N11" t="inlineStr">
         <is>
-          <t>Genoa</t>
+          <t>Pisa</t>
         </is>
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>flashscore:genoa</t>
+          <t>flashscore:pisa</t>
         </is>
       </c>
       <c r="P11" t="inlineStr">
@@ -8768,12 +8768,12 @@
       </c>
       <c r="Q11" t="inlineStr">
         <is>
-          <t>AC Milan</t>
+          <t>Napoli</t>
         </is>
       </c>
       <c r="R11" t="inlineStr">
         <is>
-          <t>flashscore:acmilan</t>
+          <t>flashscore:napoli</t>
         </is>
       </c>
       <c r="S11" t="inlineStr">
@@ -8810,7 +8810,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-05-17 13:35:09 ACST</t>
+          <t>2026-05-17 16:11:50 ACST</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -8825,7 +8825,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>17</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -8835,7 +8835,7 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Serie A</t>
+          <t>Premier League</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -8845,7 +8845,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>flashscore:SrG1hBX1</t>
+          <t>flashscore:r7lSurwo</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
@@ -8855,7 +8855,7 @@
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>19:30</t>
+          <t>21:00</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
@@ -8865,7 +8865,7 @@
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>1779012000</t>
+          <t>1779017400</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
@@ -8875,12 +8875,12 @@
       </c>
       <c r="N12" t="inlineStr">
         <is>
-          <t>Juventus</t>
+          <t>Manchester Utd</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>flashscore:juventus</t>
+          <t>flashscore:manchesterutd</t>
         </is>
       </c>
       <c r="P12" t="inlineStr">
@@ -8890,12 +8890,12 @@
       </c>
       <c r="Q12" t="inlineStr">
         <is>
-          <t>Fiorentina</t>
+          <t>Nottingham</t>
         </is>
       </c>
       <c r="R12" t="inlineStr">
         <is>
-          <t>flashscore:fiorentina</t>
+          <t>flashscore:nottingham</t>
         </is>
       </c>
       <c r="S12" t="inlineStr">
@@ -8932,7 +8932,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-05-17 13:35:09 ACST</t>
+          <t>2026-05-17 16:11:50 ACST</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -8947,7 +8947,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>37</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -8957,7 +8957,7 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Serie A</t>
+          <t>Eredivisie</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -8967,7 +8967,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>flashscore:fk8mGEP8</t>
+          <t>flashscore:h8KKYP3b</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
@@ -8977,7 +8977,7 @@
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>19:30</t>
+          <t>22:00</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
@@ -8987,7 +8987,7 @@
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>1779012000</t>
+          <t>1779021000</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
@@ -8997,12 +8997,12 @@
       </c>
       <c r="N13" t="inlineStr">
         <is>
-          <t>Pisa</t>
+          <t>AZ Alkmaar</t>
         </is>
       </c>
       <c r="O13" t="inlineStr">
         <is>
-          <t>flashscore:pisa</t>
+          <t>flashscore:azalkmaar</t>
         </is>
       </c>
       <c r="P13" t="inlineStr">
@@ -9012,12 +9012,12 @@
       </c>
       <c r="Q13" t="inlineStr">
         <is>
-          <t>Napoli</t>
+          <t>NAC Breda</t>
         </is>
       </c>
       <c r="R13" t="inlineStr">
         <is>
-          <t>flashscore:napoli</t>
+          <t>flashscore:nacbreda</t>
         </is>
       </c>
       <c r="S13" t="inlineStr">
@@ -9054,7 +9054,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-05-17 13:35:09 ACST</t>
+          <t>2026-05-17 16:11:50 ACST</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -9069,7 +9069,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>37</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -9079,7 +9079,7 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Premier League</t>
+          <t>Eredivisie</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -9089,7 +9089,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>flashscore:r7lSurwo</t>
+          <t>flashscore:6Ho2GrlU</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
@@ -9099,7 +9099,7 @@
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>21:00</t>
+          <t>22:00</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
@@ -9109,7 +9109,7 @@
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>1779017400</t>
+          <t>1779021000</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
@@ -9119,12 +9119,12 @@
       </c>
       <c r="N14" t="inlineStr">
         <is>
-          <t>Manchester Utd</t>
+          <t>FC Volendam</t>
         </is>
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>flashscore:manchesterutd</t>
+          <t>flashscore:fcvolendam</t>
         </is>
       </c>
       <c r="P14" t="inlineStr">
@@ -9134,12 +9134,12 @@
       </c>
       <c r="Q14" t="inlineStr">
         <is>
-          <t>Nottingham</t>
+          <t>Telstar</t>
         </is>
       </c>
       <c r="R14" t="inlineStr">
         <is>
-          <t>flashscore:nottingham</t>
+          <t>flashscore:telstar</t>
         </is>
       </c>
       <c r="S14" t="inlineStr">
@@ -9176,7 +9176,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-05-17 13:35:09 ACST</t>
+          <t>2026-05-17 16:11:50 ACST</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -9211,7 +9211,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>flashscore:h8KKYP3b</t>
+          <t>flashscore:lIKARQtP</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
@@ -9241,12 +9241,12 @@
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>AZ Alkmaar</t>
+          <t>Heerenveen</t>
         </is>
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>flashscore:azalkmaar</t>
+          <t>flashscore:heerenveen</t>
         </is>
       </c>
       <c r="P15" t="inlineStr">
@@ -9256,12 +9256,12 @@
       </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t>NAC Breda</t>
+          <t>Ajax</t>
         </is>
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>flashscore:nacbreda</t>
+          <t>flashscore:ajax</t>
         </is>
       </c>
       <c r="S15" t="inlineStr">
@@ -9298,7 +9298,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-05-17 13:35:09 ACST</t>
+          <t>2026-05-17 16:11:50 ACST</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -9333,7 +9333,7 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>flashscore:6Ho2GrlU</t>
+          <t>flashscore:p2cgI4JH</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
@@ -9363,12 +9363,12 @@
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>FC Volendam</t>
+          <t>Heracles</t>
         </is>
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>flashscore:fcvolendam</t>
+          <t>flashscore:heracles</t>
         </is>
       </c>
       <c r="P16" t="inlineStr">
@@ -9378,12 +9378,12 @@
       </c>
       <c r="Q16" t="inlineStr">
         <is>
-          <t>Telstar</t>
+          <t>Groningen</t>
         </is>
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>flashscore:telstar</t>
+          <t>flashscore:groningen</t>
         </is>
       </c>
       <c r="S16" t="inlineStr">
@@ -9420,7 +9420,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-05-17 13:35:09 ACST</t>
+          <t>2026-05-17 16:11:50 ACST</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -9455,7 +9455,7 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>flashscore:lIKARQtP</t>
+          <t>flashscore:hfunKQl5</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
@@ -9485,12 +9485,12 @@
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>Heerenveen</t>
+          <t>Nijmegen</t>
         </is>
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>flashscore:heerenveen</t>
+          <t>flashscore:nijmegen</t>
         </is>
       </c>
       <c r="P17" t="inlineStr">
@@ -9500,12 +9500,12 @@
       </c>
       <c r="Q17" t="inlineStr">
         <is>
-          <t>Ajax</t>
+          <t>G.A. Eagles</t>
         </is>
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>flashscore:ajax</t>
+          <t>flashscore:gaeagles</t>
         </is>
       </c>
       <c r="S17" t="inlineStr">
@@ -9542,7 +9542,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-05-17 13:35:09 ACST</t>
+          <t>2026-05-17 16:11:50 ACST</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -9577,7 +9577,7 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>flashscore:p2cgI4JH</t>
+          <t>flashscore:OEmVN8kt</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
@@ -9607,12 +9607,12 @@
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>Heracles</t>
+          <t>PSV</t>
         </is>
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>flashscore:heracles</t>
+          <t>flashscore:psv</t>
         </is>
       </c>
       <c r="P18" t="inlineStr">
@@ -9622,12 +9622,12 @@
       </c>
       <c r="Q18" t="inlineStr">
         <is>
-          <t>Groningen</t>
+          <t>Twente</t>
         </is>
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>flashscore:groningen</t>
+          <t>flashscore:twente</t>
         </is>
       </c>
       <c r="S18" t="inlineStr">
@@ -9664,7 +9664,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-05-17 13:35:09 ACST</t>
+          <t>2026-05-17 16:11:50 ACST</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -9699,7 +9699,7 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>flashscore:hfunKQl5</t>
+          <t>flashscore:21M2TnCC</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
@@ -9729,12 +9729,12 @@
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>Nijmegen</t>
+          <t>Sparta Rotterdam</t>
         </is>
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>flashscore:nijmegen</t>
+          <t>flashscore:spartarotterdam</t>
         </is>
       </c>
       <c r="P19" t="inlineStr">
@@ -9744,12 +9744,12 @@
       </c>
       <c r="Q19" t="inlineStr">
         <is>
-          <t>G.A. Eagles</t>
+          <t>Excelsior</t>
         </is>
       </c>
       <c r="R19" t="inlineStr">
         <is>
-          <t>flashscore:gaeagles</t>
+          <t>flashscore:excelsior</t>
         </is>
       </c>
       <c r="S19" t="inlineStr">
@@ -9786,7 +9786,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-05-17 13:35:09 ACST</t>
+          <t>2026-05-17 16:11:50 ACST</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -9821,7 +9821,7 @@
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>flashscore:OEmVN8kt</t>
+          <t>flashscore:dtRBznZo</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
@@ -9851,12 +9851,12 @@
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>PSV</t>
+          <t>Utrecht</t>
         </is>
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>flashscore:psv</t>
+          <t>flashscore:utrecht</t>
         </is>
       </c>
       <c r="P20" t="inlineStr">
@@ -9866,12 +9866,12 @@
       </c>
       <c r="Q20" t="inlineStr">
         <is>
-          <t>Twente</t>
+          <t>Sittard</t>
         </is>
       </c>
       <c r="R20" t="inlineStr">
         <is>
-          <t>flashscore:twente</t>
+          <t>flashscore:sittard</t>
         </is>
       </c>
       <c r="S20" t="inlineStr">
@@ -9908,7 +9908,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-05-17 13:35:09 ACST</t>
+          <t>2026-05-17 16:11:50 ACST</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -9943,7 +9943,7 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>flashscore:21M2TnCC</t>
+          <t>flashscore:dSowMnKh</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
@@ -9973,12 +9973,12 @@
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>Sparta Rotterdam</t>
+          <t>Zwolle</t>
         </is>
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>flashscore:spartarotterdam</t>
+          <t>flashscore:zwolle</t>
         </is>
       </c>
       <c r="P21" t="inlineStr">
@@ -9988,12 +9988,12 @@
       </c>
       <c r="Q21" t="inlineStr">
         <is>
-          <t>Excelsior</t>
+          <t>Feyenoord</t>
         </is>
       </c>
       <c r="R21" t="inlineStr">
         <is>
-          <t>flashscore:excelsior</t>
+          <t>flashscore:feyenoord</t>
         </is>
       </c>
       <c r="S21" t="inlineStr">
@@ -10030,7 +10030,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-05-17 13:35:09 ACST</t>
+          <t>2026-05-17 16:11:50 ACST</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -10045,7 +10045,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>37</t>
+          <t>23</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -10055,7 +10055,7 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Eredivisie</t>
+          <t>Serie A</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -10065,7 +10065,7 @@
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>flashscore:dtRBznZo</t>
+          <t>flashscore:6TRhfX2k</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
@@ -10075,7 +10075,7 @@
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>22:00</t>
+          <t>22:30</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
@@ -10085,7 +10085,7 @@
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>1779021000</t>
+          <t>1779022800</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
@@ -10095,12 +10095,12 @@
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>Utrecht</t>
+          <t>Inter</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>flashscore:utrecht</t>
+          <t>flashscore:inter</t>
         </is>
       </c>
       <c r="P22" t="inlineStr">
@@ -10110,12 +10110,12 @@
       </c>
       <c r="Q22" t="inlineStr">
         <is>
-          <t>Sittard</t>
+          <t>Verona</t>
         </is>
       </c>
       <c r="R22" t="inlineStr">
         <is>
-          <t>flashscore:sittard</t>
+          <t>flashscore:verona</t>
         </is>
       </c>
       <c r="S22" t="inlineStr">
@@ -10152,7 +10152,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-05-17 13:35:09 ACST</t>
+          <t>2026-05-17 16:11:50 ACST</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -10167,7 +10167,7 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>37</t>
+          <t>17</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -10177,7 +10177,7 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Eredivisie</t>
+          <t>Premier League</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -10187,7 +10187,7 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>flashscore:dSowMnKh</t>
+          <t>flashscore:MF2Xj8on</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
@@ -10197,7 +10197,7 @@
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>22:00</t>
+          <t>23:30</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
@@ -10207,7 +10207,7 @@
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>1779021000</t>
+          <t>1779026400</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
@@ -10217,12 +10217,12 @@
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>Zwolle</t>
+          <t>Brentford</t>
         </is>
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>flashscore:zwolle</t>
+          <t>flashscore:brentford</t>
         </is>
       </c>
       <c r="P23" t="inlineStr">
@@ -10232,12 +10232,12 @@
       </c>
       <c r="Q23" t="inlineStr">
         <is>
-          <t>Feyenoord</t>
+          <t>Crystal Palace</t>
         </is>
       </c>
       <c r="R23" t="inlineStr">
         <is>
-          <t>flashscore:feyenoord</t>
+          <t>flashscore:crystalpalace</t>
         </is>
       </c>
       <c r="S23" t="inlineStr">
@@ -10274,7 +10274,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2026-05-17 13:35:09 ACST</t>
+          <t>2026-05-17 16:11:50 ACST</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -10289,7 +10289,7 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>17</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -10299,7 +10299,7 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Serie A</t>
+          <t>Premier League</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -10309,7 +10309,7 @@
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>flashscore:6TRhfX2k</t>
+          <t>flashscore:jeflmQpB</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
@@ -10319,7 +10319,7 @@
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>22:30</t>
+          <t>23:30</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
@@ -10329,7 +10329,7 @@
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>1779022800</t>
+          <t>1779026400</t>
         </is>
       </c>
       <c r="M24" t="inlineStr">
@@ -10339,12 +10339,12 @@
       </c>
       <c r="N24" t="inlineStr">
         <is>
-          <t>Inter</t>
+          <t>Everton</t>
         </is>
       </c>
       <c r="O24" t="inlineStr">
         <is>
-          <t>flashscore:inter</t>
+          <t>flashscore:everton</t>
         </is>
       </c>
       <c r="P24" t="inlineStr">
@@ -10354,12 +10354,12 @@
       </c>
       <c r="Q24" t="inlineStr">
         <is>
-          <t>Verona</t>
+          <t>Sunderland</t>
         </is>
       </c>
       <c r="R24" t="inlineStr">
         <is>
-          <t>flashscore:verona</t>
+          <t>flashscore:sunderland</t>
         </is>
       </c>
       <c r="S24" t="inlineStr">
@@ -10396,7 +10396,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-05-17 13:35:09 ACST</t>
+          <t>2026-05-17 16:11:50 ACST</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -10431,7 +10431,7 @@
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>flashscore:MF2Xj8on</t>
+          <t>flashscore:OM7eo4FN</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
@@ -10461,12 +10461,12 @@
       </c>
       <c r="N25" t="inlineStr">
         <is>
-          <t>Brentford</t>
+          <t>Leeds</t>
         </is>
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>flashscore:brentford</t>
+          <t>flashscore:leeds</t>
         </is>
       </c>
       <c r="P25" t="inlineStr">
@@ -10476,12 +10476,12 @@
       </c>
       <c r="Q25" t="inlineStr">
         <is>
-          <t>Crystal Palace</t>
+          <t>Brighton</t>
         </is>
       </c>
       <c r="R25" t="inlineStr">
         <is>
-          <t>flashscore:crystalpalace</t>
+          <t>flashscore:brighton</t>
         </is>
       </c>
       <c r="S25" t="inlineStr">
@@ -10518,7 +10518,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2026-05-17 13:35:09 ACST</t>
+          <t>2026-05-17 16:11:50 ACST</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -10533,7 +10533,7 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>196</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -10543,7 +10543,7 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>Premier League</t>
+          <t>J1 League</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -10553,7 +10553,7 @@
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>flashscore:jeflmQpB</t>
+          <t>flashscore:GMTLJkHb</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
@@ -10563,7 +10563,7 @@
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>23:30</t>
+          <t>FT</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
@@ -10573,22 +10573,22 @@
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>1779026400</t>
+          <t>1778990400</t>
         </is>
       </c>
       <c r="M26" t="inlineStr">
         <is>
-          <t>live</t>
+          <t>FT</t>
         </is>
       </c>
       <c r="N26" t="inlineStr">
         <is>
-          <t>Everton</t>
+          <t>V-Varen Nagasaki</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>flashscore:everton</t>
+          <t>flashscore:vvarennagasaki</t>
         </is>
       </c>
       <c r="P26" t="inlineStr">
@@ -10598,12 +10598,12 @@
       </c>
       <c r="Q26" t="inlineStr">
         <is>
-          <t>Sunderland</t>
+          <t>Vissel Kobe</t>
         </is>
       </c>
       <c r="R26" t="inlineStr">
         <is>
-          <t>flashscore:sunderland</t>
+          <t>flashscore:visselkobe</t>
         </is>
       </c>
       <c r="S26" t="inlineStr">
@@ -10640,7 +10640,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-05-17 13:35:09 ACST</t>
+          <t>2026-05-17 16:11:50 ACST</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -10655,7 +10655,7 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>242</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -10665,7 +10665,7 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>Premier League</t>
+          <t>MLS</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -10675,7 +10675,7 @@
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>flashscore:OM7eo4FN</t>
+          <t>flashscore:dIYdxCy9</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
@@ -10685,7 +10685,7 @@
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>23:30</t>
+          <t>FT</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
@@ -10695,22 +10695,22 @@
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>1779026400</t>
+          <t>1778977800</t>
         </is>
       </c>
       <c r="M27" t="inlineStr">
         <is>
-          <t>live</t>
+          <t>FT</t>
         </is>
       </c>
       <c r="N27" t="inlineStr">
         <is>
-          <t>Leeds</t>
+          <t>Austin FC</t>
         </is>
       </c>
       <c r="O27" t="inlineStr">
         <is>
-          <t>flashscore:leeds</t>
+          <t>flashscore:austinfc</t>
         </is>
       </c>
       <c r="P27" t="inlineStr">
@@ -10720,12 +10720,12 @@
       </c>
       <c r="Q27" t="inlineStr">
         <is>
-          <t>Brighton</t>
+          <t>Sporting Kansas City</t>
         </is>
       </c>
       <c r="R27" t="inlineStr">
         <is>
-          <t>flashscore:brighton</t>
+          <t>flashscore:sportingkansascity</t>
         </is>
       </c>
       <c r="S27" t="inlineStr">
@@ -10762,7 +10762,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2026-05-17 13:35:09 ACST</t>
+          <t>2026-05-17 16:11:50 ACST</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -10797,7 +10797,7 @@
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>flashscore:dIYdxCy9</t>
+          <t>flashscore:bX3pLsxi</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
@@ -10817,7 +10817,7 @@
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>1778977800</t>
+          <t>1778963400</t>
         </is>
       </c>
       <c r="M28" t="inlineStr">
@@ -10827,12 +10827,12 @@
       </c>
       <c r="N28" t="inlineStr">
         <is>
-          <t>Austin FC</t>
+          <t>CF Montreal</t>
         </is>
       </c>
       <c r="O28" t="inlineStr">
         <is>
-          <t>flashscore:austinfc</t>
+          <t>flashscore:cfmontreal</t>
         </is>
       </c>
       <c r="P28" t="inlineStr">
@@ -10842,12 +10842,12 @@
       </c>
       <c r="Q28" t="inlineStr">
         <is>
-          <t>Sporting Kansas City</t>
+          <t>Chicago Fire</t>
         </is>
       </c>
       <c r="R28" t="inlineStr">
         <is>
-          <t>flashscore:sportingkansascity</t>
+          <t>flashscore:chicagofire</t>
         </is>
       </c>
       <c r="S28" t="inlineStr">
@@ -10884,7 +10884,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-05-17 13:35:09 ACST</t>
+          <t>2026-05-17 16:11:50 ACST</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -10919,7 +10919,7 @@
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>flashscore:bX3pLsxi</t>
+          <t>flashscore:21IEQ3ET</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
@@ -10939,7 +10939,7 @@
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>1778963400</t>
+          <t>1778974200</t>
         </is>
       </c>
       <c r="M29" t="inlineStr">
@@ -10949,12 +10949,12 @@
       </c>
       <c r="N29" t="inlineStr">
         <is>
-          <t>CF Montreal</t>
+          <t>Charlotte</t>
         </is>
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>flashscore:cfmontreal</t>
+          <t>flashscore:charlotte</t>
         </is>
       </c>
       <c r="P29" t="inlineStr">
@@ -10964,12 +10964,12 @@
       </c>
       <c r="Q29" t="inlineStr">
         <is>
-          <t>Chicago Fire</t>
+          <t>Toronto FC</t>
         </is>
       </c>
       <c r="R29" t="inlineStr">
         <is>
-          <t>flashscore:chicagofire</t>
+          <t>flashscore:torontofc</t>
         </is>
       </c>
       <c r="S29" t="inlineStr">
@@ -11006,7 +11006,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2026-05-17 13:35:09 ACST</t>
+          <t>2026-05-17 16:11:50 ACST</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -11041,7 +11041,7 @@
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>flashscore:21IEQ3ET</t>
+          <t>flashscore:6PmDxLVi</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
@@ -11071,12 +11071,12 @@
       </c>
       <c r="N30" t="inlineStr">
         <is>
-          <t>Charlotte</t>
+          <t>DC United</t>
         </is>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>flashscore:charlotte</t>
+          <t>flashscore:dcunited</t>
         </is>
       </c>
       <c r="P30" t="inlineStr">
@@ -11086,12 +11086,12 @@
       </c>
       <c r="Q30" t="inlineStr">
         <is>
-          <t>Toronto FC</t>
+          <t>St. Louis City</t>
         </is>
       </c>
       <c r="R30" t="inlineStr">
         <is>
-          <t>flashscore:torontofc</t>
+          <t>flashscore:stlouiscity</t>
         </is>
       </c>
       <c r="S30" t="inlineStr">
@@ -11128,7 +11128,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-05-17 13:35:09 ACST</t>
+          <t>2026-05-17 16:11:50 ACST</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -11163,7 +11163,7 @@
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>flashscore:6PmDxLVi</t>
+          <t>flashscore:SvxMza04</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
@@ -11193,12 +11193,12 @@
       </c>
       <c r="N31" t="inlineStr">
         <is>
-          <t>DC United</t>
+          <t>New England Revolution</t>
         </is>
       </c>
       <c r="O31" t="inlineStr">
         <is>
-          <t>flashscore:dcunited</t>
+          <t>flashscore:newenglandrevolution</t>
         </is>
       </c>
       <c r="P31" t="inlineStr">
@@ -11208,12 +11208,12 @@
       </c>
       <c r="Q31" t="inlineStr">
         <is>
-          <t>St. Louis City</t>
+          <t>Minnesota United</t>
         </is>
       </c>
       <c r="R31" t="inlineStr">
         <is>
-          <t>flashscore:stlouiscity</t>
+          <t>flashscore:minnesotaunited</t>
         </is>
       </c>
       <c r="S31" t="inlineStr">
@@ -11250,7 +11250,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2026-05-17 13:35:09 ACST</t>
+          <t>2026-05-17 16:11:50 ACST</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -11285,7 +11285,7 @@
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>flashscore:SvxMza04</t>
+          <t>flashscore:EezUYxVG</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
@@ -11315,12 +11315,12 @@
       </c>
       <c r="N32" t="inlineStr">
         <is>
-          <t>New England Revolution</t>
+          <t>New York Red Bulls</t>
         </is>
       </c>
       <c r="O32" t="inlineStr">
         <is>
-          <t>flashscore:newenglandrevolution</t>
+          <t>flashscore:newyorkredbulls</t>
         </is>
       </c>
       <c r="P32" t="inlineStr">
@@ -11330,12 +11330,12 @@
       </c>
       <c r="Q32" t="inlineStr">
         <is>
-          <t>Minnesota United</t>
+          <t>New York City</t>
         </is>
       </c>
       <c r="R32" t="inlineStr">
         <is>
-          <t>flashscore:minnesotaunited</t>
+          <t>flashscore:newyorkcity</t>
         </is>
       </c>
       <c r="S32" t="inlineStr">
@@ -11372,7 +11372,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-05-17 13:35:09 ACST</t>
+          <t>2026-05-17 16:11:50 ACST</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -11407,7 +11407,7 @@
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>flashscore:EezUYxVG</t>
+          <t>flashscore:8dh2GUEk</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
@@ -11437,12 +11437,12 @@
       </c>
       <c r="N33" t="inlineStr">
         <is>
-          <t>New York Red Bulls</t>
+          <t>Orlando City</t>
         </is>
       </c>
       <c r="O33" t="inlineStr">
         <is>
-          <t>flashscore:newyorkredbulls</t>
+          <t>flashscore:orlandocity</t>
         </is>
       </c>
       <c r="P33" t="inlineStr">
@@ -11452,12 +11452,12 @@
       </c>
       <c r="Q33" t="inlineStr">
         <is>
-          <t>New York City</t>
+          <t>Atlanta Utd</t>
         </is>
       </c>
       <c r="R33" t="inlineStr">
         <is>
-          <t>flashscore:newyorkcity</t>
+          <t>flashscore:atlantautd</t>
         </is>
       </c>
       <c r="S33" t="inlineStr">
@@ -11494,7 +11494,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>2026-05-17 13:35:09 ACST</t>
+          <t>2026-05-17 16:11:50 ACST</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -11529,7 +11529,7 @@
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>flashscore:8dh2GUEk</t>
+          <t>flashscore:tAjAE8q2</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
@@ -11559,12 +11559,12 @@
       </c>
       <c r="N34" t="inlineStr">
         <is>
-          <t>Orlando City</t>
+          <t>Philadelphia Union</t>
         </is>
       </c>
       <c r="O34" t="inlineStr">
         <is>
-          <t>flashscore:orlandocity</t>
+          <t>flashscore:philadelphiaunion</t>
         </is>
       </c>
       <c r="P34" t="inlineStr">
@@ -11574,12 +11574,12 @@
       </c>
       <c r="Q34" t="inlineStr">
         <is>
-          <t>Atlanta Utd</t>
+          <t>Columbus Crew</t>
         </is>
       </c>
       <c r="R34" t="inlineStr">
         <is>
-          <t>flashscore:atlantautd</t>
+          <t>flashscore:columbuscrew</t>
         </is>
       </c>
       <c r="S34" t="inlineStr">
@@ -11616,7 +11616,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-05-17 13:35:09 ACST</t>
+          <t>2026-05-17 16:11:50 ACST</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -11651,7 +11651,7 @@
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>flashscore:tAjAE8q2</t>
+          <t>flashscore:nmDyVTTr</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
@@ -11671,7 +11671,7 @@
       </c>
       <c r="L35" t="inlineStr">
         <is>
-          <t>1778974200</t>
+          <t>1778981400</t>
         </is>
       </c>
       <c r="M35" t="inlineStr">
@@ -11681,12 +11681,12 @@
       </c>
       <c r="N35" t="inlineStr">
         <is>
-          <t>Philadelphia Union</t>
+          <t>Real Salt Lake</t>
         </is>
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>flashscore:philadelphiaunion</t>
+          <t>flashscore:realsaltlake</t>
         </is>
       </c>
       <c r="P35" t="inlineStr">
@@ -11696,12 +11696,12 @@
       </c>
       <c r="Q35" t="inlineStr">
         <is>
-          <t>Columbus Crew</t>
+          <t>Colorado Rapids</t>
         </is>
       </c>
       <c r="R35" t="inlineStr">
         <is>
-          <t>flashscore:columbuscrew</t>
+          <t>flashscore:coloradorapids</t>
         </is>
       </c>
       <c r="S35" t="inlineStr">
@@ -11738,7 +11738,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>2026-05-17 13:35:09 ACST</t>
+          <t>2026-05-17 16:11:50 ACST</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -11773,7 +11773,7 @@
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>flashscore:nmDyVTTr</t>
+          <t>flashscore:fDGqT7be</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
@@ -11803,12 +11803,12 @@
       </c>
       <c r="N36" t="inlineStr">
         <is>
-          <t>Real Salt Lake</t>
+          <t>San Diego FC</t>
         </is>
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>flashscore:realsaltlake</t>
+          <t>flashscore:sandiegofc</t>
         </is>
       </c>
       <c r="P36" t="inlineStr">
@@ -11818,12 +11818,12 @@
       </c>
       <c r="Q36" t="inlineStr">
         <is>
-          <t>Colorado Rapids</t>
+          <t>FC Cincinnati</t>
         </is>
       </c>
       <c r="R36" t="inlineStr">
         <is>
-          <t>flashscore:coloradorapids</t>
+          <t>flashscore:fccincinnati</t>
         </is>
       </c>
       <c r="S36" t="inlineStr">
@@ -11860,7 +11860,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-05-17 13:35:09 ACST</t>
+          <t>2026-05-17 16:11:50 ACST</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -11895,7 +11895,7 @@
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>flashscore:fDGqT7be</t>
+          <t>flashscore:juAhRoT7</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
@@ -11915,7 +11915,7 @@
       </c>
       <c r="L37" t="inlineStr">
         <is>
-          <t>1778981400</t>
+          <t>1778985000</t>
         </is>
       </c>
       <c r="M37" t="inlineStr">
@@ -11925,12 +11925,12 @@
       </c>
       <c r="N37" t="inlineStr">
         <is>
-          <t>San Diego FC</t>
+          <t>San Jose Earthquakes</t>
         </is>
       </c>
       <c r="O37" t="inlineStr">
         <is>
-          <t>flashscore:sandiegofc</t>
+          <t>flashscore:sanjoseearthquakes</t>
         </is>
       </c>
       <c r="P37" t="inlineStr">
@@ -11940,12 +11940,12 @@
       </c>
       <c r="Q37" t="inlineStr">
         <is>
-          <t>FC Cincinnati</t>
+          <t>FC Dallas</t>
         </is>
       </c>
       <c r="R37" t="inlineStr">
         <is>
-          <t>flashscore:fccincinnati</t>
+          <t>flashscore:fcdallas</t>
         </is>
       </c>
       <c r="S37" t="inlineStr">
@@ -11982,7 +11982,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>2026-05-17 13:35:09 ACST</t>
+          <t>2026-05-17 16:11:50 ACST</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -12104,7 +12104,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-05-17 13:35:09 ACST</t>
+          <t>2026-05-17 16:11:50 ACST</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -12226,7 +12226,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>2026-05-17 13:35:09 ACST</t>
+          <t>2026-05-17 16:11:50 ACST</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -12348,7 +12348,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-05-17 13:35:09 ACST</t>
+          <t>2026-05-17 16:11:50 ACST</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -12470,7 +12470,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>2026-05-17 13:35:09 ACST</t>
+          <t>2026-05-17 16:11:50 ACST</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -12592,7 +12592,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-05-17 13:35:09 ACST</t>
+          <t>2026-05-17 16:11:50 ACST</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -12714,7 +12714,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>2026-05-17 13:35:09 ACST</t>
+          <t>2026-05-17 16:11:50 ACST</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -12836,7 +12836,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-05-17 13:35:09 ACST</t>
+          <t>2026-05-17 16:11:50 ACST</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -12958,7 +12958,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>2026-05-17 13:35:09 ACST</t>
+          <t>2026-05-17 16:11:50 ACST</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -13080,7 +13080,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-05-17 13:35:09 ACST</t>
+          <t>2026-05-17 16:11:50 ACST</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -13202,7 +13202,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>2026-05-17 13:35:09 ACST</t>
+          <t>2026-05-17 16:11:50 ACST</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -13324,7 +13324,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-05-17 13:35:09 ACST</t>
+          <t>2026-05-17 16:11:50 ACST</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -13446,7 +13446,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>2026-05-17 13:35:09 ACST</t>
+          <t>2026-05-17 16:11:50 ACST</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -13568,7 +13568,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-05-17 13:35:09 ACST</t>
+          <t>2026-05-17 16:11:50 ACST</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -13690,7 +13690,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>2026-05-17 13:35:09 ACST</t>
+          <t>2026-05-17 16:11:50 ACST</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -13812,7 +13812,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2026-05-17 13:35:09 ACST</t>
+          <t>2026-05-17 16:11:50 ACST</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -13934,7 +13934,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>2026-05-17 13:35:09 ACST</t>
+          <t>2026-05-17 16:11:50 ACST</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -14056,7 +14056,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2026-05-17 13:35:09 ACST</t>
+          <t>2026-05-17 16:11:50 ACST</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -14178,7 +14178,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>2026-05-17 13:35:09 ACST</t>
+          <t>2026-05-17 16:11:50 ACST</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -14300,7 +14300,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>2026-05-17 13:35:09 ACST</t>
+          <t>2026-05-17 16:11:50 ACST</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -14422,7 +14422,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>2026-05-17 13:35:09 ACST</t>
+          <t>2026-05-17 16:11:50 ACST</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -14544,7 +14544,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>2026-05-17 13:35:09 ACST</t>
+          <t>2026-05-17 16:11:50 ACST</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -14666,7 +14666,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>2026-05-17 13:35:09 ACST</t>
+          <t>2026-05-17 16:11:50 ACST</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -14788,7 +14788,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>2026-05-17 13:35:09 ACST</t>
+          <t>2026-05-17 16:11:50 ACST</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -15379,12 +15379,12 @@
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>5</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
     </row>
@@ -15595,12 +15595,12 @@
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>12</t>
         </is>
       </c>
     </row>
@@ -15800,7 +15800,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-05-17 13:35:09 ACST</t>
+          <t>2026-05-17 16:11:50 ACST</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -15815,7 +15815,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-05-17 to 2026-05-18</t>
+          <t>2026-05-17 to 2026-05-23</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -15866,7 +15866,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-05-17 to 2026-05-18</t>
+          <t>2026-05-17 to 2026-05-23</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Wire results review summaries
</commit_message>
<xml_diff>
--- a/docs/agent-system/outputs/Phase1_Fixture_Slate.xlsx
+++ b/docs/agent-system/outputs/Phase1_Fixture_Slate.xlsx
@@ -141,7 +141,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-05-18 01:55:05 ACST</t>
+          <t>2026-05-18 04:02:28 ACST</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -156,7 +156,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>8</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -166,7 +166,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Serie A</t>
+          <t>LaLiga</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -176,7 +176,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>flashscore:I9QHhKRp</t>
+          <t>flashscore:vyaxjXte</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -186,7 +186,7 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>01:30</t>
+          <t>02:30</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
@@ -196,7 +196,7 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>1779033600</t>
+          <t>1779037200</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
@@ -206,12 +206,12 @@
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>Atalanta</t>
+          <t>Ath. Bilbao</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>flashscore:atalanta</t>
+          <t>flashscore:athbilbao</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
@@ -221,12 +221,12 @@
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>Bologna</t>
+          <t>Celta Vigo</t>
         </is>
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>flashscore:bologna</t>
+          <t>flashscore:celtavigo</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
@@ -263,7 +263,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-05-18 01:55:05 ACST</t>
+          <t>2026-05-18 04:02:28 ACST</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -298,7 +298,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>flashscore:vyaxjXte</t>
+          <t>flashscore:n12plBB7</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -328,12 +328,12 @@
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>Ath Bilbao</t>
+          <t>Atl. Madrid</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>flashscore:athbilbao</t>
+          <t>flashscore:atlmadrid</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
@@ -343,12 +343,12 @@
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>Celta Vigo</t>
+          <t>Girona</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>flashscore:celtavigo</t>
+          <t>flashscore:girona</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
@@ -385,7 +385,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-05-18 01:55:05 ACST</t>
+          <t>2026-05-18 04:02:28 ACST</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -420,7 +420,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>flashscore:n12plBB7</t>
+          <t>flashscore:0OhvAhYQ</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -450,12 +450,12 @@
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>Atl. Madrid</t>
+          <t>Elche</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>flashscore:atlmadrid</t>
+          <t>flashscore:elche</t>
         </is>
       </c>
       <c r="P4" t="inlineStr">
@@ -465,12 +465,12 @@
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>Girona</t>
+          <t>Getafe</t>
         </is>
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>flashscore:girona</t>
+          <t>flashscore:getafe</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
@@ -507,7 +507,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-05-18 01:55:05 ACST</t>
+          <t>2026-05-18 04:02:28 ACST</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -542,7 +542,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>flashscore:0OhvAhYQ</t>
+          <t>flashscore:K8ZA4Wel</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
@@ -572,12 +572,12 @@
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>Elche</t>
+          <t>Levante</t>
         </is>
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>flashscore:elche</t>
+          <t>flashscore:levante</t>
         </is>
       </c>
       <c r="P5" t="inlineStr">
@@ -587,12 +587,12 @@
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>Getafe</t>
+          <t>Mallorca</t>
         </is>
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>flashscore:getafe</t>
+          <t>flashscore:mallorca</t>
         </is>
       </c>
       <c r="S5" t="inlineStr">
@@ -629,7 +629,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-05-18 01:55:05 ACST</t>
+          <t>2026-05-18 04:02:28 ACST</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -664,7 +664,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>flashscore:K8ZA4Wel</t>
+          <t>flashscore:YFVo6qXh</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
@@ -694,12 +694,12 @@
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>Levante</t>
+          <t>Osasuna</t>
         </is>
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>flashscore:levante</t>
+          <t>flashscore:osasuna</t>
         </is>
       </c>
       <c r="P6" t="inlineStr">
@@ -709,12 +709,12 @@
       </c>
       <c r="Q6" t="inlineStr">
         <is>
-          <t>Mallorca</t>
+          <t>Espanyol</t>
         </is>
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>flashscore:mallorca</t>
+          <t>flashscore:espanyol</t>
         </is>
       </c>
       <c r="S6" t="inlineStr">
@@ -751,7 +751,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-05-18 01:55:05 ACST</t>
+          <t>2026-05-18 04:02:28 ACST</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -786,7 +786,7 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>flashscore:YFVo6qXh</t>
+          <t>flashscore:C0sw852t</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
@@ -816,12 +816,12 @@
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>Osasuna</t>
+          <t>Oviedo</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>flashscore:osasuna</t>
+          <t>flashscore:oviedo</t>
         </is>
       </c>
       <c r="P7" t="inlineStr">
@@ -831,12 +831,12 @@
       </c>
       <c r="Q7" t="inlineStr">
         <is>
-          <t>Espanyol</t>
+          <t>Alaves</t>
         </is>
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>flashscore:espanyol</t>
+          <t>flashscore:alaves</t>
         </is>
       </c>
       <c r="S7" t="inlineStr">
@@ -873,7 +873,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-05-18 01:55:05 ACST</t>
+          <t>2026-05-18 04:02:28 ACST</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -908,7 +908,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>flashscore:C0sw852t</t>
+          <t>flashscore:llRR0leD</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
@@ -938,12 +938,12 @@
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>Oviedo</t>
+          <t>Real Sociedad</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>flashscore:oviedo</t>
+          <t>flashscore:realsociedad</t>
         </is>
       </c>
       <c r="P8" t="inlineStr">
@@ -953,12 +953,12 @@
       </c>
       <c r="Q8" t="inlineStr">
         <is>
-          <t>Alaves</t>
+          <t>Valencia</t>
         </is>
       </c>
       <c r="R8" t="inlineStr">
         <is>
-          <t>flashscore:alaves</t>
+          <t>flashscore:valencia</t>
         </is>
       </c>
       <c r="S8" t="inlineStr">
@@ -995,7 +995,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-05-18 01:55:05 ACST</t>
+          <t>2026-05-18 04:02:28 ACST</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -1030,7 +1030,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>flashscore:hMXI2AQ0</t>
+          <t>flashscore:ttZg4N15</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
@@ -1060,12 +1060,12 @@
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>Rayo Vallecano</t>
+          <t>Sevilla</t>
         </is>
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>flashscore:rayovallecano</t>
+          <t>flashscore:sevilla</t>
         </is>
       </c>
       <c r="P9" t="inlineStr">
@@ -1075,12 +1075,12 @@
       </c>
       <c r="Q9" t="inlineStr">
         <is>
-          <t>Villarreal</t>
+          <t>Real Madrid</t>
         </is>
       </c>
       <c r="R9" t="inlineStr">
         <is>
-          <t>flashscore:villarreal</t>
+          <t>flashscore:realmadrid</t>
         </is>
       </c>
       <c r="S9" t="inlineStr">
@@ -1117,7 +1117,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-05-18 01:55:05 ACST</t>
+          <t>2026-05-18 04:02:28 ACST</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -1152,7 +1152,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>flashscore:llRR0leD</t>
+          <t>flashscore:hMXI2AQ0</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
@@ -1182,12 +1182,12 @@
       </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>Real Sociedad</t>
+          <t>Vallecano</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>flashscore:realsociedad</t>
+          <t>flashscore:vallecano</t>
         </is>
       </c>
       <c r="P10" t="inlineStr">
@@ -1197,12 +1197,12 @@
       </c>
       <c r="Q10" t="inlineStr">
         <is>
-          <t>Valencia</t>
+          <t>Villarreal</t>
         </is>
       </c>
       <c r="R10" t="inlineStr">
         <is>
-          <t>flashscore:valencia</t>
+          <t>flashscore:villarreal</t>
         </is>
       </c>
       <c r="S10" t="inlineStr">
@@ -1239,7 +1239,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-05-18 01:55:05 ACST</t>
+          <t>2026-05-18 04:02:28 ACST</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -1254,7 +1254,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>23</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -1264,7 +1264,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>LaLiga</t>
+          <t>Serie A</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -1274,7 +1274,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>flashscore:ttZg4N15</t>
+          <t>flashscore:YH84GNJi</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
@@ -1284,7 +1284,7 @@
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>02:30</t>
+          <t>04:15</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
@@ -1294,7 +1294,7 @@
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>1779037200</t>
+          <t>1779043500</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
@@ -1304,12 +1304,12 @@
       </c>
       <c r="N11" t="inlineStr">
         <is>
-          <t>Sevilla</t>
+          <t>Cagliari</t>
         </is>
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>flashscore:sevilla</t>
+          <t>flashscore:cagliari</t>
         </is>
       </c>
       <c r="P11" t="inlineStr">
@@ -1319,12 +1319,12 @@
       </c>
       <c r="Q11" t="inlineStr">
         <is>
-          <t>Real Madrid</t>
+          <t>Torino</t>
         </is>
       </c>
       <c r="R11" t="inlineStr">
         <is>
-          <t>flashscore:realmadrid</t>
+          <t>flashscore:torino</t>
         </is>
       </c>
       <c r="S11" t="inlineStr">
@@ -1361,7 +1361,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-05-18 01:55:05 ACST</t>
+          <t>2026-05-18 04:02:28 ACST</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -1396,7 +1396,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>flashscore:YH84GNJi</t>
+          <t>flashscore:nmmS8WHr</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
@@ -1426,12 +1426,12 @@
       </c>
       <c r="N12" t="inlineStr">
         <is>
-          <t>Cagliari</t>
+          <t>Sassuolo</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>flashscore:cagliari</t>
+          <t>flashscore:sassuolo</t>
         </is>
       </c>
       <c r="P12" t="inlineStr">
@@ -1441,12 +1441,12 @@
       </c>
       <c r="Q12" t="inlineStr">
         <is>
-          <t>Torino</t>
+          <t>Lecce</t>
         </is>
       </c>
       <c r="R12" t="inlineStr">
         <is>
-          <t>flashscore:torino</t>
+          <t>flashscore:lecce</t>
         </is>
       </c>
       <c r="S12" t="inlineStr">
@@ -1483,7 +1483,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-05-18 01:55:05 ACST</t>
+          <t>2026-05-18 04:02:28 ACST</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1518,7 +1518,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>flashscore:nmmS8WHr</t>
+          <t>flashscore:h0IS6Ane</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
@@ -1548,12 +1548,12 @@
       </c>
       <c r="N13" t="inlineStr">
         <is>
-          <t>Sassuolo</t>
+          <t>Udinese</t>
         </is>
       </c>
       <c r="O13" t="inlineStr">
         <is>
-          <t>flashscore:sassuolo</t>
+          <t>flashscore:udinese</t>
         </is>
       </c>
       <c r="P13" t="inlineStr">
@@ -1563,12 +1563,12 @@
       </c>
       <c r="Q13" t="inlineStr">
         <is>
-          <t>Lecce</t>
+          <t>Cremonese</t>
         </is>
       </c>
       <c r="R13" t="inlineStr">
         <is>
-          <t>flashscore:lecce</t>
+          <t>flashscore:cremonese</t>
         </is>
       </c>
       <c r="S13" t="inlineStr">
@@ -1605,7 +1605,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-05-18 01:55:05 ACST</t>
+          <t>2026-05-18 04:02:28 ACST</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -1620,7 +1620,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>34</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -1630,7 +1630,7 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Serie A</t>
+          <t>Ligue 1</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -1640,7 +1640,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>flashscore:h0IS6Ane</t>
+          <t>flashscore:prPnPy9r</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
@@ -1650,7 +1650,7 @@
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>04:15</t>
+          <t>04:30</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
@@ -1660,7 +1660,7 @@
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>1779043500</t>
+          <t>1779044400</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
@@ -1670,12 +1670,12 @@
       </c>
       <c r="N14" t="inlineStr">
         <is>
-          <t>Udinese</t>
+          <t>Brest</t>
         </is>
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>flashscore:udinese</t>
+          <t>flashscore:brest</t>
         </is>
       </c>
       <c r="P14" t="inlineStr">
@@ -1685,12 +1685,12 @@
       </c>
       <c r="Q14" t="inlineStr">
         <is>
-          <t>Cremonese</t>
+          <t>Angers</t>
         </is>
       </c>
       <c r="R14" t="inlineStr">
         <is>
-          <t>flashscore:cremonese</t>
+          <t>flashscore:angers</t>
         </is>
       </c>
       <c r="S14" t="inlineStr">
@@ -1727,7 +1727,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-05-18 01:55:05 ACST</t>
+          <t>2026-05-18 04:02:28 ACST</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1762,7 +1762,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>flashscore:prPnPy9r</t>
+          <t>flashscore:IXv8WJG8</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
@@ -1792,12 +1792,12 @@
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>Brest</t>
+          <t>Lille</t>
         </is>
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>flashscore:brest</t>
+          <t>flashscore:lille</t>
         </is>
       </c>
       <c r="P15" t="inlineStr">
@@ -1807,12 +1807,12 @@
       </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t>Angers</t>
+          <t>Auxerre</t>
         </is>
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>flashscore:angers</t>
+          <t>flashscore:auxerre</t>
         </is>
       </c>
       <c r="S15" t="inlineStr">
@@ -1849,7 +1849,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-05-18 01:55:05 ACST</t>
+          <t>2026-05-18 04:02:28 ACST</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -1884,7 +1884,7 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>flashscore:IXv8WJG8</t>
+          <t>flashscore:r1cGQTSk</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
@@ -1914,12 +1914,12 @@
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>Lille</t>
+          <t>Lorient</t>
         </is>
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>flashscore:lille</t>
+          <t>flashscore:lorient</t>
         </is>
       </c>
       <c r="P16" t="inlineStr">
@@ -1929,12 +1929,12 @@
       </c>
       <c r="Q16" t="inlineStr">
         <is>
-          <t>Auxerre</t>
+          <t>Le Havre</t>
         </is>
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>flashscore:auxerre</t>
+          <t>flashscore:lehavre</t>
         </is>
       </c>
       <c r="S16" t="inlineStr">
@@ -1971,7 +1971,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-05-18 01:55:05 ACST</t>
+          <t>2026-05-18 04:02:28 ACST</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -2006,7 +2006,7 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>flashscore:r1cGQTSk</t>
+          <t>flashscore:OhrGQlpm</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
@@ -2036,12 +2036,12 @@
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>Lorient</t>
+          <t>Lyon</t>
         </is>
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>flashscore:lorient</t>
+          <t>flashscore:lyon</t>
         </is>
       </c>
       <c r="P17" t="inlineStr">
@@ -2051,12 +2051,12 @@
       </c>
       <c r="Q17" t="inlineStr">
         <is>
-          <t>Le Havre</t>
+          <t>Lens</t>
         </is>
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>flashscore:lehavre</t>
+          <t>flashscore:lens</t>
         </is>
       </c>
       <c r="S17" t="inlineStr">
@@ -2093,7 +2093,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-05-18 01:55:05 ACST</t>
+          <t>2026-05-18 04:02:28 ACST</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -2128,7 +2128,7 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>flashscore:OhrGQlpm</t>
+          <t>flashscore:xbwdLg87</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
@@ -2158,12 +2158,12 @@
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>Lyon</t>
+          <t>Marseille</t>
         </is>
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>flashscore:lyon</t>
+          <t>flashscore:marseille</t>
         </is>
       </c>
       <c r="P18" t="inlineStr">
@@ -2173,12 +2173,12 @@
       </c>
       <c r="Q18" t="inlineStr">
         <is>
-          <t>Lens</t>
+          <t>Rennes</t>
         </is>
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>flashscore:lens</t>
+          <t>flashscore:rennes</t>
         </is>
       </c>
       <c r="S18" t="inlineStr">
@@ -2215,7 +2215,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-05-18 01:55:05 ACST</t>
+          <t>2026-05-18 04:02:28 ACST</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -2250,7 +2250,7 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>flashscore:xbwdLg87</t>
+          <t>flashscore:z9FNO7c2</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
@@ -2280,12 +2280,12 @@
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>Marseille</t>
+          <t>Nantes</t>
         </is>
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>flashscore:marseille</t>
+          <t>flashscore:nantes</t>
         </is>
       </c>
       <c r="P19" t="inlineStr">
@@ -2295,12 +2295,12 @@
       </c>
       <c r="Q19" t="inlineStr">
         <is>
-          <t>Rennes</t>
+          <t>Toulouse</t>
         </is>
       </c>
       <c r="R19" t="inlineStr">
         <is>
-          <t>flashscore:rennes</t>
+          <t>flashscore:toulouse</t>
         </is>
       </c>
       <c r="S19" t="inlineStr">
@@ -2337,7 +2337,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-05-18 01:55:05 ACST</t>
+          <t>2026-05-18 04:02:28 ACST</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -2372,7 +2372,7 @@
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>flashscore:z9FNO7c2</t>
+          <t>flashscore:QcrGUcoL</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
@@ -2402,12 +2402,12 @@
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>Nantes</t>
+          <t>Nice</t>
         </is>
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>flashscore:nantes</t>
+          <t>flashscore:nice</t>
         </is>
       </c>
       <c r="P20" t="inlineStr">
@@ -2417,12 +2417,12 @@
       </c>
       <c r="Q20" t="inlineStr">
         <is>
-          <t>Toulouse</t>
+          <t>Metz</t>
         </is>
       </c>
       <c r="R20" t="inlineStr">
         <is>
-          <t>flashscore:toulouse</t>
+          <t>flashscore:metz</t>
         </is>
       </c>
       <c r="S20" t="inlineStr">
@@ -2459,7 +2459,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-05-18 01:55:05 ACST</t>
+          <t>2026-05-18 04:02:28 ACST</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -2494,7 +2494,7 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>flashscore:QcrGUcoL</t>
+          <t>flashscore:IeNfNFwe</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
@@ -2524,12 +2524,12 @@
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>Nice</t>
+          <t>Paris FC</t>
         </is>
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>flashscore:nice</t>
+          <t>flashscore:parisfc</t>
         </is>
       </c>
       <c r="P21" t="inlineStr">
@@ -2539,12 +2539,12 @@
       </c>
       <c r="Q21" t="inlineStr">
         <is>
-          <t>Metz</t>
+          <t>PSG</t>
         </is>
       </c>
       <c r="R21" t="inlineStr">
         <is>
-          <t>flashscore:metz</t>
+          <t>flashscore:psg</t>
         </is>
       </c>
       <c r="S21" t="inlineStr">
@@ -2581,7 +2581,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-05-18 01:55:05 ACST</t>
+          <t>2026-05-18 04:02:28 ACST</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -2616,7 +2616,7 @@
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>flashscore:IeNfNFwe</t>
+          <t>flashscore:44Vsqc0E</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
@@ -2646,12 +2646,12 @@
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>Paris FC</t>
+          <t>Strasbourg</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>flashscore:parisfc</t>
+          <t>flashscore:strasbourg</t>
         </is>
       </c>
       <c r="P22" t="inlineStr">
@@ -2661,12 +2661,12 @@
       </c>
       <c r="Q22" t="inlineStr">
         <is>
-          <t>PSG</t>
+          <t>Monaco</t>
         </is>
       </c>
       <c r="R22" t="inlineStr">
         <is>
-          <t>flashscore:psg</t>
+          <t>flashscore:monaco</t>
         </is>
       </c>
       <c r="S22" t="inlineStr">
@@ -2703,7 +2703,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-05-18 01:55:05 ACST</t>
+          <t>2026-05-18 04:02:28 ACST</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -2718,7 +2718,7 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>34</t>
+          <t>8</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -2728,7 +2728,7 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Ligue 1</t>
+          <t>LaLiga</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -2738,7 +2738,7 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>flashscore:44Vsqc0E</t>
+          <t>flashscore:SduXBE3E</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
@@ -2748,7 +2748,7 @@
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>04:30</t>
+          <t>04:45</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
@@ -2758,7 +2758,7 @@
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>1779044400</t>
+          <t>1779045300</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
@@ -2768,12 +2768,12 @@
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>Strasbourg</t>
+          <t>Barcelona</t>
         </is>
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>flashscore:strasbourg</t>
+          <t>flashscore:barcelona</t>
         </is>
       </c>
       <c r="P23" t="inlineStr">
@@ -2783,12 +2783,12 @@
       </c>
       <c r="Q23" t="inlineStr">
         <is>
-          <t>Monaco</t>
+          <t>Betis</t>
         </is>
       </c>
       <c r="R23" t="inlineStr">
         <is>
-          <t>flashscore:monaco</t>
+          <t>flashscore:betis</t>
         </is>
       </c>
       <c r="S23" t="inlineStr">
@@ -2825,7 +2825,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2026-05-18 01:55:05 ACST</t>
+          <t>2026-05-18 04:02:28 ACST</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -2840,7 +2840,7 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>23</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -2850,7 +2850,7 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>LaLiga</t>
+          <t>Serie A</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -2860,7 +2860,7 @@
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>flashscore:SduXBE3E</t>
+          <t>flashscore:I9QHhKRp</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
@@ -2870,7 +2870,7 @@
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>04:45</t>
+          <t>FT</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
@@ -2880,22 +2880,22 @@
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>1779045300</t>
+          <t>1779033600</t>
         </is>
       </c>
       <c r="M24" t="inlineStr">
         <is>
-          <t>live</t>
+          <t>FT</t>
         </is>
       </c>
       <c r="N24" t="inlineStr">
         <is>
-          <t>Barcelona</t>
+          <t>Atalanta</t>
         </is>
       </c>
       <c r="O24" t="inlineStr">
         <is>
-          <t>flashscore:barcelona</t>
+          <t>flashscore:atalanta</t>
         </is>
       </c>
       <c r="P24" t="inlineStr">
@@ -2905,12 +2905,12 @@
       </c>
       <c r="Q24" t="inlineStr">
         <is>
-          <t>Betis</t>
+          <t>Bologna</t>
         </is>
       </c>
       <c r="R24" t="inlineStr">
         <is>
-          <t>flashscore:betis</t>
+          <t>flashscore:bologna</t>
         </is>
       </c>
       <c r="S24" t="inlineStr">
@@ -3076,7 +3076,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-05-18 01:55:05 ACST</t>
+          <t>2026-05-18 04:02:28 ACST</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -3091,7 +3091,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>8</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -3101,7 +3101,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Serie A</t>
+          <t>LaLiga</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -3111,7 +3111,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>flashscore:I9QHhKRp</t>
+          <t>flashscore:vyaxjXte</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -3121,7 +3121,7 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>01:30</t>
+          <t>02:30</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
@@ -3131,7 +3131,7 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>1779033600</t>
+          <t>1779037200</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
@@ -3141,12 +3141,12 @@
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>Atalanta</t>
+          <t>Ath. Bilbao</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>flashscore:atalanta</t>
+          <t>flashscore:athbilbao</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
@@ -3156,12 +3156,12 @@
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>Bologna</t>
+          <t>Celta Vigo</t>
         </is>
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>flashscore:bologna</t>
+          <t>flashscore:celtavigo</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
@@ -3198,7 +3198,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-05-18 01:55:05 ACST</t>
+          <t>2026-05-18 04:02:28 ACST</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -3233,7 +3233,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>flashscore:vyaxjXte</t>
+          <t>flashscore:n12plBB7</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -3263,12 +3263,12 @@
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>Ath Bilbao</t>
+          <t>Atl. Madrid</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>flashscore:athbilbao</t>
+          <t>flashscore:atlmadrid</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
@@ -3278,12 +3278,12 @@
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>Celta Vigo</t>
+          <t>Girona</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>flashscore:celtavigo</t>
+          <t>flashscore:girona</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
@@ -3320,7 +3320,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-05-18 01:55:05 ACST</t>
+          <t>2026-05-18 04:02:28 ACST</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -3355,7 +3355,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>flashscore:n12plBB7</t>
+          <t>flashscore:0OhvAhYQ</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -3385,12 +3385,12 @@
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>Atl. Madrid</t>
+          <t>Elche</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>flashscore:atlmadrid</t>
+          <t>flashscore:elche</t>
         </is>
       </c>
       <c r="P4" t="inlineStr">
@@ -3400,12 +3400,12 @@
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>Girona</t>
+          <t>Getafe</t>
         </is>
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>flashscore:girona</t>
+          <t>flashscore:getafe</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
@@ -3442,7 +3442,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-05-18 01:55:05 ACST</t>
+          <t>2026-05-18 04:02:28 ACST</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -3477,7 +3477,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>flashscore:0OhvAhYQ</t>
+          <t>flashscore:K8ZA4Wel</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
@@ -3507,12 +3507,12 @@
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>Elche</t>
+          <t>Levante</t>
         </is>
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>flashscore:elche</t>
+          <t>flashscore:levante</t>
         </is>
       </c>
       <c r="P5" t="inlineStr">
@@ -3522,12 +3522,12 @@
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>Getafe</t>
+          <t>Mallorca</t>
         </is>
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>flashscore:getafe</t>
+          <t>flashscore:mallorca</t>
         </is>
       </c>
       <c r="S5" t="inlineStr">
@@ -3564,7 +3564,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-05-18 01:55:05 ACST</t>
+          <t>2026-05-18 04:02:28 ACST</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -3599,7 +3599,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>flashscore:K8ZA4Wel</t>
+          <t>flashscore:YFVo6qXh</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
@@ -3629,12 +3629,12 @@
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>Levante</t>
+          <t>Osasuna</t>
         </is>
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>flashscore:levante</t>
+          <t>flashscore:osasuna</t>
         </is>
       </c>
       <c r="P6" t="inlineStr">
@@ -3644,12 +3644,12 @@
       </c>
       <c r="Q6" t="inlineStr">
         <is>
-          <t>Mallorca</t>
+          <t>Espanyol</t>
         </is>
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>flashscore:mallorca</t>
+          <t>flashscore:espanyol</t>
         </is>
       </c>
       <c r="S6" t="inlineStr">
@@ -3686,7 +3686,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-05-18 01:55:05 ACST</t>
+          <t>2026-05-18 04:02:28 ACST</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -3721,7 +3721,7 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>flashscore:YFVo6qXh</t>
+          <t>flashscore:C0sw852t</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
@@ -3751,12 +3751,12 @@
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>Osasuna</t>
+          <t>Oviedo</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>flashscore:osasuna</t>
+          <t>flashscore:oviedo</t>
         </is>
       </c>
       <c r="P7" t="inlineStr">
@@ -3766,12 +3766,12 @@
       </c>
       <c r="Q7" t="inlineStr">
         <is>
-          <t>Espanyol</t>
+          <t>Alaves</t>
         </is>
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>flashscore:espanyol</t>
+          <t>flashscore:alaves</t>
         </is>
       </c>
       <c r="S7" t="inlineStr">
@@ -3808,7 +3808,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-05-18 01:55:05 ACST</t>
+          <t>2026-05-18 04:02:28 ACST</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -3843,7 +3843,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>flashscore:C0sw852t</t>
+          <t>flashscore:llRR0leD</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
@@ -3873,12 +3873,12 @@
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>Oviedo</t>
+          <t>Real Sociedad</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>flashscore:oviedo</t>
+          <t>flashscore:realsociedad</t>
         </is>
       </c>
       <c r="P8" t="inlineStr">
@@ -3888,12 +3888,12 @@
       </c>
       <c r="Q8" t="inlineStr">
         <is>
-          <t>Alaves</t>
+          <t>Valencia</t>
         </is>
       </c>
       <c r="R8" t="inlineStr">
         <is>
-          <t>flashscore:alaves</t>
+          <t>flashscore:valencia</t>
         </is>
       </c>
       <c r="S8" t="inlineStr">
@@ -3930,7 +3930,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-05-18 01:55:05 ACST</t>
+          <t>2026-05-18 04:02:28 ACST</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -3965,7 +3965,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>flashscore:hMXI2AQ0</t>
+          <t>flashscore:ttZg4N15</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
@@ -3995,12 +3995,12 @@
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>Rayo Vallecano</t>
+          <t>Sevilla</t>
         </is>
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>flashscore:rayovallecano</t>
+          <t>flashscore:sevilla</t>
         </is>
       </c>
       <c r="P9" t="inlineStr">
@@ -4010,12 +4010,12 @@
       </c>
       <c r="Q9" t="inlineStr">
         <is>
-          <t>Villarreal</t>
+          <t>Real Madrid</t>
         </is>
       </c>
       <c r="R9" t="inlineStr">
         <is>
-          <t>flashscore:villarreal</t>
+          <t>flashscore:realmadrid</t>
         </is>
       </c>
       <c r="S9" t="inlineStr">
@@ -4052,7 +4052,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-05-18 01:55:05 ACST</t>
+          <t>2026-05-18 04:02:28 ACST</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -4087,7 +4087,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>flashscore:llRR0leD</t>
+          <t>flashscore:hMXI2AQ0</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
@@ -4117,12 +4117,12 @@
       </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>Real Sociedad</t>
+          <t>Vallecano</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>flashscore:realsociedad</t>
+          <t>flashscore:vallecano</t>
         </is>
       </c>
       <c r="P10" t="inlineStr">
@@ -4132,12 +4132,12 @@
       </c>
       <c r="Q10" t="inlineStr">
         <is>
-          <t>Valencia</t>
+          <t>Villarreal</t>
         </is>
       </c>
       <c r="R10" t="inlineStr">
         <is>
-          <t>flashscore:valencia</t>
+          <t>flashscore:villarreal</t>
         </is>
       </c>
       <c r="S10" t="inlineStr">
@@ -4174,7 +4174,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-05-18 01:55:05 ACST</t>
+          <t>2026-05-18 04:02:28 ACST</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -4189,7 +4189,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>23</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -4199,7 +4199,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>LaLiga</t>
+          <t>Serie A</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -4209,7 +4209,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>flashscore:ttZg4N15</t>
+          <t>flashscore:YH84GNJi</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
@@ -4219,7 +4219,7 @@
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>02:30</t>
+          <t>04:15</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
@@ -4229,7 +4229,7 @@
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>1779037200</t>
+          <t>1779043500</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
@@ -4239,12 +4239,12 @@
       </c>
       <c r="N11" t="inlineStr">
         <is>
-          <t>Sevilla</t>
+          <t>Cagliari</t>
         </is>
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>flashscore:sevilla</t>
+          <t>flashscore:cagliari</t>
         </is>
       </c>
       <c r="P11" t="inlineStr">
@@ -4254,12 +4254,12 @@
       </c>
       <c r="Q11" t="inlineStr">
         <is>
-          <t>Real Madrid</t>
+          <t>Torino</t>
         </is>
       </c>
       <c r="R11" t="inlineStr">
         <is>
-          <t>flashscore:realmadrid</t>
+          <t>flashscore:torino</t>
         </is>
       </c>
       <c r="S11" t="inlineStr">
@@ -4296,7 +4296,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-05-18 01:55:05 ACST</t>
+          <t>2026-05-18 04:02:28 ACST</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -4331,7 +4331,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>flashscore:YH84GNJi</t>
+          <t>flashscore:nmmS8WHr</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
@@ -4361,12 +4361,12 @@
       </c>
       <c r="N12" t="inlineStr">
         <is>
-          <t>Cagliari</t>
+          <t>Sassuolo</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>flashscore:cagliari</t>
+          <t>flashscore:sassuolo</t>
         </is>
       </c>
       <c r="P12" t="inlineStr">
@@ -4376,12 +4376,12 @@
       </c>
       <c r="Q12" t="inlineStr">
         <is>
-          <t>Torino</t>
+          <t>Lecce</t>
         </is>
       </c>
       <c r="R12" t="inlineStr">
         <is>
-          <t>flashscore:torino</t>
+          <t>flashscore:lecce</t>
         </is>
       </c>
       <c r="S12" t="inlineStr">
@@ -4418,7 +4418,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-05-18 01:55:05 ACST</t>
+          <t>2026-05-18 04:02:28 ACST</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -4453,7 +4453,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>flashscore:nmmS8WHr</t>
+          <t>flashscore:h0IS6Ane</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
@@ -4483,12 +4483,12 @@
       </c>
       <c r="N13" t="inlineStr">
         <is>
-          <t>Sassuolo</t>
+          <t>Udinese</t>
         </is>
       </c>
       <c r="O13" t="inlineStr">
         <is>
-          <t>flashscore:sassuolo</t>
+          <t>flashscore:udinese</t>
         </is>
       </c>
       <c r="P13" t="inlineStr">
@@ -4498,12 +4498,12 @@
       </c>
       <c r="Q13" t="inlineStr">
         <is>
-          <t>Lecce</t>
+          <t>Cremonese</t>
         </is>
       </c>
       <c r="R13" t="inlineStr">
         <is>
-          <t>flashscore:lecce</t>
+          <t>flashscore:cremonese</t>
         </is>
       </c>
       <c r="S13" t="inlineStr">
@@ -4540,7 +4540,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-05-18 01:55:05 ACST</t>
+          <t>2026-05-18 04:02:28 ACST</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -4555,7 +4555,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>34</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -4565,7 +4565,7 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Serie A</t>
+          <t>Ligue 1</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -4575,7 +4575,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>flashscore:h0IS6Ane</t>
+          <t>flashscore:prPnPy9r</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
@@ -4585,7 +4585,7 @@
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>04:15</t>
+          <t>04:30</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
@@ -4595,7 +4595,7 @@
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>1779043500</t>
+          <t>1779044400</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
@@ -4605,12 +4605,12 @@
       </c>
       <c r="N14" t="inlineStr">
         <is>
-          <t>Udinese</t>
+          <t>Brest</t>
         </is>
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>flashscore:udinese</t>
+          <t>flashscore:brest</t>
         </is>
       </c>
       <c r="P14" t="inlineStr">
@@ -4620,12 +4620,12 @@
       </c>
       <c r="Q14" t="inlineStr">
         <is>
-          <t>Cremonese</t>
+          <t>Angers</t>
         </is>
       </c>
       <c r="R14" t="inlineStr">
         <is>
-          <t>flashscore:cremonese</t>
+          <t>flashscore:angers</t>
         </is>
       </c>
       <c r="S14" t="inlineStr">
@@ -4662,7 +4662,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-05-18 01:55:05 ACST</t>
+          <t>2026-05-18 04:02:28 ACST</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -4697,7 +4697,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>flashscore:prPnPy9r</t>
+          <t>flashscore:IXv8WJG8</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
@@ -4727,12 +4727,12 @@
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>Brest</t>
+          <t>Lille</t>
         </is>
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>flashscore:brest</t>
+          <t>flashscore:lille</t>
         </is>
       </c>
       <c r="P15" t="inlineStr">
@@ -4742,12 +4742,12 @@
       </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t>Angers</t>
+          <t>Auxerre</t>
         </is>
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>flashscore:angers</t>
+          <t>flashscore:auxerre</t>
         </is>
       </c>
       <c r="S15" t="inlineStr">
@@ -4784,7 +4784,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-05-18 01:55:05 ACST</t>
+          <t>2026-05-18 04:02:28 ACST</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -4819,7 +4819,7 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>flashscore:IXv8WJG8</t>
+          <t>flashscore:r1cGQTSk</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
@@ -4849,12 +4849,12 @@
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>Lille</t>
+          <t>Lorient</t>
         </is>
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>flashscore:lille</t>
+          <t>flashscore:lorient</t>
         </is>
       </c>
       <c r="P16" t="inlineStr">
@@ -4864,12 +4864,12 @@
       </c>
       <c r="Q16" t="inlineStr">
         <is>
-          <t>Auxerre</t>
+          <t>Le Havre</t>
         </is>
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>flashscore:auxerre</t>
+          <t>flashscore:lehavre</t>
         </is>
       </c>
       <c r="S16" t="inlineStr">
@@ -4906,7 +4906,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-05-18 01:55:05 ACST</t>
+          <t>2026-05-18 04:02:28 ACST</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -4941,7 +4941,7 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>flashscore:r1cGQTSk</t>
+          <t>flashscore:OhrGQlpm</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
@@ -4971,12 +4971,12 @@
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>Lorient</t>
+          <t>Lyon</t>
         </is>
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>flashscore:lorient</t>
+          <t>flashscore:lyon</t>
         </is>
       </c>
       <c r="P17" t="inlineStr">
@@ -4986,12 +4986,12 @@
       </c>
       <c r="Q17" t="inlineStr">
         <is>
-          <t>Le Havre</t>
+          <t>Lens</t>
         </is>
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>flashscore:lehavre</t>
+          <t>flashscore:lens</t>
         </is>
       </c>
       <c r="S17" t="inlineStr">
@@ -5028,7 +5028,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-05-18 01:55:05 ACST</t>
+          <t>2026-05-18 04:02:28 ACST</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -5063,7 +5063,7 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>flashscore:OhrGQlpm</t>
+          <t>flashscore:xbwdLg87</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
@@ -5093,12 +5093,12 @@
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>Lyon</t>
+          <t>Marseille</t>
         </is>
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>flashscore:lyon</t>
+          <t>flashscore:marseille</t>
         </is>
       </c>
       <c r="P18" t="inlineStr">
@@ -5108,12 +5108,12 @@
       </c>
       <c r="Q18" t="inlineStr">
         <is>
-          <t>Lens</t>
+          <t>Rennes</t>
         </is>
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>flashscore:lens</t>
+          <t>flashscore:rennes</t>
         </is>
       </c>
       <c r="S18" t="inlineStr">
@@ -5150,7 +5150,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-05-18 01:55:05 ACST</t>
+          <t>2026-05-18 04:02:28 ACST</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -5185,7 +5185,7 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>flashscore:xbwdLg87</t>
+          <t>flashscore:z9FNO7c2</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
@@ -5215,12 +5215,12 @@
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>Marseille</t>
+          <t>Nantes</t>
         </is>
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>flashscore:marseille</t>
+          <t>flashscore:nantes</t>
         </is>
       </c>
       <c r="P19" t="inlineStr">
@@ -5230,12 +5230,12 @@
       </c>
       <c r="Q19" t="inlineStr">
         <is>
-          <t>Rennes</t>
+          <t>Toulouse</t>
         </is>
       </c>
       <c r="R19" t="inlineStr">
         <is>
-          <t>flashscore:rennes</t>
+          <t>flashscore:toulouse</t>
         </is>
       </c>
       <c r="S19" t="inlineStr">
@@ -5272,7 +5272,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-05-18 01:55:05 ACST</t>
+          <t>2026-05-18 04:02:28 ACST</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -5307,7 +5307,7 @@
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>flashscore:z9FNO7c2</t>
+          <t>flashscore:QcrGUcoL</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
@@ -5337,12 +5337,12 @@
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>Nantes</t>
+          <t>Nice</t>
         </is>
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>flashscore:nantes</t>
+          <t>flashscore:nice</t>
         </is>
       </c>
       <c r="P20" t="inlineStr">
@@ -5352,12 +5352,12 @@
       </c>
       <c r="Q20" t="inlineStr">
         <is>
-          <t>Toulouse</t>
+          <t>Metz</t>
         </is>
       </c>
       <c r="R20" t="inlineStr">
         <is>
-          <t>flashscore:toulouse</t>
+          <t>flashscore:metz</t>
         </is>
       </c>
       <c r="S20" t="inlineStr">
@@ -5394,7 +5394,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-05-18 01:55:05 ACST</t>
+          <t>2026-05-18 04:02:28 ACST</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -5429,7 +5429,7 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>flashscore:QcrGUcoL</t>
+          <t>flashscore:IeNfNFwe</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
@@ -5459,12 +5459,12 @@
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>Nice</t>
+          <t>Paris FC</t>
         </is>
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>flashscore:nice</t>
+          <t>flashscore:parisfc</t>
         </is>
       </c>
       <c r="P21" t="inlineStr">
@@ -5474,12 +5474,12 @@
       </c>
       <c r="Q21" t="inlineStr">
         <is>
-          <t>Metz</t>
+          <t>PSG</t>
         </is>
       </c>
       <c r="R21" t="inlineStr">
         <is>
-          <t>flashscore:metz</t>
+          <t>flashscore:psg</t>
         </is>
       </c>
       <c r="S21" t="inlineStr">
@@ -5516,7 +5516,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-05-18 01:55:05 ACST</t>
+          <t>2026-05-18 04:02:28 ACST</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -5551,7 +5551,7 @@
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>flashscore:IeNfNFwe</t>
+          <t>flashscore:44Vsqc0E</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
@@ -5581,12 +5581,12 @@
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>Paris FC</t>
+          <t>Strasbourg</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>flashscore:parisfc</t>
+          <t>flashscore:strasbourg</t>
         </is>
       </c>
       <c r="P22" t="inlineStr">
@@ -5596,12 +5596,12 @@
       </c>
       <c r="Q22" t="inlineStr">
         <is>
-          <t>PSG</t>
+          <t>Monaco</t>
         </is>
       </c>
       <c r="R22" t="inlineStr">
         <is>
-          <t>flashscore:psg</t>
+          <t>flashscore:monaco</t>
         </is>
       </c>
       <c r="S22" t="inlineStr">
@@ -5638,7 +5638,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-05-18 01:55:05 ACST</t>
+          <t>2026-05-18 04:02:28 ACST</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -5653,7 +5653,7 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>34</t>
+          <t>8</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -5663,7 +5663,7 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Ligue 1</t>
+          <t>LaLiga</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -5673,7 +5673,7 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>flashscore:44Vsqc0E</t>
+          <t>flashscore:SduXBE3E</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
@@ -5683,7 +5683,7 @@
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>04:30</t>
+          <t>04:45</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
@@ -5693,7 +5693,7 @@
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>1779044400</t>
+          <t>1779045300</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
@@ -5703,12 +5703,12 @@
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>Strasbourg</t>
+          <t>Barcelona</t>
         </is>
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>flashscore:strasbourg</t>
+          <t>flashscore:barcelona</t>
         </is>
       </c>
       <c r="P23" t="inlineStr">
@@ -5718,12 +5718,12 @@
       </c>
       <c r="Q23" t="inlineStr">
         <is>
-          <t>Monaco</t>
+          <t>Betis</t>
         </is>
       </c>
       <c r="R23" t="inlineStr">
         <is>
-          <t>flashscore:monaco</t>
+          <t>flashscore:betis</t>
         </is>
       </c>
       <c r="S23" t="inlineStr">
@@ -5760,7 +5760,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2026-05-18 01:55:05 ACST</t>
+          <t>2026-05-18 04:02:28 ACST</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -5775,7 +5775,7 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>23</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -5785,7 +5785,7 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>LaLiga</t>
+          <t>Serie A</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -5795,7 +5795,7 @@
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>flashscore:SduXBE3E</t>
+          <t>flashscore:I9QHhKRp</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
@@ -5805,7 +5805,7 @@
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>04:45</t>
+          <t>FT</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
@@ -5815,22 +5815,22 @@
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>1779045300</t>
+          <t>1779033600</t>
         </is>
       </c>
       <c r="M24" t="inlineStr">
         <is>
-          <t>live</t>
+          <t>FT</t>
         </is>
       </c>
       <c r="N24" t="inlineStr">
         <is>
-          <t>Barcelona</t>
+          <t>Atalanta</t>
         </is>
       </c>
       <c r="O24" t="inlineStr">
         <is>
-          <t>flashscore:barcelona</t>
+          <t>flashscore:atalanta</t>
         </is>
       </c>
       <c r="P24" t="inlineStr">
@@ -5840,12 +5840,12 @@
       </c>
       <c r="Q24" t="inlineStr">
         <is>
-          <t>Betis</t>
+          <t>Bologna</t>
         </is>
       </c>
       <c r="R24" t="inlineStr">
         <is>
-          <t>flashscore:betis</t>
+          <t>flashscore:bologna</t>
         </is>
       </c>
       <c r="S24" t="inlineStr">
@@ -6423,12 +6423,12 @@
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
     </row>
@@ -6484,7 +6484,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-05-18 01:55:05 ACST</t>
+          <t>2026-05-18 04:02:28 ACST</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -6494,7 +6494,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>https://2.flashscore.ninja/2/x/feed/f_1_0_3_en-uk_1</t>
+          <t>https://www.flashscore.com.au/x/feed/f_1_0_3_en-au_1</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -6519,7 +6519,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>events=1192 league_hit=63 skipped_women=3 out_of_window=37 matched=23 by_league={'Ligue 1': 9, 'Serie A': 4, 'LaLiga': 10} sample_leagues=['Africa|AFRICA: CAF Champions League - Play Offs', 'Africa|AFRICA: Africa Cup of Nations U17', 'Albania|ALBANIA: Abissnet Superiore - Final Group', 'Andorra|ANDORRA: Primera Divisió', 'Angola|ANGOLA: Girabola', 'Argentina|ARGENTINA: Liga Profesional - Apertura - Play Offs', 'Argentina|ARGENTINA: Primera Nacional', 'Argentina|ARGENTINA: Torneo Federal']</t>
+          <t>events=1195 league_hit=57 skipped_women=1 out_of_window=33 matched=23 by_league={'Ligue 1': 9, 'Serie A': 4, 'LaLiga': 10} sample_leagues=['Africa|AFRICA: CAF Champions League - Play Offs', 'Africa|AFRICA: Africa Cup of Nations U17', 'Albania|ALBANIA: Abissnet Superiore - Final Group', 'Andorra|ANDORRA: Primera Divisió', 'Angola|ANGOLA: Girabola', 'Argentina|ARGENTINA: Liga Profesional - Apertura - Play Offs', 'Argentina|ARGENTINA: Primera Nacional', 'Argentina|ARGENTINA: Torneo Federal']</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Refresh match data and pipeline outputs
Manual data:refresh run on 2026-05-17: 470 matches, 379 FT, 91 upcoming. Includes Phase1-7 outputs, model calibration, and updated match_data.json for the next Firestore upload.

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/agent-system/outputs/Phase1_Fixture_Slate.xlsx
+++ b/docs/agent-system/outputs/Phase1_Fixture_Slate.xlsx
@@ -141,7 +141,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-05-18 04:02:28 ACST</t>
+          <t>2026-05-18 05:54:08 ACST</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -156,7 +156,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>23</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -166,7 +166,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>LaLiga</t>
+          <t>Serie A</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -176,7 +176,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>flashscore:vyaxjXte</t>
+          <t>flashscore:YH84GNJi</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -186,7 +186,7 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>02:30</t>
+          <t>04:15</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
@@ -196,7 +196,7 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>1779037200</t>
+          <t>1779043500</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
@@ -206,12 +206,12 @@
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>Ath. Bilbao</t>
+          <t>Cagliari</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>flashscore:athbilbao</t>
+          <t>flashscore:cagliari</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
@@ -221,12 +221,12 @@
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>Celta Vigo</t>
+          <t>Torino</t>
         </is>
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>flashscore:celtavigo</t>
+          <t>flashscore:torino</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
@@ -263,7 +263,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-05-18 04:02:28 ACST</t>
+          <t>2026-05-18 05:54:08 ACST</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -278,7 +278,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>23</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -288,7 +288,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>LaLiga</t>
+          <t>Serie A</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -298,7 +298,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>flashscore:n12plBB7</t>
+          <t>flashscore:nmmS8WHr</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -308,7 +308,7 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>02:30</t>
+          <t>04:15</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
@@ -318,7 +318,7 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>1779037200</t>
+          <t>1779043500</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
@@ -328,12 +328,12 @@
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>Atl. Madrid</t>
+          <t>Sassuolo</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>flashscore:atlmadrid</t>
+          <t>flashscore:sassuolo</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
@@ -343,12 +343,12 @@
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>Girona</t>
+          <t>Lecce</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>flashscore:girona</t>
+          <t>flashscore:lecce</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
@@ -385,7 +385,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-05-18 04:02:28 ACST</t>
+          <t>2026-05-18 05:54:08 ACST</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -400,7 +400,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>23</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -410,7 +410,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>LaLiga</t>
+          <t>Serie A</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -420,7 +420,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>flashscore:0OhvAhYQ</t>
+          <t>flashscore:h0IS6Ane</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -430,7 +430,7 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>02:30</t>
+          <t>04:15</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
@@ -440,7 +440,7 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>1779037200</t>
+          <t>1779043500</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
@@ -450,12 +450,12 @@
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>Elche</t>
+          <t>Udinese</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>flashscore:elche</t>
+          <t>flashscore:udinese</t>
         </is>
       </c>
       <c r="P4" t="inlineStr">
@@ -465,12 +465,12 @@
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>Getafe</t>
+          <t>Cremonese</t>
         </is>
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>flashscore:getafe</t>
+          <t>flashscore:cremonese</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
@@ -507,7 +507,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-05-18 04:02:28 ACST</t>
+          <t>2026-05-18 05:54:08 ACST</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -522,7 +522,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>34</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -532,7 +532,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>LaLiga</t>
+          <t>Ligue 1</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -542,7 +542,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>flashscore:K8ZA4Wel</t>
+          <t>flashscore:prPnPy9r</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
@@ -552,7 +552,7 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>02:30</t>
+          <t>04:30</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
@@ -562,7 +562,7 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>1779037200</t>
+          <t>1779044400</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
@@ -572,12 +572,12 @@
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>Levante</t>
+          <t>Brest</t>
         </is>
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>flashscore:levante</t>
+          <t>flashscore:brest</t>
         </is>
       </c>
       <c r="P5" t="inlineStr">
@@ -587,12 +587,12 @@
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>Mallorca</t>
+          <t>Angers</t>
         </is>
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>flashscore:mallorca</t>
+          <t>flashscore:angers</t>
         </is>
       </c>
       <c r="S5" t="inlineStr">
@@ -629,7 +629,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-05-18 04:02:28 ACST</t>
+          <t>2026-05-18 05:54:08 ACST</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -644,7 +644,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>34</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -654,7 +654,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>LaLiga</t>
+          <t>Ligue 1</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -664,7 +664,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>flashscore:YFVo6qXh</t>
+          <t>flashscore:IXv8WJG8</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
@@ -674,7 +674,7 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>02:30</t>
+          <t>04:30</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
@@ -684,7 +684,7 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>1779037200</t>
+          <t>1779044400</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
@@ -694,12 +694,12 @@
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>Osasuna</t>
+          <t>Lille</t>
         </is>
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>flashscore:osasuna</t>
+          <t>flashscore:lille</t>
         </is>
       </c>
       <c r="P6" t="inlineStr">
@@ -709,12 +709,12 @@
       </c>
       <c r="Q6" t="inlineStr">
         <is>
-          <t>Espanyol</t>
+          <t>Auxerre</t>
         </is>
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>flashscore:espanyol</t>
+          <t>flashscore:auxerre</t>
         </is>
       </c>
       <c r="S6" t="inlineStr">
@@ -751,7 +751,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-05-18 04:02:28 ACST</t>
+          <t>2026-05-18 05:54:08 ACST</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -766,7 +766,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>34</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -776,7 +776,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>LaLiga</t>
+          <t>Ligue 1</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -786,7 +786,7 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>flashscore:C0sw852t</t>
+          <t>flashscore:r1cGQTSk</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
@@ -796,7 +796,7 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>02:30</t>
+          <t>04:30</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
@@ -806,7 +806,7 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>1779037200</t>
+          <t>1779044400</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
@@ -816,12 +816,12 @@
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>Oviedo</t>
+          <t>Lorient</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>flashscore:oviedo</t>
+          <t>flashscore:lorient</t>
         </is>
       </c>
       <c r="P7" t="inlineStr">
@@ -831,12 +831,12 @@
       </c>
       <c r="Q7" t="inlineStr">
         <is>
-          <t>Alaves</t>
+          <t>Le Havre</t>
         </is>
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>flashscore:alaves</t>
+          <t>flashscore:lehavre</t>
         </is>
       </c>
       <c r="S7" t="inlineStr">
@@ -873,7 +873,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-05-18 04:02:28 ACST</t>
+          <t>2026-05-18 05:54:08 ACST</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -888,7 +888,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>34</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -898,7 +898,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>LaLiga</t>
+          <t>Ligue 1</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -908,7 +908,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>flashscore:llRR0leD</t>
+          <t>flashscore:OhrGQlpm</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
@@ -918,7 +918,7 @@
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>02:30</t>
+          <t>04:30</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
@@ -928,7 +928,7 @@
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>1779037200</t>
+          <t>1779044400</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
@@ -938,12 +938,12 @@
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>Real Sociedad</t>
+          <t>Lyon</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>flashscore:realsociedad</t>
+          <t>flashscore:lyon</t>
         </is>
       </c>
       <c r="P8" t="inlineStr">
@@ -953,12 +953,12 @@
       </c>
       <c r="Q8" t="inlineStr">
         <is>
-          <t>Valencia</t>
+          <t>Lens</t>
         </is>
       </c>
       <c r="R8" t="inlineStr">
         <is>
-          <t>flashscore:valencia</t>
+          <t>flashscore:lens</t>
         </is>
       </c>
       <c r="S8" t="inlineStr">
@@ -995,7 +995,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-05-18 04:02:28 ACST</t>
+          <t>2026-05-18 05:54:08 ACST</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -1010,7 +1010,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>34</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -1020,7 +1020,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>LaLiga</t>
+          <t>Ligue 1</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -1030,7 +1030,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>flashscore:ttZg4N15</t>
+          <t>flashscore:xbwdLg87</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
@@ -1040,7 +1040,7 @@
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>02:30</t>
+          <t>04:30</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
@@ -1050,7 +1050,7 @@
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>1779037200</t>
+          <t>1779044400</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
@@ -1060,12 +1060,12 @@
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>Sevilla</t>
+          <t>Marseille</t>
         </is>
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>flashscore:sevilla</t>
+          <t>flashscore:marseille</t>
         </is>
       </c>
       <c r="P9" t="inlineStr">
@@ -1075,12 +1075,12 @@
       </c>
       <c r="Q9" t="inlineStr">
         <is>
-          <t>Real Madrid</t>
+          <t>Rennes</t>
         </is>
       </c>
       <c r="R9" t="inlineStr">
         <is>
-          <t>flashscore:realmadrid</t>
+          <t>flashscore:rennes</t>
         </is>
       </c>
       <c r="S9" t="inlineStr">
@@ -1117,7 +1117,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-05-18 04:02:28 ACST</t>
+          <t>2026-05-18 05:54:08 ACST</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -1132,7 +1132,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>34</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -1142,7 +1142,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>LaLiga</t>
+          <t>Ligue 1</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -1152,7 +1152,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>flashscore:hMXI2AQ0</t>
+          <t>flashscore:QcrGUcoL</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
@@ -1162,7 +1162,7 @@
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>02:30</t>
+          <t>04:30</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
@@ -1172,7 +1172,7 @@
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>1779037200</t>
+          <t>1779044400</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
@@ -1182,12 +1182,12 @@
       </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>Vallecano</t>
+          <t>Nice</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>flashscore:vallecano</t>
+          <t>flashscore:nice</t>
         </is>
       </c>
       <c r="P10" t="inlineStr">
@@ -1197,12 +1197,12 @@
       </c>
       <c r="Q10" t="inlineStr">
         <is>
-          <t>Villarreal</t>
+          <t>Metz</t>
         </is>
       </c>
       <c r="R10" t="inlineStr">
         <is>
-          <t>flashscore:villarreal</t>
+          <t>flashscore:metz</t>
         </is>
       </c>
       <c r="S10" t="inlineStr">
@@ -1239,7 +1239,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-05-18 04:02:28 ACST</t>
+          <t>2026-05-18 05:54:08 ACST</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -1254,7 +1254,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>34</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -1264,7 +1264,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Serie A</t>
+          <t>Ligue 1</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -1274,7 +1274,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>flashscore:YH84GNJi</t>
+          <t>flashscore:IeNfNFwe</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
@@ -1284,7 +1284,7 @@
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>04:15</t>
+          <t>04:30</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
@@ -1294,7 +1294,7 @@
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>1779043500</t>
+          <t>1779044400</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
@@ -1304,12 +1304,12 @@
       </c>
       <c r="N11" t="inlineStr">
         <is>
-          <t>Cagliari</t>
+          <t>Paris FC</t>
         </is>
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>flashscore:cagliari</t>
+          <t>flashscore:parisfc</t>
         </is>
       </c>
       <c r="P11" t="inlineStr">
@@ -1319,12 +1319,12 @@
       </c>
       <c r="Q11" t="inlineStr">
         <is>
-          <t>Torino</t>
+          <t>PSG</t>
         </is>
       </c>
       <c r="R11" t="inlineStr">
         <is>
-          <t>flashscore:torino</t>
+          <t>flashscore:psg</t>
         </is>
       </c>
       <c r="S11" t="inlineStr">
@@ -1361,7 +1361,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-05-18 04:02:28 ACST</t>
+          <t>2026-05-18 05:54:08 ACST</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -1376,7 +1376,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>34</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -1386,7 +1386,7 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Serie A</t>
+          <t>Ligue 1</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -1396,7 +1396,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>flashscore:nmmS8WHr</t>
+          <t>flashscore:44Vsqc0E</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
@@ -1406,7 +1406,7 @@
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>04:15</t>
+          <t>04:30</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
@@ -1416,7 +1416,7 @@
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>1779043500</t>
+          <t>1779044400</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
@@ -1426,12 +1426,12 @@
       </c>
       <c r="N12" t="inlineStr">
         <is>
-          <t>Sassuolo</t>
+          <t>Strasbourg</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>flashscore:sassuolo</t>
+          <t>flashscore:strasbourg</t>
         </is>
       </c>
       <c r="P12" t="inlineStr">
@@ -1441,12 +1441,12 @@
       </c>
       <c r="Q12" t="inlineStr">
         <is>
-          <t>Lecce</t>
+          <t>Monaco</t>
         </is>
       </c>
       <c r="R12" t="inlineStr">
         <is>
-          <t>flashscore:lecce</t>
+          <t>flashscore:monaco</t>
         </is>
       </c>
       <c r="S12" t="inlineStr">
@@ -1483,7 +1483,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-05-18 04:02:28 ACST</t>
+          <t>2026-05-18 05:54:08 ACST</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1498,7 +1498,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>8</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -1508,7 +1508,7 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Serie A</t>
+          <t>LaLiga</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -1518,7 +1518,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>flashscore:h0IS6Ane</t>
+          <t>flashscore:SduXBE3E</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
@@ -1528,7 +1528,7 @@
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>04:15</t>
+          <t>04:45</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
@@ -1538,7 +1538,7 @@
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>1779043500</t>
+          <t>1779045300</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
@@ -1548,12 +1548,12 @@
       </c>
       <c r="N13" t="inlineStr">
         <is>
-          <t>Udinese</t>
+          <t>Barcelona</t>
         </is>
       </c>
       <c r="O13" t="inlineStr">
         <is>
-          <t>flashscore:udinese</t>
+          <t>flashscore:barcelona</t>
         </is>
       </c>
       <c r="P13" t="inlineStr">
@@ -1563,12 +1563,12 @@
       </c>
       <c r="Q13" t="inlineStr">
         <is>
-          <t>Cremonese</t>
+          <t>Betis</t>
         </is>
       </c>
       <c r="R13" t="inlineStr">
         <is>
-          <t>flashscore:cremonese</t>
+          <t>flashscore:betis</t>
         </is>
       </c>
       <c r="S13" t="inlineStr">
@@ -1605,7 +1605,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-05-18 04:02:28 ACST</t>
+          <t>2026-05-18 05:54:08 ACST</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -1620,7 +1620,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>34</t>
+          <t>8</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -1630,7 +1630,7 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Ligue 1</t>
+          <t>LaLiga</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -1640,7 +1640,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>flashscore:prPnPy9r</t>
+          <t>flashscore:vyaxjXte</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
@@ -1650,7 +1650,7 @@
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>04:30</t>
+          <t>FT</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
@@ -1660,22 +1660,22 @@
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>1779044400</t>
+          <t>1779037200</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>live</t>
+          <t>FT</t>
         </is>
       </c>
       <c r="N14" t="inlineStr">
         <is>
-          <t>Brest</t>
+          <t>Ath. Bilbao</t>
         </is>
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>flashscore:brest</t>
+          <t>flashscore:athbilbao</t>
         </is>
       </c>
       <c r="P14" t="inlineStr">
@@ -1685,12 +1685,12 @@
       </c>
       <c r="Q14" t="inlineStr">
         <is>
-          <t>Angers</t>
+          <t>Celta Vigo</t>
         </is>
       </c>
       <c r="R14" t="inlineStr">
         <is>
-          <t>flashscore:angers</t>
+          <t>flashscore:celtavigo</t>
         </is>
       </c>
       <c r="S14" t="inlineStr">
@@ -1727,7 +1727,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-05-18 04:02:28 ACST</t>
+          <t>2026-05-18 05:54:08 ACST</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1742,7 +1742,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>34</t>
+          <t>8</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -1752,7 +1752,7 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Ligue 1</t>
+          <t>LaLiga</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -1762,7 +1762,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>flashscore:IXv8WJG8</t>
+          <t>flashscore:n12plBB7</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
@@ -1772,7 +1772,7 @@
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>04:30</t>
+          <t>FT</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
@@ -1782,22 +1782,22 @@
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>1779044400</t>
+          <t>1779037200</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>live</t>
+          <t>FT</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>Lille</t>
+          <t>Atl. Madrid</t>
         </is>
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>flashscore:lille</t>
+          <t>flashscore:atlmadrid</t>
         </is>
       </c>
       <c r="P15" t="inlineStr">
@@ -1807,12 +1807,12 @@
       </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t>Auxerre</t>
+          <t>Girona</t>
         </is>
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>flashscore:auxerre</t>
+          <t>flashscore:girona</t>
         </is>
       </c>
       <c r="S15" t="inlineStr">
@@ -1849,7 +1849,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-05-18 04:02:28 ACST</t>
+          <t>2026-05-18 05:54:08 ACST</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -1864,7 +1864,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>34</t>
+          <t>8</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -1874,7 +1874,7 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Ligue 1</t>
+          <t>LaLiga</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -1884,7 +1884,7 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>flashscore:r1cGQTSk</t>
+          <t>flashscore:0OhvAhYQ</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
@@ -1894,7 +1894,7 @@
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>04:30</t>
+          <t>FT</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
@@ -1904,22 +1904,22 @@
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>1779044400</t>
+          <t>1779037200</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>live</t>
+          <t>FT</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>Lorient</t>
+          <t>Elche</t>
         </is>
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>flashscore:lorient</t>
+          <t>flashscore:elche</t>
         </is>
       </c>
       <c r="P16" t="inlineStr">
@@ -1929,12 +1929,12 @@
       </c>
       <c r="Q16" t="inlineStr">
         <is>
-          <t>Le Havre</t>
+          <t>Getafe</t>
         </is>
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>flashscore:lehavre</t>
+          <t>flashscore:getafe</t>
         </is>
       </c>
       <c r="S16" t="inlineStr">
@@ -1971,7 +1971,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-05-18 04:02:28 ACST</t>
+          <t>2026-05-18 05:54:08 ACST</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -1986,7 +1986,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>34</t>
+          <t>8</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -1996,7 +1996,7 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Ligue 1</t>
+          <t>LaLiga</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -2006,7 +2006,7 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>flashscore:OhrGQlpm</t>
+          <t>flashscore:K8ZA4Wel</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
@@ -2016,7 +2016,7 @@
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>04:30</t>
+          <t>FT</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
@@ -2026,22 +2026,22 @@
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>1779044400</t>
+          <t>1779037200</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>live</t>
+          <t>FT</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>Lyon</t>
+          <t>Levante</t>
         </is>
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>flashscore:lyon</t>
+          <t>flashscore:levante</t>
         </is>
       </c>
       <c r="P17" t="inlineStr">
@@ -2051,12 +2051,12 @@
       </c>
       <c r="Q17" t="inlineStr">
         <is>
-          <t>Lens</t>
+          <t>Mallorca</t>
         </is>
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>flashscore:lens</t>
+          <t>flashscore:mallorca</t>
         </is>
       </c>
       <c r="S17" t="inlineStr">
@@ -2093,7 +2093,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-05-18 04:02:28 ACST</t>
+          <t>2026-05-18 05:54:08 ACST</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -2108,7 +2108,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>34</t>
+          <t>8</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -2118,7 +2118,7 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Ligue 1</t>
+          <t>LaLiga</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -2128,7 +2128,7 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>flashscore:xbwdLg87</t>
+          <t>flashscore:YFVo6qXh</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
@@ -2138,7 +2138,7 @@
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>04:30</t>
+          <t>FT</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
@@ -2148,22 +2148,22 @@
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>1779044400</t>
+          <t>1779037200</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>live</t>
+          <t>FT</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>Marseille</t>
+          <t>Osasuna</t>
         </is>
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>flashscore:marseille</t>
+          <t>flashscore:osasuna</t>
         </is>
       </c>
       <c r="P18" t="inlineStr">
@@ -2173,12 +2173,12 @@
       </c>
       <c r="Q18" t="inlineStr">
         <is>
-          <t>Rennes</t>
+          <t>Espanyol</t>
         </is>
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>flashscore:rennes</t>
+          <t>flashscore:espanyol</t>
         </is>
       </c>
       <c r="S18" t="inlineStr">
@@ -2215,7 +2215,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-05-18 04:02:28 ACST</t>
+          <t>2026-05-18 05:54:08 ACST</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -2230,7 +2230,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>34</t>
+          <t>8</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -2240,7 +2240,7 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Ligue 1</t>
+          <t>LaLiga</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -2250,7 +2250,7 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>flashscore:z9FNO7c2</t>
+          <t>flashscore:C0sw852t</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
@@ -2260,7 +2260,7 @@
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>04:30</t>
+          <t>FT</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
@@ -2270,22 +2270,22 @@
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>1779044400</t>
+          <t>1779037200</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>live</t>
+          <t>FT</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>Nantes</t>
+          <t>Oviedo</t>
         </is>
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>flashscore:nantes</t>
+          <t>flashscore:oviedo</t>
         </is>
       </c>
       <c r="P19" t="inlineStr">
@@ -2295,12 +2295,12 @@
       </c>
       <c r="Q19" t="inlineStr">
         <is>
-          <t>Toulouse</t>
+          <t>Alaves</t>
         </is>
       </c>
       <c r="R19" t="inlineStr">
         <is>
-          <t>flashscore:toulouse</t>
+          <t>flashscore:alaves</t>
         </is>
       </c>
       <c r="S19" t="inlineStr">
@@ -2337,7 +2337,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-05-18 04:02:28 ACST</t>
+          <t>2026-05-18 05:54:08 ACST</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -2352,7 +2352,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>34</t>
+          <t>8</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -2362,7 +2362,7 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Ligue 1</t>
+          <t>LaLiga</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -2372,7 +2372,7 @@
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>flashscore:QcrGUcoL</t>
+          <t>flashscore:llRR0leD</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
@@ -2382,7 +2382,7 @@
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>04:30</t>
+          <t>FT</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
@@ -2392,22 +2392,22 @@
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>1779044400</t>
+          <t>1779037200</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>live</t>
+          <t>FT</t>
         </is>
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>Nice</t>
+          <t>Real Sociedad</t>
         </is>
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>flashscore:nice</t>
+          <t>flashscore:realsociedad</t>
         </is>
       </c>
       <c r="P20" t="inlineStr">
@@ -2417,12 +2417,12 @@
       </c>
       <c r="Q20" t="inlineStr">
         <is>
-          <t>Metz</t>
+          <t>Valencia</t>
         </is>
       </c>
       <c r="R20" t="inlineStr">
         <is>
-          <t>flashscore:metz</t>
+          <t>flashscore:valencia</t>
         </is>
       </c>
       <c r="S20" t="inlineStr">
@@ -2459,7 +2459,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-05-18 04:02:28 ACST</t>
+          <t>2026-05-18 05:54:08 ACST</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -2474,7 +2474,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>34</t>
+          <t>8</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -2484,7 +2484,7 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Ligue 1</t>
+          <t>LaLiga</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -2494,7 +2494,7 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>flashscore:IeNfNFwe</t>
+          <t>flashscore:ttZg4N15</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
@@ -2504,7 +2504,7 @@
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>04:30</t>
+          <t>FT</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
@@ -2514,22 +2514,22 @@
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>1779044400</t>
+          <t>1779037200</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>live</t>
+          <t>FT</t>
         </is>
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>Paris FC</t>
+          <t>Sevilla</t>
         </is>
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>flashscore:parisfc</t>
+          <t>flashscore:sevilla</t>
         </is>
       </c>
       <c r="P21" t="inlineStr">
@@ -2539,12 +2539,12 @@
       </c>
       <c r="Q21" t="inlineStr">
         <is>
-          <t>PSG</t>
+          <t>Real Madrid</t>
         </is>
       </c>
       <c r="R21" t="inlineStr">
         <is>
-          <t>flashscore:psg</t>
+          <t>flashscore:realmadrid</t>
         </is>
       </c>
       <c r="S21" t="inlineStr">
@@ -2581,7 +2581,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-05-18 04:02:28 ACST</t>
+          <t>2026-05-18 05:54:08 ACST</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -2596,7 +2596,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>34</t>
+          <t>8</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -2606,7 +2606,7 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Ligue 1</t>
+          <t>LaLiga</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -2616,7 +2616,7 @@
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>flashscore:44Vsqc0E</t>
+          <t>flashscore:hMXI2AQ0</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
@@ -2626,7 +2626,7 @@
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>04:30</t>
+          <t>FT</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
@@ -2636,22 +2636,22 @@
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>1779044400</t>
+          <t>1779037200</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>live</t>
+          <t>FT</t>
         </is>
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>Strasbourg</t>
+          <t>Vallecano</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>flashscore:strasbourg</t>
+          <t>flashscore:vallecano</t>
         </is>
       </c>
       <c r="P22" t="inlineStr">
@@ -2661,12 +2661,12 @@
       </c>
       <c r="Q22" t="inlineStr">
         <is>
-          <t>Monaco</t>
+          <t>Villarreal</t>
         </is>
       </c>
       <c r="R22" t="inlineStr">
         <is>
-          <t>flashscore:monaco</t>
+          <t>flashscore:villarreal</t>
         </is>
       </c>
       <c r="S22" t="inlineStr">
@@ -2703,7 +2703,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-05-18 04:02:28 ACST</t>
+          <t>2026-05-18 05:54:08 ACST</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -2718,7 +2718,7 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>34</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -2728,7 +2728,7 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>LaLiga</t>
+          <t>Ligue 1</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -2738,7 +2738,7 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>flashscore:SduXBE3E</t>
+          <t>flashscore:z9FNO7c2</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
@@ -2748,7 +2748,7 @@
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>04:45</t>
+          <t>FT</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
@@ -2758,22 +2758,22 @@
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>1779045300</t>
+          <t>1779044400</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>live</t>
+          <t>FT</t>
         </is>
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>Barcelona</t>
+          <t>Nantes</t>
         </is>
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>flashscore:barcelona</t>
+          <t>flashscore:nantes</t>
         </is>
       </c>
       <c r="P23" t="inlineStr">
@@ -2783,12 +2783,12 @@
       </c>
       <c r="Q23" t="inlineStr">
         <is>
-          <t>Betis</t>
+          <t>Toulouse</t>
         </is>
       </c>
       <c r="R23" t="inlineStr">
         <is>
-          <t>flashscore:betis</t>
+          <t>flashscore:toulouse</t>
         </is>
       </c>
       <c r="S23" t="inlineStr">
@@ -2825,7 +2825,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2026-05-18 04:02:28 ACST</t>
+          <t>2026-05-18 05:54:08 ACST</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -3076,7 +3076,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-05-18 04:02:28 ACST</t>
+          <t>2026-05-18 05:54:08 ACST</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -3091,7 +3091,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>23</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -3101,7 +3101,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>LaLiga</t>
+          <t>Serie A</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -3111,7 +3111,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>flashscore:vyaxjXte</t>
+          <t>flashscore:YH84GNJi</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -3121,7 +3121,7 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>02:30</t>
+          <t>04:15</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
@@ -3131,7 +3131,7 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>1779037200</t>
+          <t>1779043500</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
@@ -3141,12 +3141,12 @@
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>Ath. Bilbao</t>
+          <t>Cagliari</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>flashscore:athbilbao</t>
+          <t>flashscore:cagliari</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
@@ -3156,12 +3156,12 @@
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>Celta Vigo</t>
+          <t>Torino</t>
         </is>
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>flashscore:celtavigo</t>
+          <t>flashscore:torino</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
@@ -3198,7 +3198,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-05-18 04:02:28 ACST</t>
+          <t>2026-05-18 05:54:08 ACST</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -3213,7 +3213,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>23</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -3223,7 +3223,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>LaLiga</t>
+          <t>Serie A</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -3233,7 +3233,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>flashscore:n12plBB7</t>
+          <t>flashscore:nmmS8WHr</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -3243,7 +3243,7 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>02:30</t>
+          <t>04:15</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
@@ -3253,7 +3253,7 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>1779037200</t>
+          <t>1779043500</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
@@ -3263,12 +3263,12 @@
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>Atl. Madrid</t>
+          <t>Sassuolo</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>flashscore:atlmadrid</t>
+          <t>flashscore:sassuolo</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
@@ -3278,12 +3278,12 @@
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>Girona</t>
+          <t>Lecce</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>flashscore:girona</t>
+          <t>flashscore:lecce</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
@@ -3320,7 +3320,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-05-18 04:02:28 ACST</t>
+          <t>2026-05-18 05:54:08 ACST</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -3335,7 +3335,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>23</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -3345,7 +3345,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>LaLiga</t>
+          <t>Serie A</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -3355,7 +3355,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>flashscore:0OhvAhYQ</t>
+          <t>flashscore:h0IS6Ane</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -3365,7 +3365,7 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>02:30</t>
+          <t>04:15</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
@@ -3375,7 +3375,7 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>1779037200</t>
+          <t>1779043500</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
@@ -3385,12 +3385,12 @@
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>Elche</t>
+          <t>Udinese</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>flashscore:elche</t>
+          <t>flashscore:udinese</t>
         </is>
       </c>
       <c r="P4" t="inlineStr">
@@ -3400,12 +3400,12 @@
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>Getafe</t>
+          <t>Cremonese</t>
         </is>
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>flashscore:getafe</t>
+          <t>flashscore:cremonese</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
@@ -3442,7 +3442,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-05-18 04:02:28 ACST</t>
+          <t>2026-05-18 05:54:08 ACST</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -3457,7 +3457,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>34</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -3467,7 +3467,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>LaLiga</t>
+          <t>Ligue 1</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -3477,7 +3477,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>flashscore:K8ZA4Wel</t>
+          <t>flashscore:prPnPy9r</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
@@ -3487,7 +3487,7 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>02:30</t>
+          <t>04:30</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
@@ -3497,7 +3497,7 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>1779037200</t>
+          <t>1779044400</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
@@ -3507,12 +3507,12 @@
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>Levante</t>
+          <t>Brest</t>
         </is>
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>flashscore:levante</t>
+          <t>flashscore:brest</t>
         </is>
       </c>
       <c r="P5" t="inlineStr">
@@ -3522,12 +3522,12 @@
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>Mallorca</t>
+          <t>Angers</t>
         </is>
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>flashscore:mallorca</t>
+          <t>flashscore:angers</t>
         </is>
       </c>
       <c r="S5" t="inlineStr">
@@ -3564,7 +3564,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-05-18 04:02:28 ACST</t>
+          <t>2026-05-18 05:54:08 ACST</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -3579,7 +3579,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>34</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -3589,7 +3589,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>LaLiga</t>
+          <t>Ligue 1</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -3599,7 +3599,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>flashscore:YFVo6qXh</t>
+          <t>flashscore:IXv8WJG8</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
@@ -3609,7 +3609,7 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>02:30</t>
+          <t>04:30</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
@@ -3619,7 +3619,7 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>1779037200</t>
+          <t>1779044400</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
@@ -3629,12 +3629,12 @@
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>Osasuna</t>
+          <t>Lille</t>
         </is>
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>flashscore:osasuna</t>
+          <t>flashscore:lille</t>
         </is>
       </c>
       <c r="P6" t="inlineStr">
@@ -3644,12 +3644,12 @@
       </c>
       <c r="Q6" t="inlineStr">
         <is>
-          <t>Espanyol</t>
+          <t>Auxerre</t>
         </is>
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>flashscore:espanyol</t>
+          <t>flashscore:auxerre</t>
         </is>
       </c>
       <c r="S6" t="inlineStr">
@@ -3686,7 +3686,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-05-18 04:02:28 ACST</t>
+          <t>2026-05-18 05:54:08 ACST</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -3701,7 +3701,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>34</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -3711,7 +3711,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>LaLiga</t>
+          <t>Ligue 1</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -3721,7 +3721,7 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>flashscore:C0sw852t</t>
+          <t>flashscore:r1cGQTSk</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
@@ -3731,7 +3731,7 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>02:30</t>
+          <t>04:30</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
@@ -3741,7 +3741,7 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>1779037200</t>
+          <t>1779044400</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
@@ -3751,12 +3751,12 @@
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>Oviedo</t>
+          <t>Lorient</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>flashscore:oviedo</t>
+          <t>flashscore:lorient</t>
         </is>
       </c>
       <c r="P7" t="inlineStr">
@@ -3766,12 +3766,12 @@
       </c>
       <c r="Q7" t="inlineStr">
         <is>
-          <t>Alaves</t>
+          <t>Le Havre</t>
         </is>
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>flashscore:alaves</t>
+          <t>flashscore:lehavre</t>
         </is>
       </c>
       <c r="S7" t="inlineStr">
@@ -3808,7 +3808,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-05-18 04:02:28 ACST</t>
+          <t>2026-05-18 05:54:08 ACST</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -3823,7 +3823,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>34</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -3833,7 +3833,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>LaLiga</t>
+          <t>Ligue 1</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -3843,7 +3843,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>flashscore:llRR0leD</t>
+          <t>flashscore:OhrGQlpm</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
@@ -3853,7 +3853,7 @@
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>02:30</t>
+          <t>04:30</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
@@ -3863,7 +3863,7 @@
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>1779037200</t>
+          <t>1779044400</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
@@ -3873,12 +3873,12 @@
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>Real Sociedad</t>
+          <t>Lyon</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>flashscore:realsociedad</t>
+          <t>flashscore:lyon</t>
         </is>
       </c>
       <c r="P8" t="inlineStr">
@@ -3888,12 +3888,12 @@
       </c>
       <c r="Q8" t="inlineStr">
         <is>
-          <t>Valencia</t>
+          <t>Lens</t>
         </is>
       </c>
       <c r="R8" t="inlineStr">
         <is>
-          <t>flashscore:valencia</t>
+          <t>flashscore:lens</t>
         </is>
       </c>
       <c r="S8" t="inlineStr">
@@ -3930,7 +3930,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-05-18 04:02:28 ACST</t>
+          <t>2026-05-18 05:54:08 ACST</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -3945,7 +3945,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>34</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -3955,7 +3955,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>LaLiga</t>
+          <t>Ligue 1</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -3965,7 +3965,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>flashscore:ttZg4N15</t>
+          <t>flashscore:xbwdLg87</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
@@ -3975,7 +3975,7 @@
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>02:30</t>
+          <t>04:30</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
@@ -3985,7 +3985,7 @@
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>1779037200</t>
+          <t>1779044400</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
@@ -3995,12 +3995,12 @@
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>Sevilla</t>
+          <t>Marseille</t>
         </is>
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>flashscore:sevilla</t>
+          <t>flashscore:marseille</t>
         </is>
       </c>
       <c r="P9" t="inlineStr">
@@ -4010,12 +4010,12 @@
       </c>
       <c r="Q9" t="inlineStr">
         <is>
-          <t>Real Madrid</t>
+          <t>Rennes</t>
         </is>
       </c>
       <c r="R9" t="inlineStr">
         <is>
-          <t>flashscore:realmadrid</t>
+          <t>flashscore:rennes</t>
         </is>
       </c>
       <c r="S9" t="inlineStr">
@@ -4052,7 +4052,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-05-18 04:02:28 ACST</t>
+          <t>2026-05-18 05:54:08 ACST</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -4067,7 +4067,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>34</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -4077,7 +4077,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>LaLiga</t>
+          <t>Ligue 1</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -4087,7 +4087,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>flashscore:hMXI2AQ0</t>
+          <t>flashscore:QcrGUcoL</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
@@ -4097,7 +4097,7 @@
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>02:30</t>
+          <t>04:30</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
@@ -4107,7 +4107,7 @@
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>1779037200</t>
+          <t>1779044400</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
@@ -4117,12 +4117,12 @@
       </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>Vallecano</t>
+          <t>Nice</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>flashscore:vallecano</t>
+          <t>flashscore:nice</t>
         </is>
       </c>
       <c r="P10" t="inlineStr">
@@ -4132,12 +4132,12 @@
       </c>
       <c r="Q10" t="inlineStr">
         <is>
-          <t>Villarreal</t>
+          <t>Metz</t>
         </is>
       </c>
       <c r="R10" t="inlineStr">
         <is>
-          <t>flashscore:villarreal</t>
+          <t>flashscore:metz</t>
         </is>
       </c>
       <c r="S10" t="inlineStr">
@@ -4174,7 +4174,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-05-18 04:02:28 ACST</t>
+          <t>2026-05-18 05:54:08 ACST</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -4189,7 +4189,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>34</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -4199,7 +4199,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Serie A</t>
+          <t>Ligue 1</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -4209,7 +4209,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>flashscore:YH84GNJi</t>
+          <t>flashscore:IeNfNFwe</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
@@ -4219,7 +4219,7 @@
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>04:15</t>
+          <t>04:30</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
@@ -4229,7 +4229,7 @@
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>1779043500</t>
+          <t>1779044400</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
@@ -4239,12 +4239,12 @@
       </c>
       <c r="N11" t="inlineStr">
         <is>
-          <t>Cagliari</t>
+          <t>Paris FC</t>
         </is>
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>flashscore:cagliari</t>
+          <t>flashscore:parisfc</t>
         </is>
       </c>
       <c r="P11" t="inlineStr">
@@ -4254,12 +4254,12 @@
       </c>
       <c r="Q11" t="inlineStr">
         <is>
-          <t>Torino</t>
+          <t>PSG</t>
         </is>
       </c>
       <c r="R11" t="inlineStr">
         <is>
-          <t>flashscore:torino</t>
+          <t>flashscore:psg</t>
         </is>
       </c>
       <c r="S11" t="inlineStr">
@@ -4296,7 +4296,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-05-18 04:02:28 ACST</t>
+          <t>2026-05-18 05:54:08 ACST</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -4311,7 +4311,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>34</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -4321,7 +4321,7 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Serie A</t>
+          <t>Ligue 1</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -4331,7 +4331,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>flashscore:nmmS8WHr</t>
+          <t>flashscore:44Vsqc0E</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
@@ -4341,7 +4341,7 @@
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>04:15</t>
+          <t>04:30</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
@@ -4351,7 +4351,7 @@
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>1779043500</t>
+          <t>1779044400</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
@@ -4361,12 +4361,12 @@
       </c>
       <c r="N12" t="inlineStr">
         <is>
-          <t>Sassuolo</t>
+          <t>Strasbourg</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>flashscore:sassuolo</t>
+          <t>flashscore:strasbourg</t>
         </is>
       </c>
       <c r="P12" t="inlineStr">
@@ -4376,12 +4376,12 @@
       </c>
       <c r="Q12" t="inlineStr">
         <is>
-          <t>Lecce</t>
+          <t>Monaco</t>
         </is>
       </c>
       <c r="R12" t="inlineStr">
         <is>
-          <t>flashscore:lecce</t>
+          <t>flashscore:monaco</t>
         </is>
       </c>
       <c r="S12" t="inlineStr">
@@ -4418,7 +4418,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-05-18 04:02:28 ACST</t>
+          <t>2026-05-18 05:54:08 ACST</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -4433,7 +4433,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>8</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -4443,7 +4443,7 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Serie A</t>
+          <t>LaLiga</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -4453,7 +4453,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>flashscore:h0IS6Ane</t>
+          <t>flashscore:SduXBE3E</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
@@ -4463,7 +4463,7 @@
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>04:15</t>
+          <t>04:45</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
@@ -4473,7 +4473,7 @@
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>1779043500</t>
+          <t>1779045300</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
@@ -4483,12 +4483,12 @@
       </c>
       <c r="N13" t="inlineStr">
         <is>
-          <t>Udinese</t>
+          <t>Barcelona</t>
         </is>
       </c>
       <c r="O13" t="inlineStr">
         <is>
-          <t>flashscore:udinese</t>
+          <t>flashscore:barcelona</t>
         </is>
       </c>
       <c r="P13" t="inlineStr">
@@ -4498,12 +4498,12 @@
       </c>
       <c r="Q13" t="inlineStr">
         <is>
-          <t>Cremonese</t>
+          <t>Betis</t>
         </is>
       </c>
       <c r="R13" t="inlineStr">
         <is>
-          <t>flashscore:cremonese</t>
+          <t>flashscore:betis</t>
         </is>
       </c>
       <c r="S13" t="inlineStr">
@@ -4540,7 +4540,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-05-18 04:02:28 ACST</t>
+          <t>2026-05-18 05:54:08 ACST</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -4555,7 +4555,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>34</t>
+          <t>8</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -4565,7 +4565,7 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Ligue 1</t>
+          <t>LaLiga</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -4575,7 +4575,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>flashscore:prPnPy9r</t>
+          <t>flashscore:vyaxjXte</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
@@ -4585,7 +4585,7 @@
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>04:30</t>
+          <t>FT</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
@@ -4595,22 +4595,22 @@
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>1779044400</t>
+          <t>1779037200</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>live</t>
+          <t>FT</t>
         </is>
       </c>
       <c r="N14" t="inlineStr">
         <is>
-          <t>Brest</t>
+          <t>Ath. Bilbao</t>
         </is>
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>flashscore:brest</t>
+          <t>flashscore:athbilbao</t>
         </is>
       </c>
       <c r="P14" t="inlineStr">
@@ -4620,12 +4620,12 @@
       </c>
       <c r="Q14" t="inlineStr">
         <is>
-          <t>Angers</t>
+          <t>Celta Vigo</t>
         </is>
       </c>
       <c r="R14" t="inlineStr">
         <is>
-          <t>flashscore:angers</t>
+          <t>flashscore:celtavigo</t>
         </is>
       </c>
       <c r="S14" t="inlineStr">
@@ -4662,7 +4662,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-05-18 04:02:28 ACST</t>
+          <t>2026-05-18 05:54:08 ACST</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -4677,7 +4677,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>34</t>
+          <t>8</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -4687,7 +4687,7 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Ligue 1</t>
+          <t>LaLiga</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -4697,7 +4697,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>flashscore:IXv8WJG8</t>
+          <t>flashscore:n12plBB7</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
@@ -4707,7 +4707,7 @@
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>04:30</t>
+          <t>FT</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
@@ -4717,22 +4717,22 @@
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>1779044400</t>
+          <t>1779037200</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>live</t>
+          <t>FT</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>Lille</t>
+          <t>Atl. Madrid</t>
         </is>
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>flashscore:lille</t>
+          <t>flashscore:atlmadrid</t>
         </is>
       </c>
       <c r="P15" t="inlineStr">
@@ -4742,12 +4742,12 @@
       </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t>Auxerre</t>
+          <t>Girona</t>
         </is>
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>flashscore:auxerre</t>
+          <t>flashscore:girona</t>
         </is>
       </c>
       <c r="S15" t="inlineStr">
@@ -4784,7 +4784,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-05-18 04:02:28 ACST</t>
+          <t>2026-05-18 05:54:08 ACST</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -4799,7 +4799,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>34</t>
+          <t>8</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -4809,7 +4809,7 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Ligue 1</t>
+          <t>LaLiga</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -4819,7 +4819,7 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>flashscore:r1cGQTSk</t>
+          <t>flashscore:0OhvAhYQ</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
@@ -4829,7 +4829,7 @@
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>04:30</t>
+          <t>FT</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
@@ -4839,22 +4839,22 @@
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>1779044400</t>
+          <t>1779037200</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>live</t>
+          <t>FT</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>Lorient</t>
+          <t>Elche</t>
         </is>
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>flashscore:lorient</t>
+          <t>flashscore:elche</t>
         </is>
       </c>
       <c r="P16" t="inlineStr">
@@ -4864,12 +4864,12 @@
       </c>
       <c r="Q16" t="inlineStr">
         <is>
-          <t>Le Havre</t>
+          <t>Getafe</t>
         </is>
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>flashscore:lehavre</t>
+          <t>flashscore:getafe</t>
         </is>
       </c>
       <c r="S16" t="inlineStr">
@@ -4906,7 +4906,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-05-18 04:02:28 ACST</t>
+          <t>2026-05-18 05:54:08 ACST</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -4921,7 +4921,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>34</t>
+          <t>8</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -4931,7 +4931,7 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Ligue 1</t>
+          <t>LaLiga</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -4941,7 +4941,7 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>flashscore:OhrGQlpm</t>
+          <t>flashscore:K8ZA4Wel</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
@@ -4951,7 +4951,7 @@
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>04:30</t>
+          <t>FT</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
@@ -4961,22 +4961,22 @@
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>1779044400</t>
+          <t>1779037200</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>live</t>
+          <t>FT</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>Lyon</t>
+          <t>Levante</t>
         </is>
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>flashscore:lyon</t>
+          <t>flashscore:levante</t>
         </is>
       </c>
       <c r="P17" t="inlineStr">
@@ -4986,12 +4986,12 @@
       </c>
       <c r="Q17" t="inlineStr">
         <is>
-          <t>Lens</t>
+          <t>Mallorca</t>
         </is>
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>flashscore:lens</t>
+          <t>flashscore:mallorca</t>
         </is>
       </c>
       <c r="S17" t="inlineStr">
@@ -5028,7 +5028,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-05-18 04:02:28 ACST</t>
+          <t>2026-05-18 05:54:08 ACST</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -5043,7 +5043,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>34</t>
+          <t>8</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -5053,7 +5053,7 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Ligue 1</t>
+          <t>LaLiga</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -5063,7 +5063,7 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>flashscore:xbwdLg87</t>
+          <t>flashscore:YFVo6qXh</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
@@ -5073,7 +5073,7 @@
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>04:30</t>
+          <t>FT</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
@@ -5083,22 +5083,22 @@
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>1779044400</t>
+          <t>1779037200</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>live</t>
+          <t>FT</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>Marseille</t>
+          <t>Osasuna</t>
         </is>
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>flashscore:marseille</t>
+          <t>flashscore:osasuna</t>
         </is>
       </c>
       <c r="P18" t="inlineStr">
@@ -5108,12 +5108,12 @@
       </c>
       <c r="Q18" t="inlineStr">
         <is>
-          <t>Rennes</t>
+          <t>Espanyol</t>
         </is>
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>flashscore:rennes</t>
+          <t>flashscore:espanyol</t>
         </is>
       </c>
       <c r="S18" t="inlineStr">
@@ -5150,7 +5150,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-05-18 04:02:28 ACST</t>
+          <t>2026-05-18 05:54:08 ACST</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -5165,7 +5165,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>34</t>
+          <t>8</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -5175,7 +5175,7 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Ligue 1</t>
+          <t>LaLiga</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -5185,7 +5185,7 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>flashscore:z9FNO7c2</t>
+          <t>flashscore:C0sw852t</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
@@ -5195,7 +5195,7 @@
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>04:30</t>
+          <t>FT</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
@@ -5205,22 +5205,22 @@
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>1779044400</t>
+          <t>1779037200</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>live</t>
+          <t>FT</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>Nantes</t>
+          <t>Oviedo</t>
         </is>
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>flashscore:nantes</t>
+          <t>flashscore:oviedo</t>
         </is>
       </c>
       <c r="P19" t="inlineStr">
@@ -5230,12 +5230,12 @@
       </c>
       <c r="Q19" t="inlineStr">
         <is>
-          <t>Toulouse</t>
+          <t>Alaves</t>
         </is>
       </c>
       <c r="R19" t="inlineStr">
         <is>
-          <t>flashscore:toulouse</t>
+          <t>flashscore:alaves</t>
         </is>
       </c>
       <c r="S19" t="inlineStr">
@@ -5272,7 +5272,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-05-18 04:02:28 ACST</t>
+          <t>2026-05-18 05:54:08 ACST</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -5287,7 +5287,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>34</t>
+          <t>8</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -5297,7 +5297,7 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Ligue 1</t>
+          <t>LaLiga</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -5307,7 +5307,7 @@
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>flashscore:QcrGUcoL</t>
+          <t>flashscore:llRR0leD</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
@@ -5317,7 +5317,7 @@
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>04:30</t>
+          <t>FT</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
@@ -5327,22 +5327,22 @@
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>1779044400</t>
+          <t>1779037200</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>live</t>
+          <t>FT</t>
         </is>
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>Nice</t>
+          <t>Real Sociedad</t>
         </is>
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>flashscore:nice</t>
+          <t>flashscore:realsociedad</t>
         </is>
       </c>
       <c r="P20" t="inlineStr">
@@ -5352,12 +5352,12 @@
       </c>
       <c r="Q20" t="inlineStr">
         <is>
-          <t>Metz</t>
+          <t>Valencia</t>
         </is>
       </c>
       <c r="R20" t="inlineStr">
         <is>
-          <t>flashscore:metz</t>
+          <t>flashscore:valencia</t>
         </is>
       </c>
       <c r="S20" t="inlineStr">
@@ -5394,7 +5394,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-05-18 04:02:28 ACST</t>
+          <t>2026-05-18 05:54:08 ACST</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -5409,7 +5409,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>34</t>
+          <t>8</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -5419,7 +5419,7 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Ligue 1</t>
+          <t>LaLiga</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -5429,7 +5429,7 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>flashscore:IeNfNFwe</t>
+          <t>flashscore:ttZg4N15</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
@@ -5439,7 +5439,7 @@
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>04:30</t>
+          <t>FT</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
@@ -5449,22 +5449,22 @@
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>1779044400</t>
+          <t>1779037200</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>live</t>
+          <t>FT</t>
         </is>
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>Paris FC</t>
+          <t>Sevilla</t>
         </is>
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>flashscore:parisfc</t>
+          <t>flashscore:sevilla</t>
         </is>
       </c>
       <c r="P21" t="inlineStr">
@@ -5474,12 +5474,12 @@
       </c>
       <c r="Q21" t="inlineStr">
         <is>
-          <t>PSG</t>
+          <t>Real Madrid</t>
         </is>
       </c>
       <c r="R21" t="inlineStr">
         <is>
-          <t>flashscore:psg</t>
+          <t>flashscore:realmadrid</t>
         </is>
       </c>
       <c r="S21" t="inlineStr">
@@ -5516,7 +5516,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-05-18 04:02:28 ACST</t>
+          <t>2026-05-18 05:54:08 ACST</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -5531,7 +5531,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>34</t>
+          <t>8</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -5541,7 +5541,7 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Ligue 1</t>
+          <t>LaLiga</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -5551,7 +5551,7 @@
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>flashscore:44Vsqc0E</t>
+          <t>flashscore:hMXI2AQ0</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
@@ -5561,7 +5561,7 @@
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>04:30</t>
+          <t>FT</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
@@ -5571,22 +5571,22 @@
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>1779044400</t>
+          <t>1779037200</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>live</t>
+          <t>FT</t>
         </is>
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>Strasbourg</t>
+          <t>Vallecano</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>flashscore:strasbourg</t>
+          <t>flashscore:vallecano</t>
         </is>
       </c>
       <c r="P22" t="inlineStr">
@@ -5596,12 +5596,12 @@
       </c>
       <c r="Q22" t="inlineStr">
         <is>
-          <t>Monaco</t>
+          <t>Villarreal</t>
         </is>
       </c>
       <c r="R22" t="inlineStr">
         <is>
-          <t>flashscore:monaco</t>
+          <t>flashscore:villarreal</t>
         </is>
       </c>
       <c r="S22" t="inlineStr">
@@ -5638,7 +5638,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-05-18 04:02:28 ACST</t>
+          <t>2026-05-18 05:54:08 ACST</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -5653,7 +5653,7 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>34</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -5663,7 +5663,7 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>LaLiga</t>
+          <t>Ligue 1</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -5673,7 +5673,7 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>flashscore:SduXBE3E</t>
+          <t>flashscore:z9FNO7c2</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
@@ -5683,7 +5683,7 @@
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>04:45</t>
+          <t>FT</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
@@ -5693,22 +5693,22 @@
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>1779045300</t>
+          <t>1779044400</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>live</t>
+          <t>FT</t>
         </is>
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>Barcelona</t>
+          <t>Nantes</t>
         </is>
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>flashscore:barcelona</t>
+          <t>flashscore:nantes</t>
         </is>
       </c>
       <c r="P23" t="inlineStr">
@@ -5718,12 +5718,12 @@
       </c>
       <c r="Q23" t="inlineStr">
         <is>
-          <t>Betis</t>
+          <t>Toulouse</t>
         </is>
       </c>
       <c r="R23" t="inlineStr">
         <is>
-          <t>flashscore:betis</t>
+          <t>flashscore:toulouse</t>
         </is>
       </c>
       <c r="S23" t="inlineStr">
@@ -5760,7 +5760,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2026-05-18 04:02:28 ACST</t>
+          <t>2026-05-18 05:54:08 ACST</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -6279,12 +6279,12 @@
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>1</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>9</t>
         </is>
       </c>
     </row>
@@ -6351,12 +6351,12 @@
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>8</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
     </row>
@@ -6484,7 +6484,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-05-18 04:02:28 ACST</t>
+          <t>2026-05-18 05:54:08 ACST</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -6519,7 +6519,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>events=1195 league_hit=57 skipped_women=1 out_of_window=33 matched=23 by_league={'Ligue 1': 9, 'Serie A': 4, 'LaLiga': 10} sample_leagues=['Africa|AFRICA: CAF Champions League - Play Offs', 'Africa|AFRICA: Africa Cup of Nations U17', 'Albania|ALBANIA: Abissnet Superiore - Final Group', 'Andorra|ANDORRA: Primera Divisió', 'Angola|ANGOLA: Girabola', 'Argentina|ARGENTINA: Liga Profesional - Apertura - Play Offs', 'Argentina|ARGENTINA: Primera Nacional', 'Argentina|ARGENTINA: Torneo Federal']</t>
+          <t>events=1198 league_hit=57 skipped_women=1 out_of_window=33 matched=23 by_league={'Ligue 1': 9, 'Serie A': 4, 'LaLiga': 10} sample_leagues=['Africa|AFRICA: CAF Champions League - Play Offs', 'Africa|AFRICA: Africa Cup of Nations U17', 'Albania|ALBANIA: Abissnet Superiore - Final Group', 'Andorra|ANDORRA: Primera Divisió', 'Angola|ANGOLA: Girabola', 'Argentina|ARGENTINA: Liga Profesional - Apertura - Play Offs', 'Argentina|ARGENTINA: Primera Nacional', 'Argentina|ARGENTINA: Torneo Federal']</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto-push 2026-05-18T14:05: settle results + forecasts
</commit_message>
<xml_diff>
--- a/docs/agent-system/outputs/Phase1_Fixture_Slate.xlsx
+++ b/docs/agent-system/outputs/Phase1_Fixture_Slate.xlsx
@@ -141,7 +141,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-05-18 09:53:52 ACST</t>
+          <t>2026-05-18 13:53:53 ACST</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -176,7 +176,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>flashscore:lnSvmTkR</t>
+          <t>flashscore:rZdvkkLE</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -186,7 +186,7 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>09:30</t>
+          <t>FT</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
@@ -196,22 +196,22 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>1779062400</t>
+          <t>1779055200</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>live</t>
+          <t>FT</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>Nashville SC</t>
+          <t>Inter Miami</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>flashscore:nashvillesc</t>
+          <t>flashscore:intermiami</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
@@ -221,12 +221,12 @@
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>Los Angeles FC</t>
+          <t>Portland Timbers</t>
         </is>
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>flashscore:losangelesfc</t>
+          <t>flashscore:portlandtimbers</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
@@ -263,7 +263,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-05-18 09:53:52 ACST</t>
+          <t>2026-05-18 13:53:53 ACST</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -298,7 +298,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>flashscore:rZdvkkLE</t>
+          <t>flashscore:lnSvmTkR</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -318,7 +318,7 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>1779055200</t>
+          <t>1779062400</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
@@ -328,12 +328,12 @@
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>Inter Miami</t>
+          <t>Nashville SC</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>flashscore:intermiami</t>
+          <t>flashscore:nashvillesc</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
@@ -343,12 +343,12 @@
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>Portland Timbers</t>
+          <t>Los Angeles FC</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>flashscore:portlandtimbers</t>
+          <t>flashscore:losangelesfc</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
@@ -385,7 +385,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-05-18 09:53:52 ACST</t>
+          <t>2026-05-18 13:53:53 ACST</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -636,7 +636,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-05-18 09:53:52 ACST</t>
+          <t>2026-05-18 13:53:53 ACST</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -671,7 +671,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>flashscore:lnSvmTkR</t>
+          <t>flashscore:rZdvkkLE</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -681,7 +681,7 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>09:30</t>
+          <t>FT</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
@@ -691,22 +691,22 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>1779062400</t>
+          <t>1779055200</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>live</t>
+          <t>FT</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>Nashville SC</t>
+          <t>Inter Miami</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>flashscore:nashvillesc</t>
+          <t>flashscore:intermiami</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
@@ -716,12 +716,12 @@
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>Los Angeles FC</t>
+          <t>Portland Timbers</t>
         </is>
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>flashscore:losangelesfc</t>
+          <t>flashscore:portlandtimbers</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
@@ -758,7 +758,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-05-18 09:53:52 ACST</t>
+          <t>2026-05-18 13:53:53 ACST</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -793,7 +793,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>flashscore:rZdvkkLE</t>
+          <t>flashscore:lnSvmTkR</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -813,7 +813,7 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>1779055200</t>
+          <t>1779062400</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
@@ -823,12 +823,12 @@
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>Inter Miami</t>
+          <t>Nashville SC</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>flashscore:intermiami</t>
+          <t>flashscore:nashvillesc</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
@@ -838,12 +838,12 @@
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>Portland Timbers</t>
+          <t>Los Angeles FC</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>flashscore:portlandtimbers</t>
+          <t>flashscore:losangelesfc</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
@@ -880,7 +880,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-05-18 09:53:52 ACST</t>
+          <t>2026-05-18 13:53:53 ACST</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -1399,12 +1399,12 @@
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
     </row>
@@ -1532,7 +1532,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-05-18 09:53:52 ACST</t>
+          <t>2026-05-18 13:53:53 ACST</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -1567,7 +1567,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>events=200 league_hit=3 skipped_women=0 out_of_window=0 matched=3 by_league={'Premier League': 1, 'MLS': 2} sample_leagues=['Argentina|ARGENTINA: Liga Profesional - Apertura - Play Offs', 'Argentina|ARGENTINA: Primera Nacional', 'Argentina|ARGENTINA: Torneo Federal', 'Argentina|ARGENTINA: Primera B', 'Argentina|ARGENTINA: Primera C', 'Armenia|ARMENIA: Premier League', 'Armenia|ARMENIA: First League', 'Australia|AUSTRALIA: NPL Victoria']</t>
+          <t>events=196 league_hit=3 skipped_women=0 out_of_window=0 matched=3 by_league={'Premier League': 1, 'MLS': 2} sample_leagues=['Argentina|ARGENTINA: Liga Profesional - Apertura - Play Offs', 'Argentina|ARGENTINA: Primera Nacional', 'Argentina|ARGENTINA: Torneo Federal', 'Argentina|ARGENTINA: Primera B', 'Argentina|ARGENTINA: Primera C', 'Armenia|ARMENIA: Premier League', 'Armenia|ARMENIA: First League', 'Australia|AUSTRALIA: NPL Victoria']</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto-push 2026-05-18T18:05: settle results + forecasts
</commit_message>
<xml_diff>
--- a/docs/agent-system/outputs/Phase1_Fixture_Slate.xlsx
+++ b/docs/agent-system/outputs/Phase1_Fixture_Slate.xlsx
@@ -141,7 +141,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-05-18 13:53:53 ACST</t>
+          <t>2026-05-18 17:53:53 ACST</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -263,7 +263,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-05-18 13:53:53 ACST</t>
+          <t>2026-05-18 17:53:53 ACST</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -385,7 +385,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-05-18 13:53:53 ACST</t>
+          <t>2026-05-18 17:53:53 ACST</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -636,7 +636,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-05-18 13:53:53 ACST</t>
+          <t>2026-05-18 17:53:53 ACST</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -758,7 +758,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-05-18 13:53:53 ACST</t>
+          <t>2026-05-18 17:53:53 ACST</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -880,7 +880,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-05-18 13:53:53 ACST</t>
+          <t>2026-05-18 17:53:53 ACST</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -1532,7 +1532,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-05-18 13:53:53 ACST</t>
+          <t>2026-05-18 17:53:53 ACST</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">

</xml_diff>

<commit_message>
Auto-push 2026-05-19T02:05: settle results + forecasts
</commit_message>
<xml_diff>
--- a/docs/agent-system/outputs/Phase1_Fixture_Slate.xlsx
+++ b/docs/agent-system/outputs/Phase1_Fixture_Slate.xlsx
@@ -141,7 +141,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-05-18 17:53:53 ACST</t>
+          <t>2026-05-19 01:53:43 ACST</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -156,7 +156,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>242</t>
+          <t>17</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -166,7 +166,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>MLS</t>
+          <t>Premier League</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -176,17 +176,17 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>flashscore:rZdvkkLE</t>
+          <t>flashscore:Gxt6zm15</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>FT</t>
+          <t>04:30</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
@@ -196,22 +196,22 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>1779055200</t>
+          <t>1779130800</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>FT</t>
+          <t>live</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>Inter Miami</t>
+          <t>Arsenal</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>flashscore:intermiami</t>
+          <t>flashscore:arsenal</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
@@ -221,12 +221,12 @@
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>Portland Timbers</t>
+          <t>Burnley</t>
         </is>
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>flashscore:portlandtimbers</t>
+          <t>flashscore:burnley</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
@@ -255,250 +255,6 @@
         </is>
       </c>
       <c r="X2" t="inlineStr">
-        <is>
-          <t>Keyless Flashscore fixture feed.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>2026-05-18 17:53:53 ACST</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Flashscore</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>healthy</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>242</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>MLS</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>flashscore:lnSvmTkR</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>2026-05-18</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>FT</t>
-        </is>
-      </c>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>Australia/Adelaide</t>
-        </is>
-      </c>
-      <c r="L3" t="inlineStr">
-        <is>
-          <t>1779062400</t>
-        </is>
-      </c>
-      <c r="M3" t="inlineStr">
-        <is>
-          <t>FT</t>
-        </is>
-      </c>
-      <c r="N3" t="inlineStr">
-        <is>
-          <t>Nashville SC</t>
-        </is>
-      </c>
-      <c r="O3" t="inlineStr">
-        <is>
-          <t>flashscore:nashvillesc</t>
-        </is>
-      </c>
-      <c r="P3" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="Q3" t="inlineStr">
-        <is>
-          <t>Los Angeles FC</t>
-        </is>
-      </c>
-      <c r="R3" t="inlineStr">
-        <is>
-          <t>flashscore:losangelesfc</t>
-        </is>
-      </c>
-      <c r="S3" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="T3" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="U3" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="V3" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="W3" t="inlineStr">
-        <is>
-          <t>ready_for_phase_2</t>
-        </is>
-      </c>
-      <c r="X3" t="inlineStr">
-        <is>
-          <t>Keyless Flashscore fixture feed.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>2026-05-18 17:53:53 ACST</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Flashscore</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>healthy</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>17</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>Premier League</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>flashscore:Gxt6zm15</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>2026-05-19</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>04:30</t>
-        </is>
-      </c>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>Australia/Adelaide</t>
-        </is>
-      </c>
-      <c r="L4" t="inlineStr">
-        <is>
-          <t>1779130800</t>
-        </is>
-      </c>
-      <c r="M4" t="inlineStr">
-        <is>
-          <t>live</t>
-        </is>
-      </c>
-      <c r="N4" t="inlineStr">
-        <is>
-          <t>Arsenal</t>
-        </is>
-      </c>
-      <c r="O4" t="inlineStr">
-        <is>
-          <t>flashscore:arsenal</t>
-        </is>
-      </c>
-      <c r="P4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="Q4" t="inlineStr">
-        <is>
-          <t>Burnley</t>
-        </is>
-      </c>
-      <c r="R4" t="inlineStr">
-        <is>
-          <t>flashscore:burnley</t>
-        </is>
-      </c>
-      <c r="S4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="T4" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="U4" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="V4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="W4" t="inlineStr">
-        <is>
-          <t>ready_for_phase_2</t>
-        </is>
-      </c>
-      <c r="X4" t="inlineStr">
         <is>
           <t>Keyless Flashscore fixture feed.</t>
         </is>
@@ -636,7 +392,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-05-18 17:53:53 ACST</t>
+          <t>2026-05-19 01:53:43 ACST</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -651,7 +407,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>242</t>
+          <t>17</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -661,7 +417,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>MLS</t>
+          <t>Premier League</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -671,17 +427,17 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>flashscore:rZdvkkLE</t>
+          <t>flashscore:Gxt6zm15</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>FT</t>
+          <t>04:30</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
@@ -691,22 +447,22 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>1779055200</t>
+          <t>1779130800</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>FT</t>
+          <t>live</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>Inter Miami</t>
+          <t>Arsenal</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>flashscore:intermiami</t>
+          <t>flashscore:arsenal</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
@@ -716,12 +472,12 @@
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>Portland Timbers</t>
+          <t>Burnley</t>
         </is>
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>flashscore:portlandtimbers</t>
+          <t>flashscore:burnley</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
@@ -750,250 +506,6 @@
         </is>
       </c>
       <c r="X2" t="inlineStr">
-        <is>
-          <t>Keyless Flashscore fixture feed.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>2026-05-18 17:53:53 ACST</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Flashscore</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>healthy</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>242</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>MLS</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>flashscore:lnSvmTkR</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>2026-05-18</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>FT</t>
-        </is>
-      </c>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>Australia/Adelaide</t>
-        </is>
-      </c>
-      <c r="L3" t="inlineStr">
-        <is>
-          <t>1779062400</t>
-        </is>
-      </c>
-      <c r="M3" t="inlineStr">
-        <is>
-          <t>FT</t>
-        </is>
-      </c>
-      <c r="N3" t="inlineStr">
-        <is>
-          <t>Nashville SC</t>
-        </is>
-      </c>
-      <c r="O3" t="inlineStr">
-        <is>
-          <t>flashscore:nashvillesc</t>
-        </is>
-      </c>
-      <c r="P3" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="Q3" t="inlineStr">
-        <is>
-          <t>Los Angeles FC</t>
-        </is>
-      </c>
-      <c r="R3" t="inlineStr">
-        <is>
-          <t>flashscore:losangelesfc</t>
-        </is>
-      </c>
-      <c r="S3" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="T3" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="U3" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="V3" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="W3" t="inlineStr">
-        <is>
-          <t>ready_for_phase_2</t>
-        </is>
-      </c>
-      <c r="X3" t="inlineStr">
-        <is>
-          <t>Keyless Flashscore fixture feed.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>2026-05-18 17:53:53 ACST</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Flashscore</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>healthy</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>17</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>Premier League</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>flashscore:Gxt6zm15</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>2026-05-19</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>04:30</t>
-        </is>
-      </c>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>Australia/Adelaide</t>
-        </is>
-      </c>
-      <c r="L4" t="inlineStr">
-        <is>
-          <t>1779130800</t>
-        </is>
-      </c>
-      <c r="M4" t="inlineStr">
-        <is>
-          <t>live</t>
-        </is>
-      </c>
-      <c r="N4" t="inlineStr">
-        <is>
-          <t>Arsenal</t>
-        </is>
-      </c>
-      <c r="O4" t="inlineStr">
-        <is>
-          <t>flashscore:arsenal</t>
-        </is>
-      </c>
-      <c r="P4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="Q4" t="inlineStr">
-        <is>
-          <t>Burnley</t>
-        </is>
-      </c>
-      <c r="R4" t="inlineStr">
-        <is>
-          <t>flashscore:burnley</t>
-        </is>
-      </c>
-      <c r="S4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="T4" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="U4" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="V4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="W4" t="inlineStr">
-        <is>
-          <t>ready_for_phase_2</t>
-        </is>
-      </c>
-      <c r="X4" t="inlineStr">
         <is>
           <t>Keyless Flashscore fixture feed.</t>
         </is>
@@ -1339,17 +851,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>MLS</t>
+          <t>Premier League</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -1399,82 +911,10 @@
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Premier League</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="L3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="M3" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="N3" t="inlineStr">
         <is>
           <t>0</t>
         </is>
@@ -1532,7 +972,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-05-18 17:53:53 ACST</t>
+          <t>2026-05-19 01:53:43 ACST</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -1547,7 +987,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-05-18 to 2026-05-24</t>
+          <t>2026-05-19 to 2026-05-25</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -1562,12 +1002,12 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>events=196 league_hit=3 skipped_women=0 out_of_window=0 matched=3 by_league={'Premier League': 1, 'MLS': 2} sample_leagues=['Argentina|ARGENTINA: Liga Profesional - Apertura - Play Offs', 'Argentina|ARGENTINA: Primera Nacional', 'Argentina|ARGENTINA: Torneo Federal', 'Argentina|ARGENTINA: Primera B', 'Argentina|ARGENTINA: Primera C', 'Armenia|ARMENIA: Premier League', 'Armenia|ARMENIA: First League', 'Australia|AUSTRALIA: NPL Victoria']</t>
+          <t>events=202 league_hit=3 skipped_women=0 out_of_window=2 matched=1 by_league={'Premier League': 1} sample_leagues=['Argentina|ARGENTINA: Liga Profesional - Apertura - Play Offs', 'Argentina|ARGENTINA: Primera Nacional', 'Argentina|ARGENTINA: Torneo Federal', 'Argentina|ARGENTINA: Primera B', 'Argentina|ARGENTINA: Primera C', 'Armenia|ARMENIA: Premier League', 'Armenia|ARMENIA: First League', 'Aruba|ARUBA: Division di Honor - Relegation']</t>
         </is>
       </c>
     </row>
@@ -1598,7 +1038,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-05-18 to 2026-05-24</t>
+          <t>2026-05-19 to 2026-05-25</t>
         </is>
       </c>
     </row>
@@ -1634,7 +1074,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
     </row>
@@ -1646,7 +1086,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto-push 2026-05-19T18:07: settle results + forecasts
</commit_message>
<xml_diff>
--- a/docs/agent-system/outputs/Phase1_Fixture_Slate.xlsx
+++ b/docs/agent-system/outputs/Phase1_Fixture_Slate.xlsx
@@ -141,7 +141,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-05-19 01:53:43 ACST</t>
+          <t>2026-05-19 17:59:04 ACST</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -176,17 +176,17 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>flashscore:Gxt6zm15</t>
+          <t>flashscore:rkXMW40U</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>04:30</t>
+          <t>04:00</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
@@ -196,7 +196,7 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>1779130800</t>
+          <t>1779215400</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
@@ -206,12 +206,12 @@
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>Arsenal</t>
+          <t>Bournemouth</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>flashscore:arsenal</t>
+          <t>flashscore:bournemouth</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
@@ -221,12 +221,12 @@
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>Burnley</t>
+          <t>Manchester City</t>
         </is>
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>flashscore:burnley</t>
+          <t>flashscore:manchestercity</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
@@ -255,6 +255,128 @@
         </is>
       </c>
       <c r="X2" t="inlineStr">
+        <is>
+          <t>Keyless Flashscore fixture feed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-05-19 17:59:04 ACST</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Flashscore</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>healthy</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>17</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Premier League</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>flashscore:Uu6uknGb</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>04:45</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>Australia/Adelaide</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>1779218100</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>Chelsea</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>flashscore:chelsea</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>Tottenham</t>
+        </is>
+      </c>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>flashscore:tottenham</t>
+        </is>
+      </c>
+      <c r="S3" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="T3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="U3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="V3" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="W3" t="inlineStr">
+        <is>
+          <t>ready_for_phase_2</t>
+        </is>
+      </c>
+      <c r="X3" t="inlineStr">
         <is>
           <t>Keyless Flashscore fixture feed.</t>
         </is>
@@ -392,7 +514,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-05-19 01:53:43 ACST</t>
+          <t>2026-05-19 17:59:04 ACST</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -427,17 +549,17 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>flashscore:Gxt6zm15</t>
+          <t>flashscore:rkXMW40U</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>04:30</t>
+          <t>04:00</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
@@ -447,7 +569,7 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>1779130800</t>
+          <t>1779215400</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
@@ -457,12 +579,12 @@
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>Arsenal</t>
+          <t>Bournemouth</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>flashscore:arsenal</t>
+          <t>flashscore:bournemouth</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
@@ -472,12 +594,12 @@
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>Burnley</t>
+          <t>Manchester City</t>
         </is>
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>flashscore:burnley</t>
+          <t>flashscore:manchestercity</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
@@ -506,6 +628,128 @@
         </is>
       </c>
       <c r="X2" t="inlineStr">
+        <is>
+          <t>Keyless Flashscore fixture feed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-05-19 17:59:04 ACST</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Flashscore</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>healthy</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>17</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Premier League</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>flashscore:Uu6uknGb</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>04:45</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>Australia/Adelaide</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>1779218100</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>Chelsea</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>flashscore:chelsea</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>Tottenham</t>
+        </is>
+      </c>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>flashscore:tottenham</t>
+        </is>
+      </c>
+      <c r="S3" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="T3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="U3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="V3" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="W3" t="inlineStr">
+        <is>
+          <t>ready_for_phase_2</t>
+        </is>
+      </c>
+      <c r="X3" t="inlineStr">
         <is>
           <t>Keyless Flashscore fixture feed.</t>
         </is>
@@ -856,12 +1100,12 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -911,7 +1155,7 @@
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
@@ -972,7 +1216,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-05-19 01:53:43 ACST</t>
+          <t>2026-05-19 17:59:04 ACST</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -1002,12 +1246,12 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>events=202 league_hit=3 skipped_women=0 out_of_window=2 matched=1 by_league={'Premier League': 1} sample_leagues=['Argentina|ARGENTINA: Liga Profesional - Apertura - Play Offs', 'Argentina|ARGENTINA: Primera Nacional', 'Argentina|ARGENTINA: Torneo Federal', 'Argentina|ARGENTINA: Primera B', 'Argentina|ARGENTINA: Primera C', 'Armenia|ARMENIA: Premier League', 'Armenia|ARMENIA: First League', 'Aruba|ARUBA: Division di Honor - Relegation']</t>
+          <t>events=153 league_hit=2 skipped_women=0 out_of_window=0 matched=2 by_league={'Premier League': 2} sample_leagues=['Africa|AFRICA: Africa Cup of Nations U17', 'Algeria|ALGERIA: Ligue 1', 'Argentina|ARGENTINA: Primera Nacional', 'Argentina|ARGENTINA: Reserve League - Apertura', 'Armenia|ARMENIA: Premier League', 'Armenia|ARMENIA: First League', 'Aruba|ARUBA: Division di Honor - Relegation', 'Asia|ASIA: AFC Asian Cup U17 - Play Offs']</t>
         </is>
       </c>
     </row>
@@ -1074,7 +1318,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
     </row>
@@ -1086,7 +1330,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto-push 2026-05-20T02:07: settle results + forecasts
</commit_message>
<xml_diff>
--- a/docs/agent-system/outputs/Phase1_Fixture_Slate.xlsx
+++ b/docs/agent-system/outputs/Phase1_Fixture_Slate.xlsx
@@ -141,7 +141,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-05-19 17:59:04 ACST</t>
+          <t>2026-05-20 01:56:04 ACST</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -263,7 +263,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-05-19 17:59:04 ACST</t>
+          <t>2026-05-20 01:56:04 ACST</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -514,7 +514,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-05-19 17:59:04 ACST</t>
+          <t>2026-05-20 01:56:04 ACST</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -636,7 +636,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-05-19 17:59:04 ACST</t>
+          <t>2026-05-20 01:56:04 ACST</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -1216,7 +1216,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-05-19 17:59:04 ACST</t>
+          <t>2026-05-20 01:56:04 ACST</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -1231,7 +1231,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-05-19 to 2026-05-25</t>
+          <t>2026-05-20 to 2026-05-26</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -1251,7 +1251,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>events=153 league_hit=2 skipped_women=0 out_of_window=0 matched=2 by_league={'Premier League': 2} sample_leagues=['Africa|AFRICA: Africa Cup of Nations U17', 'Algeria|ALGERIA: Ligue 1', 'Argentina|ARGENTINA: Primera Nacional', 'Argentina|ARGENTINA: Reserve League - Apertura', 'Armenia|ARMENIA: Premier League', 'Armenia|ARMENIA: First League', 'Aruba|ARUBA: Division di Honor - Relegation', 'Asia|ASIA: AFC Asian Cup U17 - Play Offs']</t>
+          <t>events=151 league_hit=2 skipped_women=0 out_of_window=0 matched=2 by_league={'Premier League': 2} sample_leagues=['Africa|AFRICA: Africa Cup of Nations U17', 'Algeria|ALGERIA: Ligue 1', 'Argentina|ARGENTINA: Primera Nacional', 'Argentina|ARGENTINA: Reserve League - Apertura', 'Armenia|ARMENIA: Premier League', 'Armenia|ARMENIA: First League', 'Aruba|ARUBA: Division di Honor - Relegation', 'Asia|ASIA: AFC Asian Cup U17 - Play Offs']</t>
         </is>
       </c>
     </row>
@@ -1282,7 +1282,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-05-19 to 2026-05-25</t>
+          <t>2026-05-20 to 2026-05-26</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto-push 2026-05-20T06:06: settle results + forecasts
</commit_message>
<xml_diff>
--- a/docs/agent-system/outputs/Phase1_Fixture_Slate.xlsx
+++ b/docs/agent-system/outputs/Phase1_Fixture_Slate.xlsx
@@ -141,7 +141,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-05-20 01:56:04 ACST</t>
+          <t>2026-05-20 05:55:35 ACST</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -176,7 +176,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>flashscore:rkXMW40U</t>
+          <t>flashscore:Uu6uknGb</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -186,7 +186,7 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>04:00</t>
+          <t>04:45</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
@@ -196,7 +196,7 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>1779215400</t>
+          <t>1779218100</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
@@ -206,12 +206,12 @@
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>Bournemouth</t>
+          <t>Chelsea</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>flashscore:bournemouth</t>
+          <t>flashscore:chelsea</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
@@ -221,12 +221,12 @@
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>Manchester City</t>
+          <t>Tottenham</t>
         </is>
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>flashscore:manchestercity</t>
+          <t>flashscore:tottenham</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
@@ -263,7 +263,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-05-20 01:56:04 ACST</t>
+          <t>2026-05-20 05:55:35 ACST</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -298,7 +298,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>flashscore:Uu6uknGb</t>
+          <t>flashscore:rkXMW40U</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -308,7 +308,7 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>04:45</t>
+          <t>FT</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
@@ -318,22 +318,22 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>1779218100</t>
+          <t>1779215400</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>live</t>
+          <t>FT</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>Chelsea</t>
+          <t>Bournemouth</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>flashscore:chelsea</t>
+          <t>flashscore:bournemouth</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
@@ -343,12 +343,12 @@
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>Tottenham</t>
+          <t>Manchester City</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>flashscore:tottenham</t>
+          <t>flashscore:manchestercity</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
@@ -514,7 +514,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-05-20 01:56:04 ACST</t>
+          <t>2026-05-20 05:55:35 ACST</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -549,7 +549,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>flashscore:rkXMW40U</t>
+          <t>flashscore:Uu6uknGb</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -559,7 +559,7 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>04:00</t>
+          <t>04:45</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
@@ -569,7 +569,7 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>1779215400</t>
+          <t>1779218100</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
@@ -579,12 +579,12 @@
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>Bournemouth</t>
+          <t>Chelsea</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>flashscore:bournemouth</t>
+          <t>flashscore:chelsea</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
@@ -594,12 +594,12 @@
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>Manchester City</t>
+          <t>Tottenham</t>
         </is>
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>flashscore:manchestercity</t>
+          <t>flashscore:tottenham</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
@@ -636,7 +636,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-05-20 01:56:04 ACST</t>
+          <t>2026-05-20 05:55:35 ACST</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -671,7 +671,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>flashscore:Uu6uknGb</t>
+          <t>flashscore:rkXMW40U</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -681,7 +681,7 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>04:45</t>
+          <t>FT</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
@@ -691,22 +691,22 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>1779218100</t>
+          <t>1779215400</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>live</t>
+          <t>FT</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>Chelsea</t>
+          <t>Bournemouth</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>flashscore:chelsea</t>
+          <t>flashscore:bournemouth</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
@@ -716,12 +716,12 @@
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>Tottenham</t>
+          <t>Manchester City</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>flashscore:tottenham</t>
+          <t>flashscore:manchestercity</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
@@ -1155,12 +1155,12 @@
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
     </row>
@@ -1216,7 +1216,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-05-20 01:56:04 ACST</t>
+          <t>2026-05-20 05:55:35 ACST</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">

</xml_diff>

<commit_message>
Promote phase fixtures into dashboard data
</commit_message>
<xml_diff>
--- a/docs/agent-system/outputs/Phase1_Fixture_Slate.xlsx
+++ b/docs/agent-system/outputs/Phase1_Fixture_Slate.xlsx
@@ -141,7 +141,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-05-21 01:55:45 ACST</t>
+          <t>2026-05-21 03:42:10 ACST</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -156,7 +156,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>40</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -166,7 +166,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Eliteserien</t>
+          <t>Allsvenskan</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -176,7 +176,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>flashscore:v3i3qEfD</t>
+          <t>flashscore:rJKJ2MZP</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -186,7 +186,7 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>01:30</t>
+          <t>02:30</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
@@ -196,7 +196,7 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>1779292800</t>
+          <t>1779296400</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
@@ -206,12 +206,12 @@
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>Start</t>
+          <t>GAIS</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>flashscore:start</t>
+          <t>flashscore:gais</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
@@ -221,12 +221,12 @@
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>Bodo/Glimt</t>
+          <t>Hammarby</t>
         </is>
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>flashscore:bodoglimt</t>
+          <t>flashscore:hammarby</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
@@ -263,7 +263,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-05-21 01:55:45 ACST</t>
+          <t>2026-05-21 03:42:10 ACST</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -278,7 +278,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>20</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -288,7 +288,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Allsvenskan</t>
+          <t>Eliteserien</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -298,7 +298,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>flashscore:rJKJ2MZP</t>
+          <t>flashscore:YobepuNG</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -328,12 +328,12 @@
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>GAIS</t>
+          <t>Lilleström</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>flashscore:gais</t>
+          <t>flashscore:lilleström</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
@@ -343,12 +343,12 @@
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>Hammarby</t>
+          <t>Kristiansund</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>flashscore:hammarby</t>
+          <t>flashscore:kristiansund</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
@@ -385,7 +385,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-05-21 01:55:45 ACST</t>
+          <t>2026-05-21 03:42:10 ACST</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -420,7 +420,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>flashscore:YobepuNG</t>
+          <t>flashscore:0A1Nl9Wh</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -430,7 +430,7 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>02:30</t>
+          <t>03:30</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
@@ -440,7 +440,7 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>1779296400</t>
+          <t>1779300000</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
@@ -450,12 +450,12 @@
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>Lilleström</t>
+          <t>Aalesund</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>flashscore:lilleström</t>
+          <t>flashscore:aalesund</t>
         </is>
       </c>
       <c r="P4" t="inlineStr">
@@ -465,12 +465,12 @@
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>Kristiansund</t>
+          <t>Brann</t>
         </is>
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>flashscore:kristiansund</t>
+          <t>flashscore:brann</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
@@ -507,7 +507,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-05-21 01:55:45 ACST</t>
+          <t>2026-05-21 03:42:10 ACST</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -542,7 +542,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>flashscore:0A1Nl9Wh</t>
+          <t>flashscore:v3i3qEfD</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
@@ -552,7 +552,7 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>03:30</t>
+          <t>FT</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
@@ -562,22 +562,22 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>1779300000</t>
+          <t>1779292800</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>live</t>
+          <t>FT</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>Aalesund</t>
+          <t>Start</t>
         </is>
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>flashscore:aalesund</t>
+          <t>flashscore:start</t>
         </is>
       </c>
       <c r="P5" t="inlineStr">
@@ -587,12 +587,12 @@
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>Brann</t>
+          <t>Bodo/Glimt</t>
         </is>
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>flashscore:brann</t>
+          <t>flashscore:bodoglimt</t>
         </is>
       </c>
       <c r="S5" t="inlineStr">
@@ -758,7 +758,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-05-21 01:55:45 ACST</t>
+          <t>2026-05-21 03:42:10 ACST</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -773,7 +773,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>40</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -783,7 +783,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Eliteserien</t>
+          <t>Allsvenskan</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -793,7 +793,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>flashscore:v3i3qEfD</t>
+          <t>flashscore:rJKJ2MZP</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -803,7 +803,7 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>01:30</t>
+          <t>02:30</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
@@ -813,7 +813,7 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>1779292800</t>
+          <t>1779296400</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
@@ -823,12 +823,12 @@
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>Start</t>
+          <t>GAIS</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>flashscore:start</t>
+          <t>flashscore:gais</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
@@ -838,12 +838,12 @@
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>Bodo/Glimt</t>
+          <t>Hammarby</t>
         </is>
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>flashscore:bodoglimt</t>
+          <t>flashscore:hammarby</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
@@ -880,7 +880,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-05-21 01:55:45 ACST</t>
+          <t>2026-05-21 03:42:10 ACST</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -895,7 +895,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>20</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -905,7 +905,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Allsvenskan</t>
+          <t>Eliteserien</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -915,7 +915,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>flashscore:rJKJ2MZP</t>
+          <t>flashscore:YobepuNG</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -945,12 +945,12 @@
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>GAIS</t>
+          <t>Lilleström</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>flashscore:gais</t>
+          <t>flashscore:lilleström</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
@@ -960,12 +960,12 @@
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>Hammarby</t>
+          <t>Kristiansund</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>flashscore:hammarby</t>
+          <t>flashscore:kristiansund</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
@@ -1002,7 +1002,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-05-21 01:55:45 ACST</t>
+          <t>2026-05-21 03:42:10 ACST</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -1037,7 +1037,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>flashscore:YobepuNG</t>
+          <t>flashscore:0A1Nl9Wh</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -1047,7 +1047,7 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>02:30</t>
+          <t>03:30</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
@@ -1057,7 +1057,7 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>1779296400</t>
+          <t>1779300000</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
@@ -1067,12 +1067,12 @@
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>Lilleström</t>
+          <t>Aalesund</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>flashscore:lilleström</t>
+          <t>flashscore:aalesund</t>
         </is>
       </c>
       <c r="P4" t="inlineStr">
@@ -1082,12 +1082,12 @@
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>Kristiansund</t>
+          <t>Brann</t>
         </is>
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>flashscore:kristiansund</t>
+          <t>flashscore:brann</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
@@ -1124,7 +1124,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-05-21 01:55:45 ACST</t>
+          <t>2026-05-21 03:42:10 ACST</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -1159,7 +1159,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>flashscore:0A1Nl9Wh</t>
+          <t>flashscore:v3i3qEfD</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
@@ -1169,7 +1169,7 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>03:30</t>
+          <t>FT</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
@@ -1179,22 +1179,22 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>1779300000</t>
+          <t>1779292800</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>live</t>
+          <t>FT</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>Aalesund</t>
+          <t>Start</t>
         </is>
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>flashscore:aalesund</t>
+          <t>flashscore:start</t>
         </is>
       </c>
       <c r="P5" t="inlineStr">
@@ -1204,12 +1204,12 @@
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>Brann</t>
+          <t>Bodo/Glimt</t>
         </is>
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>flashscore:brann</t>
+          <t>flashscore:bodoglimt</t>
         </is>
       </c>
       <c r="S5" t="inlineStr">
@@ -1715,12 +1715,12 @@
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
     </row>
@@ -1776,7 +1776,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-05-21 01:55:45 ACST</t>
+          <t>2026-05-21 03:42:10 ACST</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">

</xml_diff>

<commit_message>
Auto-push 2026-05-21T06:08: settle results + forecasts
</commit_message>
<xml_diff>
--- a/docs/agent-system/outputs/Phase1_Fixture_Slate.xlsx
+++ b/docs/agent-system/outputs/Phase1_Fixture_Slate.xlsx
@@ -141,7 +141,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-05-21 03:42:10 ACST</t>
+          <t>2026-05-21 05:57:28 ACST</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -186,7 +186,7 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>02:30</t>
+          <t>FT</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
@@ -201,7 +201,7 @@
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>live</t>
+          <t>FT</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
@@ -263,7 +263,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-05-21 03:42:10 ACST</t>
+          <t>2026-05-21 05:57:28 ACST</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -298,7 +298,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>flashscore:YobepuNG</t>
+          <t>flashscore:0A1Nl9Wh</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -308,7 +308,7 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>02:30</t>
+          <t>FT</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
@@ -318,22 +318,22 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>1779296400</t>
+          <t>1779300000</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>live</t>
+          <t>FT</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>Lilleström</t>
+          <t>Aalesund</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>flashscore:lilleström</t>
+          <t>flashscore:aalesund</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
@@ -343,12 +343,12 @@
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>Kristiansund</t>
+          <t>Brann</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>flashscore:kristiansund</t>
+          <t>flashscore:brann</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
@@ -385,7 +385,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-05-21 03:42:10 ACST</t>
+          <t>2026-05-21 05:57:28 ACST</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -420,7 +420,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>flashscore:0A1Nl9Wh</t>
+          <t>flashscore:YobepuNG</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -430,7 +430,7 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>03:30</t>
+          <t>FT</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
@@ -440,22 +440,22 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>1779300000</t>
+          <t>1779296400</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>live</t>
+          <t>FT</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>Aalesund</t>
+          <t>Lilleström</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>flashscore:aalesund</t>
+          <t>flashscore:lilleström</t>
         </is>
       </c>
       <c r="P4" t="inlineStr">
@@ -465,12 +465,12 @@
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>Brann</t>
+          <t>Kristiansund</t>
         </is>
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>flashscore:brann</t>
+          <t>flashscore:kristiansund</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
@@ -507,7 +507,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-05-21 03:42:10 ACST</t>
+          <t>2026-05-21 05:57:28 ACST</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -758,7 +758,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-05-21 03:42:10 ACST</t>
+          <t>2026-05-21 05:57:28 ACST</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -803,7 +803,7 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>02:30</t>
+          <t>FT</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
@@ -818,7 +818,7 @@
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>live</t>
+          <t>FT</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
@@ -880,7 +880,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-05-21 03:42:10 ACST</t>
+          <t>2026-05-21 05:57:28 ACST</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -915,7 +915,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>flashscore:YobepuNG</t>
+          <t>flashscore:0A1Nl9Wh</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -925,7 +925,7 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>02:30</t>
+          <t>FT</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
@@ -935,22 +935,22 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>1779296400</t>
+          <t>1779300000</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>live</t>
+          <t>FT</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>Lilleström</t>
+          <t>Aalesund</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>flashscore:lilleström</t>
+          <t>flashscore:aalesund</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
@@ -960,12 +960,12 @@
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>Kristiansund</t>
+          <t>Brann</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>flashscore:kristiansund</t>
+          <t>flashscore:brann</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
@@ -1002,7 +1002,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-05-21 03:42:10 ACST</t>
+          <t>2026-05-21 05:57:28 ACST</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -1037,7 +1037,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>flashscore:0A1Nl9Wh</t>
+          <t>flashscore:YobepuNG</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -1047,7 +1047,7 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>03:30</t>
+          <t>FT</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
@@ -1057,22 +1057,22 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>1779300000</t>
+          <t>1779296400</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>live</t>
+          <t>FT</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>Aalesund</t>
+          <t>Lilleström</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>flashscore:aalesund</t>
+          <t>flashscore:lilleström</t>
         </is>
       </c>
       <c r="P4" t="inlineStr">
@@ -1082,12 +1082,12 @@
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>Brann</t>
+          <t>Kristiansund</t>
         </is>
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>flashscore:brann</t>
+          <t>flashscore:kristiansund</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
@@ -1124,7 +1124,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-05-21 03:42:10 ACST</t>
+          <t>2026-05-21 05:57:28 ACST</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -1643,12 +1643,12 @@
       </c>
       <c r="M2" t="inlineStr">
         <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
           <t>1</t>
-        </is>
-      </c>
-      <c r="N2" t="inlineStr">
-        <is>
-          <t>0</t>
         </is>
       </c>
     </row>
@@ -1715,12 +1715,12 @@
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
     </row>
@@ -1776,7 +1776,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-05-21 03:42:10 ACST</t>
+          <t>2026-05-21 05:57:28 ACST</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">

</xml_diff>

<commit_message>
Auto-push 2026-05-21T18:08: settle results + forecasts
</commit_message>
<xml_diff>
--- a/docs/agent-system/outputs/Phase1_Fixture_Slate.xlsx
+++ b/docs/agent-system/outputs/Phase1_Fixture_Slate.xlsx
@@ -141,7 +141,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-05-21 05:57:28 ACST</t>
+          <t>2026-05-21 18:08:11 ACST</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -176,17 +176,17 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>flashscore:rJKJ2MZP</t>
+          <t>flashscore:zHabevSa</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>FT</t>
+          <t>02:30</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
@@ -196,22 +196,22 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>1779296400</t>
+          <t>1779382800</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>FT</t>
+          <t>live</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>GAIS</t>
+          <t>Elfsborg</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>flashscore:gais</t>
+          <t>flashscore:elfsborg</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
@@ -221,12 +221,12 @@
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>Hammarby</t>
+          <t>Mjallby</t>
         </is>
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>flashscore:hammarby</t>
+          <t>flashscore:mjallby</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
@@ -255,372 +255,6 @@
         </is>
       </c>
       <c r="X2" t="inlineStr">
-        <is>
-          <t>Keyless Flashscore fixture feed.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>2026-05-21 05:57:28 ACST</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Flashscore</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>healthy</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>20</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>Eliteserien</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>flashscore:0A1Nl9Wh</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>2026-05-21</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>FT</t>
-        </is>
-      </c>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>Australia/Adelaide</t>
-        </is>
-      </c>
-      <c r="L3" t="inlineStr">
-        <is>
-          <t>1779300000</t>
-        </is>
-      </c>
-      <c r="M3" t="inlineStr">
-        <is>
-          <t>FT</t>
-        </is>
-      </c>
-      <c r="N3" t="inlineStr">
-        <is>
-          <t>Aalesund</t>
-        </is>
-      </c>
-      <c r="O3" t="inlineStr">
-        <is>
-          <t>flashscore:aalesund</t>
-        </is>
-      </c>
-      <c r="P3" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="Q3" t="inlineStr">
-        <is>
-          <t>Brann</t>
-        </is>
-      </c>
-      <c r="R3" t="inlineStr">
-        <is>
-          <t>flashscore:brann</t>
-        </is>
-      </c>
-      <c r="S3" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="T3" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="U3" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="V3" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="W3" t="inlineStr">
-        <is>
-          <t>ready_for_phase_2</t>
-        </is>
-      </c>
-      <c r="X3" t="inlineStr">
-        <is>
-          <t>Keyless Flashscore fixture feed.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>2026-05-21 05:57:28 ACST</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Flashscore</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>healthy</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>20</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>Eliteserien</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>flashscore:YobepuNG</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>2026-05-21</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>FT</t>
-        </is>
-      </c>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>Australia/Adelaide</t>
-        </is>
-      </c>
-      <c r="L4" t="inlineStr">
-        <is>
-          <t>1779296400</t>
-        </is>
-      </c>
-      <c r="M4" t="inlineStr">
-        <is>
-          <t>FT</t>
-        </is>
-      </c>
-      <c r="N4" t="inlineStr">
-        <is>
-          <t>Lilleström</t>
-        </is>
-      </c>
-      <c r="O4" t="inlineStr">
-        <is>
-          <t>flashscore:lilleström</t>
-        </is>
-      </c>
-      <c r="P4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="Q4" t="inlineStr">
-        <is>
-          <t>Kristiansund</t>
-        </is>
-      </c>
-      <c r="R4" t="inlineStr">
-        <is>
-          <t>flashscore:kristiansund</t>
-        </is>
-      </c>
-      <c r="S4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="T4" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="U4" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="V4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="W4" t="inlineStr">
-        <is>
-          <t>ready_for_phase_2</t>
-        </is>
-      </c>
-      <c r="X4" t="inlineStr">
-        <is>
-          <t>Keyless Flashscore fixture feed.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>2026-05-21 05:57:28 ACST</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Flashscore</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>healthy</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>20</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>Eliteserien</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>flashscore:v3i3qEfD</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>2026-05-21</t>
-        </is>
-      </c>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t>FT</t>
-        </is>
-      </c>
-      <c r="K5" t="inlineStr">
-        <is>
-          <t>Australia/Adelaide</t>
-        </is>
-      </c>
-      <c r="L5" t="inlineStr">
-        <is>
-          <t>1779292800</t>
-        </is>
-      </c>
-      <c r="M5" t="inlineStr">
-        <is>
-          <t>FT</t>
-        </is>
-      </c>
-      <c r="N5" t="inlineStr">
-        <is>
-          <t>Start</t>
-        </is>
-      </c>
-      <c r="O5" t="inlineStr">
-        <is>
-          <t>flashscore:start</t>
-        </is>
-      </c>
-      <c r="P5" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="Q5" t="inlineStr">
-        <is>
-          <t>Bodo/Glimt</t>
-        </is>
-      </c>
-      <c r="R5" t="inlineStr">
-        <is>
-          <t>flashscore:bodoglimt</t>
-        </is>
-      </c>
-      <c r="S5" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="T5" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="U5" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="V5" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="W5" t="inlineStr">
-        <is>
-          <t>ready_for_phase_2</t>
-        </is>
-      </c>
-      <c r="X5" t="inlineStr">
         <is>
           <t>Keyless Flashscore fixture feed.</t>
         </is>
@@ -758,7 +392,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-05-21 05:57:28 ACST</t>
+          <t>2026-05-21 18:08:11 ACST</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -793,17 +427,17 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>flashscore:rJKJ2MZP</t>
+          <t>flashscore:zHabevSa</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>FT</t>
+          <t>02:30</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
@@ -813,22 +447,22 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>1779296400</t>
+          <t>1779382800</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>FT</t>
+          <t>live</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>GAIS</t>
+          <t>Elfsborg</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>flashscore:gais</t>
+          <t>flashscore:elfsborg</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
@@ -838,12 +472,12 @@
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>Hammarby</t>
+          <t>Mjallby</t>
         </is>
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>flashscore:hammarby</t>
+          <t>flashscore:mjallby</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
@@ -872,372 +506,6 @@
         </is>
       </c>
       <c r="X2" t="inlineStr">
-        <is>
-          <t>Keyless Flashscore fixture feed.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>2026-05-21 05:57:28 ACST</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Flashscore</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>healthy</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>20</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>Eliteserien</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>flashscore:0A1Nl9Wh</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>2026-05-21</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>FT</t>
-        </is>
-      </c>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>Australia/Adelaide</t>
-        </is>
-      </c>
-      <c r="L3" t="inlineStr">
-        <is>
-          <t>1779300000</t>
-        </is>
-      </c>
-      <c r="M3" t="inlineStr">
-        <is>
-          <t>FT</t>
-        </is>
-      </c>
-      <c r="N3" t="inlineStr">
-        <is>
-          <t>Aalesund</t>
-        </is>
-      </c>
-      <c r="O3" t="inlineStr">
-        <is>
-          <t>flashscore:aalesund</t>
-        </is>
-      </c>
-      <c r="P3" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="Q3" t="inlineStr">
-        <is>
-          <t>Brann</t>
-        </is>
-      </c>
-      <c r="R3" t="inlineStr">
-        <is>
-          <t>flashscore:brann</t>
-        </is>
-      </c>
-      <c r="S3" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="T3" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="U3" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="V3" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="W3" t="inlineStr">
-        <is>
-          <t>ready_for_phase_2</t>
-        </is>
-      </c>
-      <c r="X3" t="inlineStr">
-        <is>
-          <t>Keyless Flashscore fixture feed.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>2026-05-21 05:57:28 ACST</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Flashscore</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>healthy</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>20</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>Eliteserien</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>flashscore:YobepuNG</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>2026-05-21</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>FT</t>
-        </is>
-      </c>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>Australia/Adelaide</t>
-        </is>
-      </c>
-      <c r="L4" t="inlineStr">
-        <is>
-          <t>1779296400</t>
-        </is>
-      </c>
-      <c r="M4" t="inlineStr">
-        <is>
-          <t>FT</t>
-        </is>
-      </c>
-      <c r="N4" t="inlineStr">
-        <is>
-          <t>Lilleström</t>
-        </is>
-      </c>
-      <c r="O4" t="inlineStr">
-        <is>
-          <t>flashscore:lilleström</t>
-        </is>
-      </c>
-      <c r="P4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="Q4" t="inlineStr">
-        <is>
-          <t>Kristiansund</t>
-        </is>
-      </c>
-      <c r="R4" t="inlineStr">
-        <is>
-          <t>flashscore:kristiansund</t>
-        </is>
-      </c>
-      <c r="S4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="T4" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="U4" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="V4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="W4" t="inlineStr">
-        <is>
-          <t>ready_for_phase_2</t>
-        </is>
-      </c>
-      <c r="X4" t="inlineStr">
-        <is>
-          <t>Keyless Flashscore fixture feed.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>2026-05-21 05:57:28 ACST</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Flashscore</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>healthy</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>20</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>Eliteserien</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>flashscore:v3i3qEfD</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>2026-05-21</t>
-        </is>
-      </c>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t>FT</t>
-        </is>
-      </c>
-      <c r="K5" t="inlineStr">
-        <is>
-          <t>Australia/Adelaide</t>
-        </is>
-      </c>
-      <c r="L5" t="inlineStr">
-        <is>
-          <t>1779292800</t>
-        </is>
-      </c>
-      <c r="M5" t="inlineStr">
-        <is>
-          <t>FT</t>
-        </is>
-      </c>
-      <c r="N5" t="inlineStr">
-        <is>
-          <t>Start</t>
-        </is>
-      </c>
-      <c r="O5" t="inlineStr">
-        <is>
-          <t>flashscore:start</t>
-        </is>
-      </c>
-      <c r="P5" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="Q5" t="inlineStr">
-        <is>
-          <t>Bodo/Glimt</t>
-        </is>
-      </c>
-      <c r="R5" t="inlineStr">
-        <is>
-          <t>flashscore:bodoglimt</t>
-        </is>
-      </c>
-      <c r="S5" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="T5" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="U5" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="V5" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="W5" t="inlineStr">
-        <is>
-          <t>ready_for_phase_2</t>
-        </is>
-      </c>
-      <c r="X5" t="inlineStr">
         <is>
           <t>Keyless Flashscore fixture feed.</t>
         </is>
@@ -1643,84 +911,12 @@
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>1</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Eliteserien</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="L3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="M3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="N3" t="inlineStr">
-        <is>
-          <t>3</t>
+          <t>0</t>
         </is>
       </c>
     </row>
@@ -1776,7 +972,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-05-21 05:57:28 ACST</t>
+          <t>2026-05-21 18:08:11 ACST</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -1806,12 +1002,12 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>1</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>events=301 league_hit=4 skipped_women=0 out_of_window=0 matched=4 by_league={'Eliteserien': 3, 'Allsvenskan': 1} sample_leagues=['Africa|AFRICA: Africa Cup of Nations U17', 'Algeria|ALGERIA: Ligue 1', 'Algeria|ALGERIA: Ligue 2 - Promotion - Play Offs', 'Angola|ANGOLA: Girabola', 'Argentina|ARGENTINA: Copa Argentina', 'Argentina|ARGENTINA: Reserve League - Apertura', 'Armenia|ARMENIA: First League', 'Aruba|ARUBA: Division di Honor - Relegation']</t>
+          <t>events=226 league_hit=1 skipped_women=0 out_of_window=0 matched=1 by_league={'Allsvenskan': 1} sample_leagues=['Argentina|ARGENTINA: Copa Argentina', 'Argentina|ARGENTINA: Reserve League - Apertura', 'Argentina|ARGENTINA: Primera A Women - Apertura', 'Armenia|ARMENIA: First League', 'Aruba|ARUBA: Division di Honor - Relegation', 'Austria|AUSTRIA: Regionalliga Central', 'Austria|AUSTRIA: Steiermark', 'Azerbaijan|AZERBAIJAN: Premier League']</t>
         </is>
       </c>
     </row>
@@ -1878,7 +1074,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>1</t>
         </is>
       </c>
     </row>
@@ -1890,7 +1086,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>1</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Persist stable team badges and refresh latest data artifacts
</commit_message>
<xml_diff>
--- a/docs/agent-system/outputs/Phase1_Fixture_Slate.xlsx
+++ b/docs/agent-system/outputs/Phase1_Fixture_Slate.xlsx
@@ -141,7 +141,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-05-21 18:08:11 ACST</t>
+          <t>2026-05-21 18:22:04 ACST</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -392,7 +392,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-05-21 18:08:11 ACST</t>
+          <t>2026-05-21 18:22:04 ACST</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -972,7 +972,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-05-21 18:08:11 ACST</t>
+          <t>2026-05-21 18:22:04 ACST</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">

</xml_diff>

<commit_message>
Auto-push 2026-05-22T02:10: settle results + forecasts
</commit_message>
<xml_diff>
--- a/docs/agent-system/outputs/Phase1_Fixture_Slate.xlsx
+++ b/docs/agent-system/outputs/Phase1_Fixture_Slate.xlsx
@@ -141,7 +141,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-05-21 18:22:04 ACST</t>
+          <t>2026-05-22 01:58:44 ACST</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -392,7 +392,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-05-21 18:22:04 ACST</t>
+          <t>2026-05-22 01:58:44 ACST</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -972,7 +972,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-05-21 18:22:04 ACST</t>
+          <t>2026-05-22 01:58:44 ACST</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -987,7 +987,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-05-21 to 2026-05-27</t>
+          <t>2026-05-22 to 2026-05-28</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -1007,7 +1007,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>events=226 league_hit=1 skipped_women=0 out_of_window=0 matched=1 by_league={'Allsvenskan': 1} sample_leagues=['Argentina|ARGENTINA: Copa Argentina', 'Argentina|ARGENTINA: Reserve League - Apertura', 'Argentina|ARGENTINA: Primera A Women - Apertura', 'Armenia|ARMENIA: First League', 'Aruba|ARUBA: Division di Honor - Relegation', 'Austria|AUSTRIA: Regionalliga Central', 'Austria|AUSTRIA: Steiermark', 'Azerbaijan|AZERBAIJAN: Premier League']</t>
+          <t>events=227 league_hit=1 skipped_women=0 out_of_window=0 matched=1 by_league={'Allsvenskan': 1} sample_leagues=['Argentina|ARGENTINA: Copa Argentina', 'Argentina|ARGENTINA: Reserve League - Apertura', 'Argentina|ARGENTINA: Primera A Women - Apertura', 'Armenia|ARMENIA: First League', 'Aruba|ARUBA: Division di Honor - Relegation', 'Austria|AUSTRIA: Regionalliga Central', 'Austria|AUSTRIA: Steiermark', 'Azerbaijan|AZERBAIJAN: Premier League']</t>
         </is>
       </c>
     </row>
@@ -1038,7 +1038,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-05-21 to 2026-05-27</t>
+          <t>2026-05-22 to 2026-05-28</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add market voting and persist owner groups
</commit_message>
<xml_diff>
--- a/docs/agent-system/outputs/Phase1_Fixture_Slate.xlsx
+++ b/docs/agent-system/outputs/Phase1_Fixture_Slate.xlsx
@@ -141,7 +141,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-05-22 01:58:44 ACST</t>
+          <t>2026-05-22 04:29:26 ACST</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -186,7 +186,7 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>02:30</t>
+          <t>FT</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
@@ -201,7 +201,7 @@
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>live</t>
+          <t>FT</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
@@ -392,7 +392,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-05-22 01:58:44 ACST</t>
+          <t>2026-05-22 04:29:26 ACST</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -437,7 +437,7 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>02:30</t>
+          <t>FT</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
@@ -452,7 +452,7 @@
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>live</t>
+          <t>FT</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
@@ -911,12 +911,12 @@
       </c>
       <c r="M2" t="inlineStr">
         <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
           <t>1</t>
-        </is>
-      </c>
-      <c r="N2" t="inlineStr">
-        <is>
-          <t>0</t>
         </is>
       </c>
     </row>
@@ -972,7 +972,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-05-22 01:58:44 ACST</t>
+          <t>2026-05-22 04:29:26 ACST</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">

</xml_diff>

<commit_message>
Auto-push 2026-05-22T18:09: settle results + forecasts
</commit_message>
<xml_diff>
--- a/docs/agent-system/outputs/Phase1_Fixture_Slate.xlsx
+++ b/docs/agent-system/outputs/Phase1_Fixture_Slate.xlsx
@@ -141,7 +141,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-05-22 04:29:26 ACST</t>
+          <t>2026-05-22 17:56:54 ACST</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -156,105 +156,349 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
+          <t>196</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>J1 League</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>flashscore:fXvLSp0T</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>2026-05-22</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>20:00</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>Australia/Adelaide</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>1779445800</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>Machida</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>flashscore:machida</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>Urawa</t>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>flashscore:urawa</t>
+        </is>
+      </c>
+      <c r="S2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="T2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="U2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="V2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="W2" t="inlineStr">
+        <is>
+          <t>ready_for_phase_2</t>
+        </is>
+      </c>
+      <c r="X2" t="inlineStr">
+        <is>
+          <t>Keyless Flashscore fixture feed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-05-22 17:56:54 ACST</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Flashscore</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>healthy</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
           <t>40</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
+      <c r="E3" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
         <is>
           <t>Allsvenskan</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>flashscore:zHabevSa</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>2026-05-22</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>FT</t>
-        </is>
-      </c>
-      <c r="K2" t="inlineStr">
+      <c r="G3" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>flashscore:l6SULOIj</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>2026-05-23</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>02:30</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
         <is>
           <t>Australia/Adelaide</t>
         </is>
       </c>
-      <c r="L2" t="inlineStr">
-        <is>
-          <t>1779382800</t>
-        </is>
-      </c>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>FT</t>
-        </is>
-      </c>
-      <c r="N2" t="inlineStr">
-        <is>
-          <t>Elfsborg</t>
-        </is>
-      </c>
-      <c r="O2" t="inlineStr">
-        <is>
-          <t>flashscore:elfsborg</t>
-        </is>
-      </c>
-      <c r="P2" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="Q2" t="inlineStr">
-        <is>
-          <t>Mjallby</t>
-        </is>
-      </c>
-      <c r="R2" t="inlineStr">
-        <is>
-          <t>flashscore:mjallby</t>
-        </is>
-      </c>
-      <c r="S2" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="T2" t="inlineStr">
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>1779469200</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>Djurgarden</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>flashscore:djurgarden</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>Brommapojkarna</t>
+        </is>
+      </c>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>flashscore:brommapojkarna</t>
+        </is>
+      </c>
+      <c r="S3" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="T3" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="U2" t="inlineStr">
+      <c r="U3" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="V2" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="W2" t="inlineStr">
+      <c r="V3" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="W3" t="inlineStr">
         <is>
           <t>ready_for_phase_2</t>
         </is>
       </c>
-      <c r="X2" t="inlineStr">
+      <c r="X3" t="inlineStr">
+        <is>
+          <t>Keyless Flashscore fixture feed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-05-22 17:56:54 ACST</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Flashscore</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>healthy</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Serie A</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>flashscore:ln2VQVwR</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>2026-05-23</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>04:15</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>Australia/Adelaide</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>1779475500</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>Fiorentina</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>flashscore:fiorentina</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>Atalanta</t>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>flashscore:atalanta</t>
+        </is>
+      </c>
+      <c r="S4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="T4" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="U4" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="V4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="W4" t="inlineStr">
+        <is>
+          <t>ready_for_phase_2</t>
+        </is>
+      </c>
+      <c r="X4" t="inlineStr">
         <is>
           <t>Keyless Flashscore fixture feed.</t>
         </is>
@@ -392,7 +636,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-05-22 04:29:26 ACST</t>
+          <t>2026-05-22 17:56:54 ACST</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -407,105 +651,349 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
+          <t>196</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>J1 League</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>flashscore:fXvLSp0T</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>2026-05-22</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>20:00</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>Australia/Adelaide</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>1779445800</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>Machida</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>flashscore:machida</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>Urawa</t>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>flashscore:urawa</t>
+        </is>
+      </c>
+      <c r="S2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="T2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="U2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="V2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="W2" t="inlineStr">
+        <is>
+          <t>ready_for_phase_2</t>
+        </is>
+      </c>
+      <c r="X2" t="inlineStr">
+        <is>
+          <t>Keyless Flashscore fixture feed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-05-22 17:56:54 ACST</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Flashscore</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>healthy</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
           <t>40</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
+      <c r="E3" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
         <is>
           <t>Allsvenskan</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>flashscore:zHabevSa</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>2026-05-22</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>FT</t>
-        </is>
-      </c>
-      <c r="K2" t="inlineStr">
+      <c r="G3" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>flashscore:l6SULOIj</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>2026-05-23</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>02:30</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
         <is>
           <t>Australia/Adelaide</t>
         </is>
       </c>
-      <c r="L2" t="inlineStr">
-        <is>
-          <t>1779382800</t>
-        </is>
-      </c>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>FT</t>
-        </is>
-      </c>
-      <c r="N2" t="inlineStr">
-        <is>
-          <t>Elfsborg</t>
-        </is>
-      </c>
-      <c r="O2" t="inlineStr">
-        <is>
-          <t>flashscore:elfsborg</t>
-        </is>
-      </c>
-      <c r="P2" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="Q2" t="inlineStr">
-        <is>
-          <t>Mjallby</t>
-        </is>
-      </c>
-      <c r="R2" t="inlineStr">
-        <is>
-          <t>flashscore:mjallby</t>
-        </is>
-      </c>
-      <c r="S2" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="T2" t="inlineStr">
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>1779469200</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>Djurgarden</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>flashscore:djurgarden</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>Brommapojkarna</t>
+        </is>
+      </c>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>flashscore:brommapojkarna</t>
+        </is>
+      </c>
+      <c r="S3" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="T3" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="U2" t="inlineStr">
+      <c r="U3" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="V2" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="W2" t="inlineStr">
+      <c r="V3" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="W3" t="inlineStr">
         <is>
           <t>ready_for_phase_2</t>
         </is>
       </c>
-      <c r="X2" t="inlineStr">
+      <c r="X3" t="inlineStr">
+        <is>
+          <t>Keyless Flashscore fixture feed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-05-22 17:56:54 ACST</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Flashscore</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>healthy</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Serie A</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>flashscore:ln2VQVwR</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>2026-05-23</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>04:15</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>Australia/Adelaide</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>1779475500</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>Fiorentina</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>flashscore:fiorentina</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>Atalanta</t>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>flashscore:atalanta</t>
+        </is>
+      </c>
+      <c r="S4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="T4" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="U4" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="V4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="W4" t="inlineStr">
+        <is>
+          <t>ready_for_phase_2</t>
+        </is>
+      </c>
+      <c r="X4" t="inlineStr">
         <is>
           <t>Keyless Flashscore fixture feed.</t>
         </is>
@@ -911,12 +1399,156 @@
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
         <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>J1 League</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
           <t>1</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Serie A</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>0</t>
         </is>
       </c>
     </row>
@@ -972,7 +1604,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-05-22 04:29:26 ACST</t>
+          <t>2026-05-22 17:56:54 ACST</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -1002,12 +1634,12 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>events=227 league_hit=1 skipped_women=0 out_of_window=0 matched=1 by_league={'Allsvenskan': 1} sample_leagues=['Argentina|ARGENTINA: Copa Argentina', 'Argentina|ARGENTINA: Reserve League - Apertura', 'Argentina|ARGENTINA: Primera A Women - Apertura', 'Armenia|ARMENIA: First League', 'Aruba|ARUBA: Division di Honor - Relegation', 'Austria|AUSTRIA: Regionalliga Central', 'Austria|AUSTRIA: Steiermark', 'Azerbaijan|AZERBAIJAN: Premier League']</t>
+          <t>events=405 league_hit=3 skipped_women=0 out_of_window=0 matched=3 by_league={'Serie A': 1, 'J1 League': 1, 'Allsvenskan': 1} sample_leagues=['Algeria|ALGERIA: Ligue 1', 'Argentina|ARGENTINA: Primera B', 'Argentina|ARGENTINA: Primera C', 'Argentina|ARGENTINA: Reserve League - Apertura', 'Argentina|ARGENTINA: Primera A Women - Apertura', 'Asia|ASIA: AFC Asian Cup U17 - Play Offs', 'Australia|AUSTRALIA: NPL Queensland', 'Australia|AUSTRALIA: NPL Victoria']</t>
         </is>
       </c>
     </row>
@@ -1074,7 +1706,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
     </row>
@@ -1086,7 +1718,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Cache soccer badges before Firestore upload
</commit_message>
<xml_diff>
--- a/docs/agent-system/outputs/Phase1_Fixture_Slate.xlsx
+++ b/docs/agent-system/outputs/Phase1_Fixture_Slate.xlsx
@@ -141,7 +141,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-05-22 17:56:54 ACST</t>
+          <t>2026-05-22 18:58:45 ACST</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -263,7 +263,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-05-22 17:56:54 ACST</t>
+          <t>2026-05-22 18:58:45 ACST</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -385,7 +385,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-05-22 17:56:54 ACST</t>
+          <t>2026-05-22 18:58:45 ACST</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -636,7 +636,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-05-22 17:56:54 ACST</t>
+          <t>2026-05-22 18:58:45 ACST</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -758,7 +758,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-05-22 17:56:54 ACST</t>
+          <t>2026-05-22 18:58:45 ACST</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -880,7 +880,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-05-22 17:56:54 ACST</t>
+          <t>2026-05-22 18:58:45 ACST</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -1604,7 +1604,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-05-22 17:56:54 ACST</t>
+          <t>2026-05-22 18:58:45 ACST</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">

</xml_diff>